<commit_message>
feat: new user registration - 2026-04-13 15:24 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utenti Perforce" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Utenti Perforce" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Utenti Perforce'!$A$1:$H$1</definedName>
@@ -50,7 +50,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -73,18 +73,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8F0FE"/>
         <bgColor rgb="00E8F0FE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F7"/>
-        <bgColor rgb="00F5F5F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -110,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -123,10 +111,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -494,13 +478,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -552,7 +536,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>▸ ProjectAlpha</t>
+          <t>▸ Progetto Test</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -563,285 +547,47 @@
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>4 membri</t>
+          <t>1 membri</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>2026-04-13 10:05:00</t>
+          <t>2026-04-13 15:24:42</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>sofia_russo</t>
+          <t>leonardo_villa</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Sofia Russo</t>
+          <t>Leonardo Villa</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>sofia.russo@studenti.naba.it</t>
+          <t>leonardo.villa@studenti.naba.it</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>ProjectAlpha</t>
+          <t>Progetto Test</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-13 10:03:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>anna_ferrari</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Anna Ferrari</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>anna.ferrari@studenti.naba.it</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>ProjectAlpha</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-13 10:00:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>marco_bianchi</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Marco Bianchi</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>marco.bianchi@studenti.naba.it</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>ProjectAlpha</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-13 10:01:00</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>giulia_verdi</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Giulia Verdi</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>giulia.verdi@studenti.naba.it</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>ProjectAlpha</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Sì</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="6" customHeight="1">
-      <c r="A7" s="6" t="inlineStr"/>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>▸ ProjectBeta</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>2 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-13 10:02:00</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>luca_rossi</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Luca Rossi</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>luca.rossi@studenti.naba.it</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>ProjectBeta</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-13 10:04:00</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>wang_li</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Wang Li</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>wang.li@studenti.naba.it</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>ProjectBeta</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Sì</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-13 15:40 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -50,7 +50,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +73,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8F0FE"/>
         <bgColor rgb="00E8F0FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F7"/>
+        <bgColor rgb="00F5F5F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -111,6 +123,10 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -478,13 +494,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -536,7 +552,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>▸ Progetto Test</t>
+          <t>▸ Coso</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -554,40 +570,110 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
+          <t>2026-04-13 15:40:24</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>emanuele_lomello</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>EMANUELE LOMELLO</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>emanuele_lomello@docenti.naba.it</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Coso</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1">
+      <c r="A4" s="6" t="inlineStr"/>
+      <c r="B4" s="6" t="inlineStr"/>
+      <c r="C4" s="6" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>▸ Progetto Test</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
           <t>2026-04-13 15:24:42</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>leonardo_villa</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Leonardo Villa</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>leonardo.villa@studenti.naba.it</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Progetto Test</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Sì</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-13 16:11 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,14 +494,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -679,6 +679,76 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="6" customHeight="1">
+      <c r="A7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>▸ The Test Project</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13 16:11:41</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>alex_doe</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Alex Doe</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>alex_doe@studenti.naba.it</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>The Test Project</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-13 16:42 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -692,7 +692,7 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>▸ The Test Project</t>
+          <t>▸ The Iron Lady</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
@@ -703,47 +703,201 @@
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>1 membri</t>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>2026-04-13 16:42:08</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>alex_doe</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Alex Doe</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>alex_doe@studenti.naba.it\</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>The Iron Lady</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13 16:42:08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>jane_doe</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Jane Doe</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>jane_doe@studenti.naba.it</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>The Iron Lady</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13 16:42:08</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>marie_doe</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Marie Doe</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>marie_doe@studenti.naba.it</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>The Iron Lady</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="6" customHeight="1">
+      <c r="A12" s="6" t="inlineStr"/>
+      <c r="B12" s="6" t="inlineStr"/>
+      <c r="C12" s="6" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>▸ The Test Project</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
           <t>2026-04-13 16:11:41</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>alex_doe</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Alex Doe</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>alex_doe@studenti.naba.it</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>The Test Project</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Sì</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-14 09:20 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -50,7 +50,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +73,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8F0FE"/>
         <bgColor rgb="00E8F0FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F7"/>
+        <bgColor rgb="00F5F5F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -111,6 +123,10 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -478,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -536,7 +552,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>▸ Trinity</t>
+          <t>▸ slay</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -554,40 +570,110 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
+          <t>2026-04-14 09:20:05</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>anna_rossi</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Anna Rossi</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>annabrue05@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>slay</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1">
+      <c r="A4" s="6" t="inlineStr"/>
+      <c r="B4" s="6" t="inlineStr"/>
+      <c r="C4" s="6" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>▸ Trinity</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
           <t>2026-04-13 17:53:02</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>leonardo_villa</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Leonardo Villa</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>lvilla.personal@gmail.com</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Trinity</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Sì</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-14 13:18 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,13 +494,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -552,7 +552,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>▸ slay</t>
+          <t>▸ Hammerhead</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -570,37 +570,37 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>2026-04-14 09:20:05</t>
+          <t>2026-04-14 13:18:43</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>anna_rossi</t>
+          <t>jacopo_gennari</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Anna Rossi</t>
+          <t>Jacopo Gennari</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>annabrue05@gmail.com</t>
+          <t>jacopo.gennari@studenti.naba.it</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>slay</t>
+          <t>Hammerhead</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -622,7 +622,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>▸ Trinity</t>
+          <t>▸ slay</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
@@ -640,40 +640,110 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
+          <t>2026-04-14 09:20:05</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>anna_rossi</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Anna Rossi</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>annabrue05@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>slay</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="6" customHeight="1">
+      <c r="A7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>▸ Trinity</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
           <t>2026-04-13 17:53:02</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>leonardo_villa</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Leonardo Villa</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>lvilla.personal@gmail.com</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Trinity</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Sì</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-14 13:30 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -552,7 +552,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>▸ Hammerhead</t>
+          <t>▸ Collateral</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -570,27 +570,27 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>2026-04-14 13:18:43</t>
+          <t>2026-04-14 13:30:08</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>jacopo_gennari</t>
+          <t>maria_bianchi</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Jacopo Gennari</t>
+          <t>Maria Bianchi</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>jacopo.gennari@studenti.naba.it</t>
+          <t>maria.bianchi@studenti.naba.it</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Hammerhead</t>
+          <t>Collateral</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -622,7 +622,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>▸ slay</t>
+          <t>▸ Hammerhead</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
@@ -640,37 +640,37 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 09:20:05</t>
+          <t>2026-04-14 13:18:43</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>anna_rossi</t>
+          <t>jacopo_gennari</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Anna Rossi</t>
+          <t>Jacopo Gennari</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>annabrue05@gmail.com</t>
+          <t>jacopo.gennari@studenti.naba.it</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>slay</t>
+          <t>Hammerhead</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -692,7 +692,7 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>▸ Trinity</t>
+          <t>▸ slay</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
@@ -710,40 +710,110 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>2026-04-14 09:20:05</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>anna_rossi</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Anna Rossi</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>annabrue05@gmail.com</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>slay</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="6" customHeight="1">
+      <c r="A10" s="6" t="inlineStr"/>
+      <c r="B10" s="6" t="inlineStr"/>
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>▸ Trinity</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>2026-04-13 17:53:02</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>leonardo_villa</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Leonardo Villa</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>lvilla.personal@gmail.com</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Trinity</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Sì</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-14 13:36 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,13 +494,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -552,7 +552,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>▸ Collateral</t>
+          <t>▸ Alpha</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -570,27 +570,27 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>2026-04-14 13:30:08</t>
+          <t>2026-04-14 13:36:33</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>maria_bianchi</t>
+          <t>giacomo_lambardi</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Maria Bianchi</t>
+          <t>Giacomo Lambardi</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>maria.bianchi@studenti.naba.it</t>
+          <t>giacomo.lambardi@studenti.naba.it</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Collateral</t>
+          <t>Alpha</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -622,7 +622,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>▸ Hammerhead</t>
+          <t>▸ Collateral</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
@@ -640,27 +640,27 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 13:18:43</t>
+          <t>2026-04-14 13:30:08</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>jacopo_gennari</t>
+          <t>maria_bianchi</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Jacopo Gennari</t>
+          <t>Maria Bianchi</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>jacopo.gennari@studenti.naba.it</t>
+          <t>maria.bianchi@studenti.naba.it</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Hammerhead</t>
+          <t>Collateral</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -692,7 +692,7 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>▸ slay</t>
+          <t>▸ Hammerhead</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
@@ -710,37 +710,37 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>2026-04-14 09:20:05</t>
+          <t>2026-04-14 13:18:43</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>anna_rossi</t>
+          <t>jacopo_gennari</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Anna Rossi</t>
+          <t>Jacopo Gennari</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>annabrue05@gmail.com</t>
+          <t>jacopo.gennari@studenti.naba.it</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>slay</t>
+          <t>Hammerhead</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -762,7 +762,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>▸ Trinity</t>
+          <t>▸ slay</t>
         </is>
       </c>
       <c r="B11" s="3" t="n"/>
@@ -780,40 +780,110 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
+          <t>2026-04-14 09:20:05</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>anna_rossi</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Anna Rossi</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>annabrue05@gmail.com</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>slay</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="6" customHeight="1">
+      <c r="A13" s="6" t="inlineStr"/>
+      <c r="B13" s="6" t="inlineStr"/>
+      <c r="C13" s="6" t="inlineStr"/>
+      <c r="D13" s="6" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>▸ Trinity</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>2026-04-13 17:53:02</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>leonardo_villa</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Leonardo Villa</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>lvilla.personal@gmail.com</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Trinity</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Sì</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-14 14:48 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -500,7 +500,7 @@
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -1140,7 +1140,7 @@
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>▸ Beta</t>
+          <t>▸ BlackPlague</t>
         </is>
       </c>
       <c r="B20" s="3" t="n"/>
@@ -1151,39 +1151,39 @@
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>1 membri</t>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:07:47</t>
+          <t>2026-04-14 14:03:18</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>gabriele_segata</t>
+          <t>Francesca_Huang</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Gabriele Segata</t>
+          <t>Francesca_Huang</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>gabriele.segata@studenti.naba.it</t>
+          <t>Francesca_Huang@naba.it</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>BlackPlague</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1193,119 +1193,119 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="6" customHeight="1">
-      <c r="A22" s="6" t="inlineStr"/>
-      <c r="B22" s="6" t="inlineStr"/>
-      <c r="C22" s="6" t="inlineStr"/>
-      <c r="D22" s="6" t="inlineStr"/>
-      <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="6" t="inlineStr"/>
-      <c r="G22" s="6" t="inlineStr"/>
-      <c r="H22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>▸ BlackPlague</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Francesca_Huang</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Francesca_Huang</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Francesca_Huang@naba.it</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Jiayi_Li</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Jiayi_Li</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Jiayi_Li@naba.it</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>BlackPlague</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Jiayi_Li</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Jiayi_Li</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Jiayi_Li@naba.it</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu@naba.it</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>BlackPlague</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="6" customHeight="1">
+      <c r="A24" s="6" t="inlineStr"/>
+      <c r="B24" s="6" t="inlineStr"/>
+      <c r="C24" s="6" t="inlineStr"/>
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>▸ BloodAndButter</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
         </is>
       </c>
     </row>
@@ -1317,22 +1317,22 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Zhengying_Xu</t>
+          <t>Ali_Fallahmoghadami</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Zhengying_Xu</t>
+          <t>Ali Fallahmoghadami</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Zhengying_Xu@naba.it</t>
+          <t>Ali_Fallahmoghadami@naba.it</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>BlackPlague</t>
+          <t>BloodAndButter</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -1351,199 +1351,199 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="6" customHeight="1">
-      <c r="A27" s="6" t="inlineStr"/>
-      <c r="B27" s="6" t="inlineStr"/>
-      <c r="C27" s="6" t="inlineStr"/>
-      <c r="D27" s="6" t="inlineStr"/>
-      <c r="E27" s="6" t="inlineStr"/>
-      <c r="F27" s="6" t="inlineStr"/>
-      <c r="G27" s="6" t="inlineStr"/>
-      <c r="H27" s="6" t="inlineStr"/>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>▸ BloodAndButter</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>5 membri</t>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Chen_Qilin</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Chen Qilin</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Chen_Qilin@naba.it</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>BloodAndButter</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Leonardo_Lago</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Leonardo Lago</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Leonardo_Lago@naba.it</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>BloodAndButter</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Ali_Fallahmoghadami</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Ali Fallahmoghadami</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Ali_Fallahmoghadami@naba.it</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Lorenzo_Battista</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Lorenzo Battista</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Lorenzo_Battista@naba.it</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>BloodAndButter</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Chen_Qilin</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Chen Qilin</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Chen_Qilin@naba.it</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Oliviya_Khmelidze</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Oliviya Khmelidze</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Oliviya_Khmelidze@naba.it</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>BloodAndButter</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Leonardo_Lago</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Leonardo Lago</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Leonardo_Lago@naba.it</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>BloodAndButter</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Lorenzo_Battista</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Lorenzo Battista</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>Lorenzo_Battista@naba.it</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>BloodAndButter</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="6" customHeight="1">
+      <c r="A31" s="6" t="inlineStr"/>
+      <c r="B31" s="6" t="inlineStr"/>
+      <c r="C31" s="6" t="inlineStr"/>
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>▸ FloraExMachina</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="3" t="n"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Oliviya_Khmelidze</t>
+          <t>alessandro_cova</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Oliviya Khmelidze</t>
+          <t>alessandro_cova</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Oliviya_Khmelidze@naba.it</t>
+          <t>alessandro_cova@VS_MAIN</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>BloodAndButter</t>
+          <t>FloraExMachina</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -1589,147 +1589,147 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="6" customHeight="1">
-      <c r="A34" s="6" t="inlineStr"/>
-      <c r="B34" s="6" t="inlineStr"/>
-      <c r="C34" s="6" t="inlineStr"/>
-      <c r="D34" s="6" t="inlineStr"/>
-      <c r="E34" s="6" t="inlineStr"/>
-      <c r="F34" s="6" t="inlineStr"/>
-      <c r="G34" s="6" t="inlineStr"/>
-      <c r="H34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>▸ FloraExMachina</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>alessandro_cova</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>alessandro_cova</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>alessandro_cova@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>denise_bottecchia</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>denise_bottecchia</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>denise_bottecchia@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>FloraExMachina</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>FloraExMachina</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="6" customHeight="1">
+      <c r="A36" s="6" t="inlineStr"/>
+      <c r="B36" s="6" t="inlineStr"/>
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr"/>
+      <c r="H36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>▸ Gamma</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
         </is>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-14 14:48:23</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>kiyomi_corinti</t>
+          <t>andrea_caiazzo</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>kiyomi_corinti</t>
+          <t>Andrea Caiazzo</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>kiyomi_corinti@VS_MAIN</t>
+          <t>andrea.caiazzo@studenti.naba.it</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>FloraExMachina</t>
+          <t>Gamma</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-14 18:14 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,13 +494,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -1532,7 +1532,7 @@
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>▸ FloraExMachina</t>
+          <t>▸ Delta</t>
         </is>
       </c>
       <c r="B32" s="3" t="n"/>
@@ -1550,32 +1550,32 @@
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-14 18:13:51</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>alessandro_cova</t>
+          <t>camilla_ferioli</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>alessandro_cova</t>
+          <t>Camilla Ferioli</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>alessandro_cova@VS_MAIN</t>
+          <t>camilla_ferioli@studenti.naba.it</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>FloraExMachina</t>
+          <t>Delta</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -1585,39 +1585,39 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-14 18:13:51</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>denise_bottecchia</t>
+          <t>jon_doe</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>denise_bottecchia</t>
+          <t>Jon Doe</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>denise_bottecchia@VS_MAIN</t>
+          <t>jon.doe@studenti.naba.it</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>FloraExMachina</t>
+          <t>Delta</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -1627,39 +1627,39 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-14 18:13:51</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>kiyomi_corinti</t>
+          <t>tech_a</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>kiyomi_corinti</t>
+          <t>Tech A</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>kiyomi_corinti@VS_MAIN</t>
+          <t>tech_a@studenti.naba.it</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>FloraExMachina</t>
+          <t>Delta</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>▸ Gamma</t>
+          <t>▸ FloraExMachina</t>
         </is>
       </c>
       <c r="B37" s="3" t="n"/>
@@ -1697,39 +1697,39 @@
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>1 membri</t>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>2026-04-14 14:48:23</t>
+          <t>2026-04-14 14:03:18</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>andrea_caiazzo</t>
+          <t>alessandro_cova</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Andrea Caiazzo</t>
+          <t>alessandro_cova</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>andrea.caiazzo@studenti.naba.it</t>
+          <t>alessandro_cova@VS_MAIN</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Gamma</t>
+          <t>FloraExMachina</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -1739,231 +1739,231 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="6" customHeight="1">
-      <c r="A39" s="6" t="inlineStr"/>
-      <c r="B39" s="6" t="inlineStr"/>
-      <c r="C39" s="6" t="inlineStr"/>
-      <c r="D39" s="6" t="inlineStr"/>
-      <c r="E39" s="6" t="inlineStr"/>
-      <c r="F39" s="6" t="inlineStr"/>
-      <c r="G39" s="6" t="inlineStr"/>
-      <c r="H39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>▸ HideAndSeek</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>4 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Jiayi_Li</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Jiayi_Li</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>Jiayi_Li@naba.it</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>HideAndSeek</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Julia_Bergman</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Julia_Bergman</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>Julia_Bergman@naba.it</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>HideAndSeek</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G42" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>denise_bottecchia</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>denise_bottecchia</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>denise_bottecchia@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>FloraExMachina</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>FloraExMachina</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="6" customHeight="1">
+      <c r="A41" s="6" t="inlineStr"/>
+      <c r="B41" s="6" t="inlineStr"/>
+      <c r="C41" s="6" t="inlineStr"/>
+      <c r="D41" s="6" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr"/>
+      <c r="G41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>▸ Gamma</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n"/>
+      <c r="C42" s="3" t="n"/>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n"/>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
         </is>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-14 14:48:23</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Wilma_Sved</t>
+          <t>andrea_caiazzo</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>wilma sved</t>
+          <t>Andrea Caiazzo</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>wilma_sved@studenti.naba.it</t>
+          <t>andrea.caiazzo@studenti.naba.it</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="6" customHeight="1">
+      <c r="A44" s="6" t="inlineStr"/>
+      <c r="B44" s="6" t="inlineStr"/>
+      <c r="C44" s="6" t="inlineStr"/>
+      <c r="D44" s="6" t="inlineStr"/>
+      <c r="E44" s="6" t="inlineStr"/>
+      <c r="F44" s="6" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr"/>
+      <c r="H44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>▸ HideAndSeek</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n"/>
+      <c r="C45" s="3" t="n"/>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="3" t="n"/>
+      <c r="F45" s="3" t="n"/>
+      <c r="G45" s="3" t="n"/>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Jiayi_Li</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Jiayi_Li</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Jiayi_Li@naba.it</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
           <t>HideAndSeek</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Zhengying_Xu</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>Zhengying_Xu</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>Zhengying_Xu@naba.it</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>HideAndSeek</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H44" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="6" customHeight="1">
-      <c r="A45" s="6" t="inlineStr"/>
-      <c r="B45" s="6" t="inlineStr"/>
-      <c r="C45" s="6" t="inlineStr"/>
-      <c r="D45" s="6" t="inlineStr"/>
-      <c r="E45" s="6" t="inlineStr"/>
-      <c r="F45" s="6" t="inlineStr"/>
-      <c r="G45" s="6" t="inlineStr"/>
-      <c r="H45" s="6" t="inlineStr"/>
-    </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>▸ Imagery</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="n"/>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
-      <c r="F46" s="3" t="n"/>
-      <c r="G46" s="3" t="n"/>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>6 membri</t>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Anastasia_Miani</t>
+          <t>Julia_Bergman</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Anastasia_Miani</t>
+          <t>Julia_Bergman</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Anastasia_Miani@naba.it</t>
+          <t>Julia_Bergman@naba.it</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Imagery</t>
+          <t>HideAndSeek</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2017,22 +2017,22 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Lorenzo_Mari</t>
+          <t>Wilma_Sved</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Lorenzo_Mari</t>
+          <t>wilma sved</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Lorenzo_Mari@naba.it</t>
+          <t>wilma_sved@studenti.naba.it</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Imagery</t>
+          <t>HideAndSeek</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -2059,191 +2059,191 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
+          <t>Zhengying_Xu</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu@naba.it</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>HideAndSeek</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="6" customHeight="1">
+      <c r="A50" s="6" t="inlineStr"/>
+      <c r="B50" s="6" t="inlineStr"/>
+      <c r="C50" s="6" t="inlineStr"/>
+      <c r="D50" s="6" t="inlineStr"/>
+      <c r="E50" s="6" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr"/>
+      <c r="H50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51" ht="24" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>▸ Imagery</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n"/>
+      <c r="C51" s="3" t="n"/>
+      <c r="D51" s="3" t="n"/>
+      <c r="E51" s="3" t="n"/>
+      <c r="F51" s="3" t="n"/>
+      <c r="G51" s="3" t="n"/>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Anastasia_Miani</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Anastasia_Miani</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Anastasia_Miani@naba.it</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Imagery</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Lorenzo_Mari</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Lorenzo_Mari</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Lorenzo_Mari@naba.it</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Imagery</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
           <t>Lucrezia_D'Amico</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>Lucrezia_D'Amico</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>Lucrezia_D'Amico@naba.it</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
         <is>
           <t>Imagery</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Mattia_Bombace</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Mattia_Bombace</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Mattia_Bombace@naba.it</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Imagery</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Serena_Lin</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>Serena_Lin</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Serena_Lin@naba.it</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Imagery</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Youfan_Lin</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Youfan_Lin</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Youfan_Lin@naba.it</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Imagery</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="6" customHeight="1">
-      <c r="A53" s="6" t="inlineStr"/>
-      <c r="B53" s="6" t="inlineStr"/>
-      <c r="C53" s="6" t="inlineStr"/>
-      <c r="D53" s="6" t="inlineStr"/>
-      <c r="E53" s="6" t="inlineStr"/>
-      <c r="F53" s="6" t="inlineStr"/>
-      <c r="G53" s="6" t="inlineStr"/>
-      <c r="H53" s="6" t="inlineStr"/>
-    </row>
-    <row r="54" ht="24" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>▸ Kronos</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="n"/>
-      <c r="C54" s="3" t="n"/>
-      <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n"/>
-      <c r="G54" s="3" t="n"/>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>5 membri</t>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -2255,22 +2255,22 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Alberto_Cervillio</t>
+          <t>Mattia_Bombace</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Alberto_Cervillio</t>
+          <t>Mattia_Bombace</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Alberto_Cervillio@naba.it</t>
+          <t>Mattia_Bombace@naba.it</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Kronos</t>
+          <t>Imagery</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -2297,22 +2297,22 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Bruno_Bisogno</t>
+          <t>Serena_Lin</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Bruno_Bisogno</t>
+          <t>Serena_Lin</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Bruno_Bisogno@naba.it</t>
+          <t>Serena_Lin@naba.it</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>Kronos</t>
+          <t>Imagery</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
@@ -2339,149 +2339,149 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Gaia_Aprile</t>
+          <t>Youfan_Lin</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Gaia_Aprile</t>
+          <t>Youfan_Lin</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Gaia_Aprile@naba.it</t>
+          <t>Youfan_Lin@naba.it</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
+          <t>Imagery</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="6" customHeight="1">
+      <c r="A58" s="6" t="inlineStr"/>
+      <c r="B58" s="6" t="inlineStr"/>
+      <c r="C58" s="6" t="inlineStr"/>
+      <c r="D58" s="6" t="inlineStr"/>
+      <c r="E58" s="6" t="inlineStr"/>
+      <c r="F58" s="6" t="inlineStr"/>
+      <c r="G58" s="6" t="inlineStr"/>
+      <c r="H58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59" ht="24" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>▸ Kronos</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="n"/>
+      <c r="C59" s="3" t="n"/>
+      <c r="D59" s="3" t="n"/>
+      <c r="E59" s="3" t="n"/>
+      <c r="F59" s="3" t="n"/>
+      <c r="G59" s="3" t="n"/>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Alberto_Cervillio</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Alberto_Cervillio</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Alberto_Cervillio@naba.it</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
           <t>Kronos</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Bruschi</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Bruschi</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Bruschi@naba-da.com</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Bruno_Bisogno</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Bruno_Bisogno</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Bruno_Bisogno@naba.it</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>Kronos</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>Riccardo_Bassani</t>
-        </is>
-      </c>
-      <c r="C59" s="7" t="inlineStr">
-        <is>
-          <t>Riccardo_Bassani</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>Riccardo_Bassani@naba.it</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>Kronos</t>
-        </is>
-      </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="6" customHeight="1">
-      <c r="A60" s="6" t="inlineStr"/>
-      <c r="B60" s="6" t="inlineStr"/>
-      <c r="C60" s="6" t="inlineStr"/>
-      <c r="D60" s="6" t="inlineStr"/>
-      <c r="E60" s="6" t="inlineStr"/>
-      <c r="F60" s="6" t="inlineStr"/>
-      <c r="G60" s="6" t="inlineStr"/>
-      <c r="H60" s="6" t="inlineStr"/>
-    </row>
-    <row r="61" ht="24" customHeight="1">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>▸ MidnightRunners</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="n"/>
-      <c r="C61" s="3" t="n"/>
-      <c r="D61" s="3" t="n"/>
-      <c r="E61" s="3" t="n"/>
-      <c r="F61" s="3" t="n"/>
-      <c r="G61" s="3" t="n"/>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>5 membri</t>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -2493,22 +2493,22 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Danilo_Puccio</t>
+          <t>Gaia_Aprile</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Danilo_Puccio</t>
+          <t>Gaia_Aprile</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Danilo_Puccio@naba.it</t>
+          <t>Gaia_Aprile@naba.it</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>MidnightRunners</t>
+          <t>Kronos</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -2535,22 +2535,22 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Eros_Mussuto</t>
+          <t>Jacopo_Bruschi</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Eros_Mussuto</t>
+          <t>Jacopo_Bruschi</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Eros_Mussuto@naba.it</t>
+          <t>Jacopo_Bruschi@naba-da.com</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>MidnightRunners</t>
+          <t>Kronos</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -2577,149 +2577,149 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Gianluca_Lucchini</t>
+          <t>Riccardo_Bassani</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Gianluca_Lucchini</t>
+          <t>Riccardo_Bassani</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Gianluca_Lucchini@naba.it</t>
+          <t>Riccardo_Bassani@naba.it</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
+          <t>Kronos</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="6" customHeight="1">
+      <c r="A65" s="6" t="inlineStr"/>
+      <c r="B65" s="6" t="inlineStr"/>
+      <c r="C65" s="6" t="inlineStr"/>
+      <c r="D65" s="6" t="inlineStr"/>
+      <c r="E65" s="6" t="inlineStr"/>
+      <c r="F65" s="6" t="inlineStr"/>
+      <c r="G65" s="6" t="inlineStr"/>
+      <c r="H65" s="6" t="inlineStr"/>
+    </row>
+    <row r="66" ht="24" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>▸ MidnightRunners</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="3" t="n"/>
+      <c r="D66" s="3" t="n"/>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="3" t="n"/>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Danilo_Puccio</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Danilo_Puccio</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Danilo_Puccio@naba.it</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
           <t>MidnightRunners</t>
         </is>
       </c>
-      <c r="F64" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H64" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="22" customHeight="1">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>Tommaso_Mancini</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>Tommaso_Mancini</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Tommaso_Mancini@naba.it</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Eros_Mussuto</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Eros_Mussuto</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Eros_Mussuto@naba.it</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
         <is>
           <t>MidnightRunners</t>
         </is>
       </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H65" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="inlineStr">
-        <is>
-          <t>Valeria_Portillo</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>Valeria_Portillo</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Valeria_Portillo@naba.it</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>MidnightRunners</t>
-        </is>
-      </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H66" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="6" customHeight="1">
-      <c r="A67" s="6" t="inlineStr"/>
-      <c r="B67" s="6" t="inlineStr"/>
-      <c r="C67" s="6" t="inlineStr"/>
-      <c r="D67" s="6" t="inlineStr"/>
-      <c r="E67" s="6" t="inlineStr"/>
-      <c r="F67" s="6" t="inlineStr"/>
-      <c r="G67" s="6" t="inlineStr"/>
-      <c r="H67" s="6" t="inlineStr"/>
-    </row>
-    <row r="68" ht="24" customHeight="1">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>▸ Overload</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="n"/>
-      <c r="C68" s="3" t="n"/>
-      <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="3" t="n"/>
-      <c r="G68" s="3" t="n"/>
-      <c r="H68" s="4" t="inlineStr">
-        <is>
-          <t>4 membri</t>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -2731,22 +2731,22 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>gabriele_dallari</t>
+          <t>Gianluca_Lucchini</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>gabriele_dallari</t>
+          <t>Gianluca_Lucchini</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>gabriele_dallari@VS_MAIN</t>
+          <t>Gianluca_Lucchini@naba.it</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Overload</t>
+          <t>MidnightRunners</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
@@ -2773,22 +2773,22 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>lorenzo_fiorentino</t>
+          <t>Tommaso_Mancini</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>lorenzo_fiorentino</t>
+          <t>Tommaso_Mancini</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>lorenzo_fiorentino@VS_MAIN</t>
+          <t>Tommaso_Mancini@naba.it</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>Overload</t>
+          <t>MidnightRunners</t>
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr">
@@ -2815,107 +2815,107 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>luigi_cirelli</t>
+          <t>Valeria_Portillo</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>luigi_cirelli</t>
+          <t>Valeria_Portillo</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>luigi_cirelli@VS_MAIN</t>
+          <t>Valeria_Portillo@naba.it</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
+          <t>MidnightRunners</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="6" customHeight="1">
+      <c r="A72" s="6" t="inlineStr"/>
+      <c r="B72" s="6" t="inlineStr"/>
+      <c r="C72" s="6" t="inlineStr"/>
+      <c r="D72" s="6" t="inlineStr"/>
+      <c r="E72" s="6" t="inlineStr"/>
+      <c r="F72" s="6" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73" ht="24" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>▸ Overload</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="n"/>
+      <c r="C73" s="3" t="n"/>
+      <c r="D73" s="3" t="n"/>
+      <c r="E73" s="3" t="n"/>
+      <c r="F73" s="3" t="n"/>
+      <c r="G73" s="3" t="n"/>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>gabriele_dallari</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>gabriele_dallari</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>gabriele_dallari@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
           <t>Overload</t>
         </is>
       </c>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B72" s="7" t="inlineStr">
-        <is>
-          <t>riccardo_landoni</t>
-        </is>
-      </c>
-      <c r="C72" s="7" t="inlineStr">
-        <is>
-          <t>riccardo_landoni</t>
-        </is>
-      </c>
-      <c r="D72" s="7" t="inlineStr">
-        <is>
-          <t>riccardo_landoni@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E72" s="7" t="inlineStr">
-        <is>
-          <t>Overload</t>
-        </is>
-      </c>
-      <c r="F72" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G72" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H72" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="6" customHeight="1">
-      <c r="A73" s="6" t="inlineStr"/>
-      <c r="B73" s="6" t="inlineStr"/>
-      <c r="C73" s="6" t="inlineStr"/>
-      <c r="D73" s="6" t="inlineStr"/>
-      <c r="E73" s="6" t="inlineStr"/>
-      <c r="F73" s="6" t="inlineStr"/>
-      <c r="G73" s="6" t="inlineStr"/>
-      <c r="H73" s="6" t="inlineStr"/>
-    </row>
-    <row r="74" ht="24" customHeight="1">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>▸ Psicostasia</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="n"/>
-      <c r="C74" s="3" t="n"/>
-      <c r="D74" s="3" t="n"/>
-      <c r="E74" s="3" t="n"/>
-      <c r="F74" s="3" t="n"/>
-      <c r="G74" s="3" t="n"/>
-      <c r="H74" s="4" t="inlineStr">
-        <is>
-          <t>6 membri</t>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -2927,22 +2927,22 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Beatrice_Bessone</t>
+          <t>lorenzo_fiorentino</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Beatrice_Bessone</t>
+          <t>lorenzo_fiorentino</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Beatrice_Bessone@naba.it</t>
+          <t>lorenzo_fiorentino@VS_MAIN</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>Psicostasia</t>
+          <t>Overload</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
@@ -2969,22 +2969,22 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Carmen_Alfano</t>
+          <t>luigi_cirelli</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Carmen_Alfano</t>
+          <t>luigi_cirelli</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Carmen_Alfano@naba.it</t>
+          <t>luigi_cirelli@VS_MAIN</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>Psicostasia</t>
+          <t>Overload</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -3011,191 +3011,191 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
+          <t>riccardo_landoni</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>riccardo_landoni</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>riccardo_landoni@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="6" customHeight="1">
+      <c r="A78" s="6" t="inlineStr"/>
+      <c r="B78" s="6" t="inlineStr"/>
+      <c r="C78" s="6" t="inlineStr"/>
+      <c r="D78" s="6" t="inlineStr"/>
+      <c r="E78" s="6" t="inlineStr"/>
+      <c r="F78" s="6" t="inlineStr"/>
+      <c r="G78" s="6" t="inlineStr"/>
+      <c r="H78" s="6" t="inlineStr"/>
+    </row>
+    <row r="79" ht="24" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>▸ Psicostasia</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="n"/>
+      <c r="C79" s="3" t="n"/>
+      <c r="D79" s="3" t="n"/>
+      <c r="E79" s="3" t="n"/>
+      <c r="F79" s="3" t="n"/>
+      <c r="G79" s="3" t="n"/>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>Beatrice_Bessone</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Beatrice_Bessone</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Beatrice_Bessone@naba.it</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Psicostasia</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano@naba.it</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Psicostasia</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
           <t>Emanuele_Boschi</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
+      <c r="C82" s="7" t="inlineStr">
         <is>
           <t>Emanuele_Boschi</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
+      <c r="D82" s="7" t="inlineStr">
         <is>
           <t>Emanuele_Boschi@naba.it</t>
         </is>
       </c>
-      <c r="E77" s="5" t="inlineStr">
+      <c r="E82" s="7" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F77" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="22" customHeight="1">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>Ge_Jiang</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>Ge_Jiang</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>Ge_Jiang@naba.it</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
-          <t>Psicostasia</t>
-        </is>
-      </c>
-      <c r="F78" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G78" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="22" customHeight="1">
-      <c r="A79" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng</t>
-        </is>
-      </c>
-      <c r="D79" s="5" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng@naba.it</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
-          <t>Psicostasia</t>
-        </is>
-      </c>
-      <c r="F79" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G79" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H79" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="22" customHeight="1">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Rotella</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Rotella</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Rotella@naba.it</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>Psicostasia</t>
-        </is>
-      </c>
-      <c r="F80" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G80" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H80" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="6" customHeight="1">
-      <c r="A81" s="6" t="inlineStr"/>
-      <c r="B81" s="6" t="inlineStr"/>
-      <c r="C81" s="6" t="inlineStr"/>
-      <c r="D81" s="6" t="inlineStr"/>
-      <c r="E81" s="6" t="inlineStr"/>
-      <c r="F81" s="6" t="inlineStr"/>
-      <c r="G81" s="6" t="inlineStr"/>
-      <c r="H81" s="6" t="inlineStr"/>
-    </row>
-    <row r="82" ht="24" customHeight="1">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>▸ Reality</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="n"/>
-      <c r="C82" s="3" t="n"/>
-      <c r="D82" s="3" t="n"/>
-      <c r="E82" s="3" t="n"/>
-      <c r="F82" s="3" t="n"/>
-      <c r="G82" s="3" t="n"/>
-      <c r="H82" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3207,22 +3207,22 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>Ge_Jiang</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>Ge_Jiang</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>isabella_bari@VS_MAIN</t>
+          <t>Ge_Jiang@naba.it</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>Reality</t>
+          <t>Psicostasia</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr">
@@ -3249,22 +3249,22 @@
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>maria_villarroel</t>
+          <t>Haotian_Cheng</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>maria_villarroel</t>
+          <t>Haotian_Cheng</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>maria_villarroel@VS_MAIN</t>
+          <t>Haotian_Cheng@naba.it</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>Reality</t>
+          <t>Psicostasia</t>
         </is>
       </c>
       <c r="F84" s="7" t="inlineStr">
@@ -3291,22 +3291,22 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>victor_fernandes</t>
+          <t>Martina_Rotella</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>victor_fernandes</t>
+          <t>Martina_Rotella</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>victor_fernandes@VS_MAIN</t>
+          <t>Martina_Rotella@naba.it</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>Reality</t>
+          <t>Psicostasia</t>
         </is>
       </c>
       <c r="F85" s="7" t="inlineStr">
@@ -3338,7 +3338,7 @@
     <row r="87" ht="24" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>▸ RitmoNulla</t>
+          <t>▸ Reality</t>
         </is>
       </c>
       <c r="B87" s="3" t="n"/>
@@ -3349,7 +3349,7 @@
       <c r="G87" s="3" t="n"/>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>6 membri</t>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
@@ -3361,22 +3361,22 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Alessandro_Caime</t>
+          <t>isabella_bari</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Alessandro_Caime</t>
+          <t>isabella_bari</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Alessandro_Caime@naba.it</t>
+          <t>isabella_bari@VS_MAIN</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>RitmoNulla</t>
+          <t>Reality</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
@@ -3403,22 +3403,22 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Feng_Yuchen</t>
+          <t>maria_villarroel</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Feng_Yuchen</t>
+          <t>maria_villarroel</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>Feng_Yuchen@naba.it</t>
+          <t>maria_villarroel@VS_MAIN</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>RitmoNulla</t>
+          <t>Reality</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
@@ -3445,191 +3445,191 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>victor_fernandes@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="6" customHeight="1">
+      <c r="A91" s="6" t="inlineStr"/>
+      <c r="B91" s="6" t="inlineStr"/>
+      <c r="C91" s="6" t="inlineStr"/>
+      <c r="D91" s="6" t="inlineStr"/>
+      <c r="E91" s="6" t="inlineStr"/>
+      <c r="F91" s="6" t="inlineStr"/>
+      <c r="G91" s="6" t="inlineStr"/>
+      <c r="H91" s="6" t="inlineStr"/>
+    </row>
+    <row r="92" ht="24" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>▸ RitmoNulla</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="n"/>
+      <c r="C92" s="3" t="n"/>
+      <c r="D92" s="3" t="n"/>
+      <c r="E92" s="3" t="n"/>
+      <c r="F92" s="3" t="n"/>
+      <c r="G92" s="3" t="n"/>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime@naba.it</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H93" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen@naba.it</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
           <t>Filippo_Damiano</t>
         </is>
       </c>
-      <c r="C90" s="5" t="inlineStr">
+      <c r="C95" s="7" t="inlineStr">
         <is>
           <t>Filippo_Damiano</t>
         </is>
       </c>
-      <c r="D90" s="5" t="inlineStr">
+      <c r="D95" s="7" t="inlineStr">
         <is>
           <t>Filippo_Damiano@naba.it</t>
         </is>
       </c>
-      <c r="E90" s="5" t="inlineStr">
+      <c r="E95" s="7" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F90" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H90" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="22" customHeight="1">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B91" s="5" t="inlineStr">
-        <is>
-          <t>Gaia_Cinti</t>
-        </is>
-      </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>Gaia_Cinti</t>
-        </is>
-      </c>
-      <c r="D91" s="5" t="inlineStr">
-        <is>
-          <t>Gaia_Cinti@naba.it</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F91" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H91" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="22" customHeight="1">
-      <c r="A92" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B92" s="5" t="inlineStr">
-        <is>
-          <t>Maria_Contesi</t>
-        </is>
-      </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>Maria_Contesi</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>Maria_Contesi@naba.it</t>
-        </is>
-      </c>
-      <c r="E92" s="5" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F92" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G92" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H92" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="22" customHeight="1">
-      <c r="A93" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B93" s="5" t="inlineStr">
-        <is>
-          <t>Raul_Chavez</t>
-        </is>
-      </c>
-      <c r="C93" s="5" t="inlineStr">
-        <is>
-          <t>Raul_Chavez</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
-        <is>
-          <t>Raul_Chavez@naba.it</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F93" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G93" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H93" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="6" customHeight="1">
-      <c r="A94" s="6" t="inlineStr"/>
-      <c r="B94" s="6" t="inlineStr"/>
-      <c r="C94" s="6" t="inlineStr"/>
-      <c r="D94" s="6" t="inlineStr"/>
-      <c r="E94" s="6" t="inlineStr"/>
-      <c r="F94" s="6" t="inlineStr"/>
-      <c r="G94" s="6" t="inlineStr"/>
-      <c r="H94" s="6" t="inlineStr"/>
-    </row>
-    <row r="95" ht="24" customHeight="1">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>▸ Roots</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="n"/>
-      <c r="C95" s="3" t="n"/>
-      <c r="D95" s="3" t="n"/>
-      <c r="E95" s="3" t="n"/>
-      <c r="F95" s="3" t="n"/>
-      <c r="G95" s="3" t="n"/>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H95" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3641,22 +3641,22 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Anna_Ebel</t>
+          <t>Gaia_Cinti</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>Anna_Ebel</t>
+          <t>Gaia_Cinti</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Anna_Ebel@naba.it</t>
+          <t>Gaia_Cinti@naba.it</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>Roots</t>
+          <t>RitmoNulla</t>
         </is>
       </c>
       <c r="F96" s="7" t="inlineStr">
@@ -3683,22 +3683,22 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>Ksenia_Puzankova</t>
+          <t>Maria_Contesi</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>Ksenia_Puzankova</t>
+          <t>Maria_Contesi</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>Ksenia_Puzankova@naba.it</t>
+          <t>Maria_Contesi@naba.it</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>Roots</t>
+          <t>RitmoNulla</t>
         </is>
       </c>
       <c r="F97" s="7" t="inlineStr">
@@ -3725,22 +3725,22 @@
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>Sevda_Sevim</t>
+          <t>Raul_Chavez</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>Sevda Aleyna Sevim</t>
+          <t>Raul_Chavez</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>SevdaAleynaSevim@naba.it</t>
+          <t>Raul_Chavez@naba.it</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>Roots</t>
+          <t>RitmoNulla</t>
         </is>
       </c>
       <c r="F98" s="7" t="inlineStr">
@@ -3772,7 +3772,7 @@
     <row r="100" ht="24" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>▸ SelfExe</t>
+          <t>▸ Roots</t>
         </is>
       </c>
       <c r="B100" s="3" t="n"/>
@@ -3783,7 +3783,7 @@
       <c r="G100" s="3" t="n"/>
       <c r="H100" s="4" t="inlineStr">
         <is>
-          <t>5 membri</t>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
@@ -3795,22 +3795,22 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Andrian_Cerga</t>
+          <t>Anna_Ebel</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Andrian_Cerga</t>
+          <t>Anna_Ebel</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Andrian_Cerga@naba.it</t>
+          <t>Anna_Ebel@naba.it</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>SelfExe</t>
+          <t>Roots</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
@@ -3837,22 +3837,22 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>Giacomo_Grioni</t>
+          <t>Ksenia_Puzankova</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Giacomo_Grioni</t>
+          <t>Ksenia_Puzankova</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>Giacomo_Grioni@naba.it</t>
+          <t>Ksenia_Puzankova@naba.it</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>SelfExe</t>
+          <t>Roots</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
@@ -3879,149 +3879,149 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Giulia_Scordino</t>
+          <t>Sevda_Sevim</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Giulia_Scordino</t>
+          <t>Sevda Aleyna Sevim</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>Giulia_Scordino@naba.it</t>
+          <t>SevdaAleynaSevim@naba.it</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
+          <t>Roots</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="6" customHeight="1">
+      <c r="A104" s="6" t="inlineStr"/>
+      <c r="B104" s="6" t="inlineStr"/>
+      <c r="C104" s="6" t="inlineStr"/>
+      <c r="D104" s="6" t="inlineStr"/>
+      <c r="E104" s="6" t="inlineStr"/>
+      <c r="F104" s="6" t="inlineStr"/>
+      <c r="G104" s="6" t="inlineStr"/>
+      <c r="H104" s="6" t="inlineStr"/>
+    </row>
+    <row r="105" ht="24" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>▸ SelfExe</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="n"/>
+      <c r="C105" s="3" t="n"/>
+      <c r="D105" s="3" t="n"/>
+      <c r="E105" s="3" t="n"/>
+      <c r="F105" s="3" t="n"/>
+      <c r="G105" s="3" t="n"/>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga@naba.it</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F103" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G103" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H103" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="22" customHeight="1">
-      <c r="A104" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B104" s="5" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni</t>
-        </is>
-      </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni</t>
-        </is>
-      </c>
-      <c r="D104" s="5" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni@naba.it</t>
-        </is>
-      </c>
-      <c r="E104" s="5" t="inlineStr">
+      <c r="F106" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G106" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H106" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni@naba.it</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F104" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G104" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H104" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="22" customHeight="1">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro</t>
-        </is>
-      </c>
-      <c r="C105" s="5" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro</t>
-        </is>
-      </c>
-      <c r="D105" s="5" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro@naba.it</t>
-        </is>
-      </c>
-      <c r="E105" s="5" t="inlineStr">
-        <is>
-          <t>SelfExe</t>
-        </is>
-      </c>
-      <c r="F105" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G105" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H105" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="6" customHeight="1">
-      <c r="A106" s="6" t="inlineStr"/>
-      <c r="B106" s="6" t="inlineStr"/>
-      <c r="C106" s="6" t="inlineStr"/>
-      <c r="D106" s="6" t="inlineStr"/>
-      <c r="E106" s="6" t="inlineStr"/>
-      <c r="F106" s="6" t="inlineStr"/>
-      <c r="G106" s="6" t="inlineStr"/>
-      <c r="H106" s="6" t="inlineStr"/>
-    </row>
-    <row r="107" ht="24" customHeight="1">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>▸ Taison</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="n"/>
-      <c r="C107" s="3" t="n"/>
-      <c r="D107" s="3" t="n"/>
-      <c r="E107" s="3" t="n"/>
-      <c r="F107" s="3" t="n"/>
-      <c r="G107" s="3" t="n"/>
-      <c r="H107" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>Giulia_Scordino</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>Giulia_Scordino</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>isabella_bari@VS_MAIN</t>
+          <t>Giulia_Scordino@naba.it</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>Taison</t>
+          <t>SelfExe</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr">
@@ -4075,22 +4075,22 @@
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>maria_villarroel</t>
+          <t>Jacopo_Ansaloni</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>maria_villarroel</t>
+          <t>Jacopo_Ansaloni</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>maria_villarroel@VS_MAIN</t>
+          <t>Jacopo_Ansaloni@naba.it</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>Taison</t>
+          <t>SelfExe</t>
         </is>
       </c>
       <c r="F109" s="7" t="inlineStr">
@@ -4117,22 +4117,22 @@
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>victor_fernandes</t>
+          <t>Sonia_DiGennaro</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>victor_fernandes</t>
+          <t>Sonia_DiGennaro</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>victor_fernandes@VS_MAIN</t>
+          <t>Sonia_DiGennaro@naba.it</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>Taison</t>
+          <t>SelfExe</t>
         </is>
       </c>
       <c r="F110" s="7" t="inlineStr">
@@ -4164,7 +4164,7 @@
     <row r="112" ht="24" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>▸ TrainOfThoughts</t>
+          <t>▸ Taison</t>
         </is>
       </c>
       <c r="B112" s="3" t="n"/>
@@ -4175,7 +4175,7 @@
       <c r="G112" s="3" t="n"/>
       <c r="H112" s="4" t="inlineStr">
         <is>
-          <t>4 membri</t>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
@@ -4187,22 +4187,22 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale</t>
+          <t>isabella_bari</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale</t>
+          <t>isabella_bari</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale@naba.it</t>
+          <t>isabella_bari@VS_MAIN</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>TrainOfThoughts</t>
+          <t>Taison</t>
         </is>
       </c>
       <c r="F113" s="5" t="inlineStr">
@@ -4229,22 +4229,22 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>Bianca_Montobbio</t>
+          <t>maria_villarroel</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>Bianca_Montobbio</t>
+          <t>maria_villarroel</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t>Bianca_Montobbio@naba.it</t>
+          <t>maria_villarroel@VS_MAIN</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>TrainOfThoughts</t>
+          <t>Taison</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
@@ -4271,107 +4271,107 @@
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>Francesca_Huang</t>
+          <t>victor_fernandes</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Francesca_Huang</t>
+          <t>victor_fernandes</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t>Francesca_Huang@naba.it</t>
+          <t>victor_fernandes@VS_MAIN</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
+          <t>Taison</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="6" customHeight="1">
+      <c r="A116" s="6" t="inlineStr"/>
+      <c r="B116" s="6" t="inlineStr"/>
+      <c r="C116" s="6" t="inlineStr"/>
+      <c r="D116" s="6" t="inlineStr"/>
+      <c r="E116" s="6" t="inlineStr"/>
+      <c r="F116" s="6" t="inlineStr"/>
+      <c r="G116" s="6" t="inlineStr"/>
+      <c r="H116" s="6" t="inlineStr"/>
+    </row>
+    <row r="117" ht="24" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>▸ TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="n"/>
+      <c r="C117" s="3" t="n"/>
+      <c r="D117" s="3" t="n"/>
+      <c r="E117" s="3" t="n"/>
+      <c r="F117" s="3" t="n"/>
+      <c r="G117" s="3" t="n"/>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale@naba.it</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
           <t>TrainOfThoughts</t>
         </is>
       </c>
-      <c r="F115" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G115" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H115" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="22" customHeight="1">
-      <c r="A116" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B116" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco</t>
-        </is>
-      </c>
-      <c r="C116" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco</t>
-        </is>
-      </c>
-      <c r="D116" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco@naba.it</t>
-        </is>
-      </c>
-      <c r="E116" s="5" t="inlineStr">
-        <is>
-          <t>TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="F116" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G116" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H116" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="6" customHeight="1">
-      <c r="A117" s="6" t="inlineStr"/>
-      <c r="B117" s="6" t="inlineStr"/>
-      <c r="C117" s="6" t="inlineStr"/>
-      <c r="D117" s="6" t="inlineStr"/>
-      <c r="E117" s="6" t="inlineStr"/>
-      <c r="F117" s="6" t="inlineStr"/>
-      <c r="G117" s="6" t="inlineStr"/>
-      <c r="H117" s="6" t="inlineStr"/>
-    </row>
-    <row r="118" ht="24" customHeight="1">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>▸ Unassigned</t>
-        </is>
-      </c>
-      <c r="B118" s="3" t="n"/>
-      <c r="C118" s="3" t="n"/>
-      <c r="D118" s="3" t="n"/>
-      <c r="E118" s="3" t="n"/>
-      <c r="F118" s="3" t="n"/>
-      <c r="G118" s="3" t="n"/>
-      <c r="H118" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F118" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G118" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H118" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4383,22 +4383,22 @@
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
-          <t>administrator</t>
+          <t>Bianca_Montobbio</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>administator</t>
+          <t>Bianca_Montobbio</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>tech@naba.it</t>
+          <t>Bianca_Montobbio@naba.it</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>TrainOfThoughts</t>
         </is>
       </c>
       <c r="F119" s="7" t="inlineStr">
@@ -4425,22 +4425,22 @@
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
-          <t>anna_brue</t>
+          <t>Francesca_Huang</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>Anna Brue</t>
+          <t>Francesca_Huang</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>anna.brue@naba.it</t>
+          <t>Francesca_Huang@naba.it</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>TrainOfThoughts</t>
         </is>
       </c>
       <c r="F120" s="7" t="inlineStr">
@@ -4467,35 +4467,189 @@
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
+          <t>Martina_Tedesco</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco@naba.it</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H121" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="6" customHeight="1">
+      <c r="A122" s="6" t="inlineStr"/>
+      <c r="B122" s="6" t="inlineStr"/>
+      <c r="C122" s="6" t="inlineStr"/>
+      <c r="D122" s="6" t="inlineStr"/>
+      <c r="E122" s="6" t="inlineStr"/>
+      <c r="F122" s="6" t="inlineStr"/>
+      <c r="G122" s="6" t="inlineStr"/>
+      <c r="H122" s="6" t="inlineStr"/>
+    </row>
+    <row r="123" ht="24" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>▸ Unassigned</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="n"/>
+      <c r="C123" s="3" t="n"/>
+      <c r="D123" s="3" t="n"/>
+      <c r="E123" s="3" t="n"/>
+      <c r="F123" s="3" t="n"/>
+      <c r="G123" s="3" t="n"/>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>administrator</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>administator</t>
+        </is>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>tech@naba.it</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H124" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="22" customHeight="1">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>anna_brue</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Anna Brue</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>anna.brue@naba.it</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H125" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
           <t>rendernodes</t>
         </is>
       </c>
-      <c r="C121" s="7" t="inlineStr">
+      <c r="C126" s="5" t="inlineStr">
         <is>
           <t>rendernodes</t>
         </is>
       </c>
-      <c r="D121" s="7" t="inlineStr">
+      <c r="D126" s="5" t="inlineStr">
         <is>
           <t>rendernodes@naba.it</t>
         </is>
       </c>
-      <c r="E121" s="7" t="inlineStr">
+      <c r="E126" s="5" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="F121" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G121" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H121" s="7" t="inlineStr">
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H126" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-15 10:37 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,13 +494,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H126"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -1543,7 +1543,7 @@
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>3 membri</t>
+          <t>1 membri</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>camilla_ferioli@studenti.naba.it</t>
+          <t>camillaf3rioli@gmail.com</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -1589,115 +1589,115 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 18:13:51</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>jon_doe</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Jon Doe</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>jon.doe@studenti.naba.it</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>Delta</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>Sì</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 18:13:51</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>tech_a</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>Tech A</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>tech_a@studenti.naba.it</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>Delta</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Sì</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="6" customHeight="1">
-      <c r="A36" s="6" t="inlineStr"/>
-      <c r="B36" s="6" t="inlineStr"/>
-      <c r="C36" s="6" t="inlineStr"/>
-      <c r="D36" s="6" t="inlineStr"/>
-      <c r="E36" s="6" t="inlineStr"/>
-      <c r="F36" s="6" t="inlineStr"/>
-      <c r="G36" s="6" t="inlineStr"/>
-      <c r="H36" s="6" t="inlineStr"/>
-    </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="34" ht="6" customHeight="1">
+      <c r="A34" s="6" t="inlineStr"/>
+      <c r="B34" s="6" t="inlineStr"/>
+      <c r="C34" s="6" t="inlineStr"/>
+      <c r="D34" s="6" t="inlineStr"/>
+      <c r="E34" s="6" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr"/>
+      <c r="H34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>▸ FloraExMachina</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="n"/>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="3" t="n"/>
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>alessandro_cova</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>alessandro_cova</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>alessandro_cova@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>FloraExMachina</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>denise_bottecchia</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>denise_bottecchia</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>denise_bottecchia@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>FloraExMachina</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -1709,17 +1709,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>alessandro_cova</t>
+          <t>kiyomi_corinti</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>alessandro_cova</t>
+          <t>kiyomi_corinti</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>alessandro_cova@VS_MAIN</t>
+          <t>kiyomi_corinti@VS_MAIN</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -1743,147 +1743,147 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>FloraExMachina</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>kiyomi_corinti</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>kiyomi_corinti</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>kiyomi_corinti@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>FloraExMachina</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="6" customHeight="1">
-      <c r="A41" s="6" t="inlineStr"/>
-      <c r="B41" s="6" t="inlineStr"/>
-      <c r="C41" s="6" t="inlineStr"/>
-      <c r="D41" s="6" t="inlineStr"/>
-      <c r="E41" s="6" t="inlineStr"/>
-      <c r="F41" s="6" t="inlineStr"/>
-      <c r="G41" s="6" t="inlineStr"/>
-      <c r="H41" s="6" t="inlineStr"/>
-    </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>▸ Gamma</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n"/>
-      <c r="G42" s="3" t="n"/>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>1 membri</t>
+    <row r="39" ht="6" customHeight="1">
+      <c r="A39" s="6" t="inlineStr"/>
+      <c r="B39" s="6" t="inlineStr"/>
+      <c r="C39" s="6" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr"/>
+      <c r="G39" s="6" t="inlineStr"/>
+      <c r="H39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>▸ HideAndSeek</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n"/>
+      <c r="C40" s="3" t="n"/>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
+      <c r="G40" s="3" t="n"/>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Jiayi_Li</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Jiayi_Li</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Jiayi_Li@naba.it</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>HideAndSeek</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Julia_Bergman</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Julia_Bergman</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Julia_Bergman@naba.it</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>HideAndSeek</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:48:23</t>
+          <t>2026-04-14 14:03:18</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>andrea_caiazzo</t>
+          <t>Wilma_Sved</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Andrea Caiazzo</t>
+          <t>wilma sved</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>andrea.caiazzo@studenti.naba.it</t>
+          <t>wilma_sved@studenti.naba.it</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Gamma</t>
+          <t>HideAndSeek</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -1893,77 +1893,77 @@
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="6" customHeight="1">
-      <c r="A44" s="6" t="inlineStr"/>
-      <c r="B44" s="6" t="inlineStr"/>
-      <c r="C44" s="6" t="inlineStr"/>
-      <c r="D44" s="6" t="inlineStr"/>
-      <c r="E44" s="6" t="inlineStr"/>
-      <c r="F44" s="6" t="inlineStr"/>
-      <c r="G44" s="6" t="inlineStr"/>
-      <c r="H44" s="6" t="inlineStr"/>
-    </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>▸ HideAndSeek</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="n"/>
-      <c r="C45" s="3" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
-      <c r="F45" s="3" t="n"/>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>4 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Jiayi_Li</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Jiayi_Li</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Jiayi_Li@naba.it</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu@naba.it</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
         <is>
           <t>HideAndSeek</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="6" customHeight="1">
+      <c r="A45" s="6" t="inlineStr"/>
+      <c r="B45" s="6" t="inlineStr"/>
+      <c r="C45" s="6" t="inlineStr"/>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" s="6" t="inlineStr"/>
+      <c r="H45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>▸ Imagery</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Julia_Bergman</t>
+          <t>Anastasia_Miani</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Julia_Bergman</t>
+          <t>Anastasia_Miani</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Julia_Bergman@naba.it</t>
+          <t>Anastasia_Miani@naba.it</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>HideAndSeek</t>
+          <t>Imagery</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2017,22 +2017,22 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Wilma_Sved</t>
+          <t>Lorenzo_Mari</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>wilma sved</t>
+          <t>Lorenzo_Mari</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>wilma_sved@studenti.naba.it</t>
+          <t>Lorenzo_Mari@naba.it</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>HideAndSeek</t>
+          <t>Imagery</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -2059,22 +2059,22 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Zhengying_Xu</t>
+          <t>Lucrezia_D'Amico</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Zhengying_Xu</t>
+          <t>Lucrezia_D'Amico</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Zhengying_Xu@naba.it</t>
+          <t>Lucrezia_D'Amico@naba.it</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>HideAndSeek</t>
+          <t>Imagery</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -2093,157 +2093,157 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="6" customHeight="1">
-      <c r="A50" s="6" t="inlineStr"/>
-      <c r="B50" s="6" t="inlineStr"/>
-      <c r="C50" s="6" t="inlineStr"/>
-      <c r="D50" s="6" t="inlineStr"/>
-      <c r="E50" s="6" t="inlineStr"/>
-      <c r="F50" s="6" t="inlineStr"/>
-      <c r="G50" s="6" t="inlineStr"/>
-      <c r="H50" s="6" t="inlineStr"/>
-    </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>▸ Imagery</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="n"/>
-      <c r="C51" s="3" t="n"/>
-      <c r="D51" s="3" t="n"/>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="3" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>6 membri</t>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Mattia_Bombace</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Mattia_Bombace</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Mattia_Bombace@naba.it</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Imagery</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Serena_Lin</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Serena_Lin</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Serena_Lin@naba.it</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Imagery</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>Anastasia_Miani</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>Anastasia_Miani</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>Anastasia_Miani@naba.it</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Youfan_Lin</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Youfan_Lin</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Youfan_Lin@naba.it</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>Imagery</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>Lorenzo_Mari</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
-        <is>
-          <t>Lorenzo_Mari</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>Lorenzo_Mari@naba.it</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>Imagery</t>
-        </is>
-      </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H53" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>Lucrezia_D'Amico</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="inlineStr">
-        <is>
-          <t>Lucrezia_D'Amico</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="inlineStr">
-        <is>
-          <t>Lucrezia_D'Amico@naba.it</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>Imagery</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H54" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="6" customHeight="1">
+      <c r="A53" s="6" t="inlineStr"/>
+      <c r="B53" s="6" t="inlineStr"/>
+      <c r="C53" s="6" t="inlineStr"/>
+      <c r="D53" s="6" t="inlineStr"/>
+      <c r="E53" s="6" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr"/>
+      <c r="G53" s="6" t="inlineStr"/>
+      <c r="H53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54" ht="24" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>▸ Kronos</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n"/>
+      <c r="C54" s="3" t="n"/>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="3" t="n"/>
+      <c r="F54" s="3" t="n"/>
+      <c r="G54" s="3" t="n"/>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
         </is>
       </c>
     </row>
@@ -2255,22 +2255,22 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Mattia_Bombace</t>
+          <t>Alberto_Cervillio</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Mattia_Bombace</t>
+          <t>Alberto_Cervillio</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Mattia_Bombace@naba.it</t>
+          <t>Alberto_Cervillio@naba.it</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Imagery</t>
+          <t>Kronos</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -2297,22 +2297,22 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Serena_Lin</t>
+          <t>Bruno_Bisogno</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Serena_Lin</t>
+          <t>Bruno_Bisogno</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Serena_Lin@naba.it</t>
+          <t>Bruno_Bisogno@naba.it</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>Imagery</t>
+          <t>Kronos</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
@@ -2339,22 +2339,22 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Youfan_Lin</t>
+          <t>Gaia_Aprile</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Youfan_Lin</t>
+          <t>Gaia_Aprile</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Youfan_Lin@naba.it</t>
+          <t>Gaia_Aprile@naba.it</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Imagery</t>
+          <t>Kronos</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
@@ -2373,115 +2373,115 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="6" customHeight="1">
-      <c r="A58" s="6" t="inlineStr"/>
-      <c r="B58" s="6" t="inlineStr"/>
-      <c r="C58" s="6" t="inlineStr"/>
-      <c r="D58" s="6" t="inlineStr"/>
-      <c r="E58" s="6" t="inlineStr"/>
-      <c r="F58" s="6" t="inlineStr"/>
-      <c r="G58" s="6" t="inlineStr"/>
-      <c r="H58" s="6" t="inlineStr"/>
-    </row>
-    <row r="59" ht="24" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>▸ Kronos</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="n"/>
-      <c r="C59" s="3" t="n"/>
-      <c r="D59" s="3" t="n"/>
-      <c r="E59" s="3" t="n"/>
-      <c r="F59" s="3" t="n"/>
-      <c r="G59" s="3" t="n"/>
-      <c r="H59" s="4" t="inlineStr">
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Jacopo_Bruschi</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Jacopo_Bruschi</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Jacopo_Bruschi@naba-da.com</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Kronos</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Riccardo_Bassani</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Riccardo_Bassani</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Riccardo_Bassani@naba.it</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Kronos</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="6" customHeight="1">
+      <c r="A60" s="6" t="inlineStr"/>
+      <c r="B60" s="6" t="inlineStr"/>
+      <c r="C60" s="6" t="inlineStr"/>
+      <c r="D60" s="6" t="inlineStr"/>
+      <c r="E60" s="6" t="inlineStr"/>
+      <c r="F60" s="6" t="inlineStr"/>
+      <c r="G60" s="6" t="inlineStr"/>
+      <c r="H60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61" ht="24" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>▸ MidnightRunners</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="n"/>
+      <c r="C61" s="3" t="n"/>
+      <c r="D61" s="3" t="n"/>
+      <c r="E61" s="3" t="n"/>
+      <c r="F61" s="3" t="n"/>
+      <c r="G61" s="3" t="n"/>
+      <c r="H61" s="4" t="inlineStr">
         <is>
           <t>5 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="22" customHeight="1">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>Alberto_Cervillio</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Alberto_Cervillio</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Alberto_Cervillio@naba.it</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Kronos</t>
-        </is>
-      </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H60" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="22" customHeight="1">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>Bruno_Bisogno</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Bruno_Bisogno</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Bruno_Bisogno@naba.it</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Kronos</t>
-        </is>
-      </c>
-      <c r="F61" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G61" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H61" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -2493,22 +2493,22 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Gaia_Aprile</t>
+          <t>Danilo_Puccio</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Gaia_Aprile</t>
+          <t>Danilo_Puccio</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Gaia_Aprile@naba.it</t>
+          <t>Danilo_Puccio@naba.it</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Kronos</t>
+          <t>MidnightRunners</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -2535,22 +2535,22 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Jacopo_Bruschi</t>
+          <t>Eros_Mussuto</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Jacopo_Bruschi</t>
+          <t>Eros_Mussuto</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Jacopo_Bruschi@naba-da.com</t>
+          <t>Eros_Mussuto@naba.it</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Kronos</t>
+          <t>MidnightRunners</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -2577,22 +2577,22 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Riccardo_Bassani</t>
+          <t>Gianluca_Lucchini</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Riccardo_Bassani</t>
+          <t>Gianluca_Lucchini</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Riccardo_Bassani@naba.it</t>
+          <t>Gianluca_Lucchini@naba.it</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>Kronos</t>
+          <t>MidnightRunners</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
@@ -2611,147 +2611,147 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="6" customHeight="1">
-      <c r="A65" s="6" t="inlineStr"/>
-      <c r="B65" s="6" t="inlineStr"/>
-      <c r="C65" s="6" t="inlineStr"/>
-      <c r="D65" s="6" t="inlineStr"/>
-      <c r="E65" s="6" t="inlineStr"/>
-      <c r="F65" s="6" t="inlineStr"/>
-      <c r="G65" s="6" t="inlineStr"/>
-      <c r="H65" s="6" t="inlineStr"/>
-    </row>
-    <row r="66" ht="24" customHeight="1">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>▸ MidnightRunners</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
-      <c r="G66" s="3" t="n"/>
-      <c r="H66" s="4" t="inlineStr">
-        <is>
-          <t>5 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="22" customHeight="1">
-      <c r="A67" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B67" s="7" t="inlineStr">
-        <is>
-          <t>Danilo_Puccio</t>
-        </is>
-      </c>
-      <c r="C67" s="7" t="inlineStr">
-        <is>
-          <t>Danilo_Puccio</t>
-        </is>
-      </c>
-      <c r="D67" s="7" t="inlineStr">
-        <is>
-          <t>Danilo_Puccio@naba.it</t>
-        </is>
-      </c>
-      <c r="E67" s="7" t="inlineStr">
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Tommaso_Mancini</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Tommaso_Mancini</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Tommaso_Mancini@naba.it</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>MidnightRunners</t>
         </is>
       </c>
-      <c r="F67" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G67" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H67" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B68" s="7" t="inlineStr">
-        <is>
-          <t>Eros_Mussuto</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>Eros_Mussuto</t>
-        </is>
-      </c>
-      <c r="D68" s="7" t="inlineStr">
-        <is>
-          <t>Eros_Mussuto@naba.it</t>
-        </is>
-      </c>
-      <c r="E68" s="7" t="inlineStr">
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Valeria_Portillo</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Valeria_Portillo</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Valeria_Portillo@naba.it</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
         <is>
           <t>MidnightRunners</t>
         </is>
       </c>
-      <c r="F68" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G68" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H68" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="6" customHeight="1">
+      <c r="A67" s="6" t="inlineStr"/>
+      <c r="B67" s="6" t="inlineStr"/>
+      <c r="C67" s="6" t="inlineStr"/>
+      <c r="D67" s="6" t="inlineStr"/>
+      <c r="E67" s="6" t="inlineStr"/>
+      <c r="F67" s="6" t="inlineStr"/>
+      <c r="G67" s="6" t="inlineStr"/>
+      <c r="H67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68" ht="24" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>▸ Omega</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="n"/>
+      <c r="C68" s="3" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
+      <c r="G68" s="3" t="n"/>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
         </is>
       </c>
     </row>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-15 10:36:52</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Gianluca_Lucchini</t>
+          <t>giovanni_visai</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Gianluca_Lucchini</t>
+          <t>Giovanni Visai</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Gianluca_Lucchini@naba.it</t>
+          <t>giovanni.visai@naba.it</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>MidnightRunners</t>
+          <t>Omega</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -2761,119 +2761,119 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B70" s="7" t="inlineStr">
-        <is>
-          <t>Tommaso_Mancini</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="inlineStr">
-        <is>
-          <t>Tommaso_Mancini</t>
-        </is>
-      </c>
-      <c r="D70" s="7" t="inlineStr">
-        <is>
-          <t>Tommaso_Mancini@naba.it</t>
-        </is>
-      </c>
-      <c r="E70" s="7" t="inlineStr">
-        <is>
-          <t>MidnightRunners</t>
-        </is>
-      </c>
-      <c r="F70" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
-        <is>
-          <t>Valeria_Portillo</t>
-        </is>
-      </c>
-      <c r="C71" s="7" t="inlineStr">
-        <is>
-          <t>Valeria_Portillo</t>
-        </is>
-      </c>
-      <c r="D71" s="7" t="inlineStr">
-        <is>
-          <t>Valeria_Portillo@naba.it</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="inlineStr">
-        <is>
-          <t>MidnightRunners</t>
-        </is>
-      </c>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="6" customHeight="1">
-      <c r="A72" s="6" t="inlineStr"/>
-      <c r="B72" s="6" t="inlineStr"/>
-      <c r="C72" s="6" t="inlineStr"/>
-      <c r="D72" s="6" t="inlineStr"/>
-      <c r="E72" s="6" t="inlineStr"/>
-      <c r="F72" s="6" t="inlineStr"/>
-      <c r="G72" s="6" t="inlineStr"/>
-      <c r="H72" s="6" t="inlineStr"/>
-    </row>
-    <row r="73" ht="24" customHeight="1">
-      <c r="A73" s="2" t="inlineStr">
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="6" customHeight="1">
+      <c r="A70" s="6" t="inlineStr"/>
+      <c r="B70" s="6" t="inlineStr"/>
+      <c r="C70" s="6" t="inlineStr"/>
+      <c r="D70" s="6" t="inlineStr"/>
+      <c r="E70" s="6" t="inlineStr"/>
+      <c r="F70" s="6" t="inlineStr"/>
+      <c r="G70" s="6" t="inlineStr"/>
+      <c r="H70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71" ht="24" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>▸ Overload</t>
         </is>
       </c>
-      <c r="B73" s="3" t="n"/>
-      <c r="C73" s="3" t="n"/>
-      <c r="D73" s="3" t="n"/>
-      <c r="E73" s="3" t="n"/>
-      <c r="F73" s="3" t="n"/>
-      <c r="G73" s="3" t="n"/>
-      <c r="H73" s="4" t="inlineStr">
+      <c r="B71" s="3" t="n"/>
+      <c r="C71" s="3" t="n"/>
+      <c r="D71" s="3" t="n"/>
+      <c r="E71" s="3" t="n"/>
+      <c r="F71" s="3" t="n"/>
+      <c r="G71" s="3" t="n"/>
+      <c r="H71" s="4" t="inlineStr">
         <is>
           <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>gabriele_dallari</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>gabriele_dallari</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>gabriele_dallari@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>lorenzo_fiorentino</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>lorenzo_fiorentino</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>lorenzo_fiorentino@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -2885,17 +2885,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>gabriele_dallari</t>
+          <t>luigi_cirelli</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>gabriele_dallari</t>
+          <t>luigi_cirelli</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>gabriele_dallari@VS_MAIN</t>
+          <t>luigi_cirelli@VS_MAIN</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -2927,17 +2927,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>lorenzo_fiorentino</t>
+          <t>riccardo_landoni</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>lorenzo_fiorentino</t>
+          <t>riccardo_landoni</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>lorenzo_fiorentino@VS_MAIN</t>
+          <t>riccardo_landoni@VS_MAIN</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -2961,115 +2961,115 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="22" customHeight="1">
-      <c r="A76" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>luigi_cirelli</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>luigi_cirelli</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="inlineStr">
-        <is>
-          <t>luigi_cirelli@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E76" s="5" t="inlineStr">
-        <is>
-          <t>Overload</t>
-        </is>
-      </c>
-      <c r="F76" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G76" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H76" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="22" customHeight="1">
-      <c r="A77" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>riccardo_landoni</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>riccardo_landoni</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>riccardo_landoni@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>Overload</t>
-        </is>
-      </c>
-      <c r="F77" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="6" customHeight="1">
-      <c r="A78" s="6" t="inlineStr"/>
-      <c r="B78" s="6" t="inlineStr"/>
-      <c r="C78" s="6" t="inlineStr"/>
-      <c r="D78" s="6" t="inlineStr"/>
-      <c r="E78" s="6" t="inlineStr"/>
-      <c r="F78" s="6" t="inlineStr"/>
-      <c r="G78" s="6" t="inlineStr"/>
-      <c r="H78" s="6" t="inlineStr"/>
-    </row>
-    <row r="79" ht="24" customHeight="1">
-      <c r="A79" s="2" t="inlineStr">
+    <row r="76" ht="6" customHeight="1">
+      <c r="A76" s="6" t="inlineStr"/>
+      <c r="B76" s="6" t="inlineStr"/>
+      <c r="C76" s="6" t="inlineStr"/>
+      <c r="D76" s="6" t="inlineStr"/>
+      <c r="E76" s="6" t="inlineStr"/>
+      <c r="F76" s="6" t="inlineStr"/>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77" ht="24" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>▸ Psicostasia</t>
         </is>
       </c>
-      <c r="B79" s="3" t="n"/>
-      <c r="C79" s="3" t="n"/>
-      <c r="D79" s="3" t="n"/>
-      <c r="E79" s="3" t="n"/>
-      <c r="F79" s="3" t="n"/>
-      <c r="G79" s="3" t="n"/>
-      <c r="H79" s="4" t="inlineStr">
+      <c r="B77" s="3" t="n"/>
+      <c r="C77" s="3" t="n"/>
+      <c r="D77" s="3" t="n"/>
+      <c r="E77" s="3" t="n"/>
+      <c r="F77" s="3" t="n"/>
+      <c r="G77" s="3" t="n"/>
+      <c r="H77" s="4" t="inlineStr">
         <is>
           <t>6 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Beatrice_Bessone</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Beatrice_Bessone</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Beatrice_Bessone@naba.it</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>Psicostasia</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano@naba.it</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Psicostasia</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3081,17 +3081,17 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>Beatrice_Bessone</t>
+          <t>Emanuele_Boschi</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>Beatrice_Bessone</t>
+          <t>Emanuele_Boschi</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>Beatrice_Bessone@naba.it</t>
+          <t>Emanuele_Boschi@naba.it</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
@@ -3123,17 +3123,17 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Carmen_Alfano</t>
+          <t>Ge_Jiang</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Carmen_Alfano</t>
+          <t>Ge_Jiang</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>Carmen_Alfano@naba.it</t>
+          <t>Ge_Jiang@naba.it</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
@@ -3165,17 +3165,17 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>Emanuele_Boschi</t>
+          <t>Haotian_Cheng</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>Emanuele_Boschi</t>
+          <t>Haotian_Cheng</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>Emanuele_Boschi@naba.it</t>
+          <t>Haotian_Cheng@naba.it</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
@@ -3207,17 +3207,17 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>Ge_Jiang</t>
+          <t>Martina_Rotella</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Ge_Jiang</t>
+          <t>Martina_Rotella</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Ge_Jiang@naba.it</t>
+          <t>Martina_Rotella@naba.it</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -3241,115 +3241,115 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="22" customHeight="1">
-      <c r="A84" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B84" s="7" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng</t>
-        </is>
-      </c>
-      <c r="C84" s="7" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng</t>
-        </is>
-      </c>
-      <c r="D84" s="7" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng@naba.it</t>
-        </is>
-      </c>
-      <c r="E84" s="7" t="inlineStr">
-        <is>
-          <t>Psicostasia</t>
-        </is>
-      </c>
-      <c r="F84" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G84" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H84" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="22" customHeight="1">
-      <c r="A85" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B85" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Rotella</t>
-        </is>
-      </c>
-      <c r="C85" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Rotella</t>
-        </is>
-      </c>
-      <c r="D85" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Rotella@naba.it</t>
-        </is>
-      </c>
-      <c r="E85" s="7" t="inlineStr">
-        <is>
-          <t>Psicostasia</t>
-        </is>
-      </c>
-      <c r="F85" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G85" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H85" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="6" customHeight="1">
-      <c r="A86" s="6" t="inlineStr"/>
-      <c r="B86" s="6" t="inlineStr"/>
-      <c r="C86" s="6" t="inlineStr"/>
-      <c r="D86" s="6" t="inlineStr"/>
-      <c r="E86" s="6" t="inlineStr"/>
-      <c r="F86" s="6" t="inlineStr"/>
-      <c r="G86" s="6" t="inlineStr"/>
-      <c r="H86" s="6" t="inlineStr"/>
-    </row>
-    <row r="87" ht="24" customHeight="1">
-      <c r="A87" s="2" t="inlineStr">
+    <row r="84" ht="6" customHeight="1">
+      <c r="A84" s="6" t="inlineStr"/>
+      <c r="B84" s="6" t="inlineStr"/>
+      <c r="C84" s="6" t="inlineStr"/>
+      <c r="D84" s="6" t="inlineStr"/>
+      <c r="E84" s="6" t="inlineStr"/>
+      <c r="F84" s="6" t="inlineStr"/>
+      <c r="G84" s="6" t="inlineStr"/>
+      <c r="H84" s="6" t="inlineStr"/>
+    </row>
+    <row r="85" ht="24" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>▸ Reality</t>
         </is>
       </c>
-      <c r="B87" s="3" t="n"/>
-      <c r="C87" s="3" t="n"/>
-      <c r="D87" s="3" t="n"/>
-      <c r="E87" s="3" t="n"/>
-      <c r="F87" s="3" t="n"/>
-      <c r="G87" s="3" t="n"/>
-      <c r="H87" s="4" t="inlineStr">
+      <c r="B85" s="3" t="n"/>
+      <c r="C85" s="3" t="n"/>
+      <c r="D85" s="3" t="n"/>
+      <c r="E85" s="3" t="n"/>
+      <c r="F85" s="3" t="n"/>
+      <c r="G85" s="3" t="n"/>
+      <c r="H85" s="4" t="inlineStr">
         <is>
           <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>isabella_bari</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>isabella_bari</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>isabella_bari@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>maria_villarroel</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>maria_villarroel</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>maria_villarroel@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3361,17 +3361,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>victor_fernandes</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>victor_fernandes</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari@VS_MAIN</t>
+          <t>victor_fernandes@VS_MAIN</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -3395,115 +3395,115 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="22" customHeight="1">
-      <c r="A89" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel</t>
-        </is>
-      </c>
-      <c r="C89" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel</t>
-        </is>
-      </c>
-      <c r="D89" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="inlineStr">
-        <is>
-          <t>Reality</t>
-        </is>
-      </c>
-      <c r="F89" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G89" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H89" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="22" customHeight="1">
-      <c r="A90" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B90" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="D90" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>Reality</t>
-        </is>
-      </c>
-      <c r="F90" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H90" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="6" customHeight="1">
-      <c r="A91" s="6" t="inlineStr"/>
-      <c r="B91" s="6" t="inlineStr"/>
-      <c r="C91" s="6" t="inlineStr"/>
-      <c r="D91" s="6" t="inlineStr"/>
-      <c r="E91" s="6" t="inlineStr"/>
-      <c r="F91" s="6" t="inlineStr"/>
-      <c r="G91" s="6" t="inlineStr"/>
-      <c r="H91" s="6" t="inlineStr"/>
-    </row>
-    <row r="92" ht="24" customHeight="1">
-      <c r="A92" s="2" t="inlineStr">
+    <row r="89" ht="6" customHeight="1">
+      <c r="A89" s="6" t="inlineStr"/>
+      <c r="B89" s="6" t="inlineStr"/>
+      <c r="C89" s="6" t="inlineStr"/>
+      <c r="D89" s="6" t="inlineStr"/>
+      <c r="E89" s="6" t="inlineStr"/>
+      <c r="F89" s="6" t="inlineStr"/>
+      <c r="G89" s="6" t="inlineStr"/>
+      <c r="H89" s="6" t="inlineStr"/>
+    </row>
+    <row r="90" ht="24" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>▸ RitmoNulla</t>
         </is>
       </c>
-      <c r="B92" s="3" t="n"/>
-      <c r="C92" s="3" t="n"/>
-      <c r="D92" s="3" t="n"/>
-      <c r="E92" s="3" t="n"/>
-      <c r="F92" s="3" t="n"/>
-      <c r="G92" s="3" t="n"/>
-      <c r="H92" s="4" t="inlineStr">
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="3" t="n"/>
+      <c r="D90" s="3" t="n"/>
+      <c r="E90" s="3" t="n"/>
+      <c r="F90" s="3" t="n"/>
+      <c r="G90" s="3" t="n"/>
+      <c r="H90" s="4" t="inlineStr">
         <is>
           <t>6 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime@naba.it</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen@naba.it</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3515,17 +3515,17 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Alessandro_Caime</t>
+          <t>Filippo_Damiano</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>Alessandro_Caime</t>
+          <t>Filippo_Damiano</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Alessandro_Caime@naba.it</t>
+          <t>Filippo_Damiano@naba.it</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
@@ -3557,17 +3557,17 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>Feng_Yuchen</t>
+          <t>Gaia_Cinti</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>Feng_Yuchen</t>
+          <t>Gaia_Cinti</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>Feng_Yuchen@naba.it</t>
+          <t>Gaia_Cinti@naba.it</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
@@ -3599,17 +3599,17 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Filippo_Damiano</t>
+          <t>Maria_Contesi</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Filippo_Damiano</t>
+          <t>Maria_Contesi</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>Filippo_Damiano@naba.it</t>
+          <t>Maria_Contesi@naba.it</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Gaia_Cinti</t>
+          <t>Raul_Chavez</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>Gaia_Cinti</t>
+          <t>Raul_Chavez</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Gaia_Cinti@naba.it</t>
+          <t>Raul_Chavez@naba.it</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
@@ -3675,115 +3675,115 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="22" customHeight="1">
-      <c r="A97" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B97" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi</t>
-        </is>
-      </c>
-      <c r="C97" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi</t>
-        </is>
-      </c>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi@naba.it</t>
-        </is>
-      </c>
-      <c r="E97" s="7" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F97" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G97" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H97" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="22" customHeight="1">
-      <c r="A98" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B98" s="7" t="inlineStr">
-        <is>
-          <t>Raul_Chavez</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr">
-        <is>
-          <t>Raul_Chavez</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>Raul_Chavez@naba.it</t>
-        </is>
-      </c>
-      <c r="E98" s="7" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F98" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G98" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H98" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="6" customHeight="1">
-      <c r="A99" s="6" t="inlineStr"/>
-      <c r="B99" s="6" t="inlineStr"/>
-      <c r="C99" s="6" t="inlineStr"/>
-      <c r="D99" s="6" t="inlineStr"/>
-      <c r="E99" s="6" t="inlineStr"/>
-      <c r="F99" s="6" t="inlineStr"/>
-      <c r="G99" s="6" t="inlineStr"/>
-      <c r="H99" s="6" t="inlineStr"/>
-    </row>
-    <row r="100" ht="24" customHeight="1">
-      <c r="A100" s="2" t="inlineStr">
+    <row r="97" ht="6" customHeight="1">
+      <c r="A97" s="6" t="inlineStr"/>
+      <c r="B97" s="6" t="inlineStr"/>
+      <c r="C97" s="6" t="inlineStr"/>
+      <c r="D97" s="6" t="inlineStr"/>
+      <c r="E97" s="6" t="inlineStr"/>
+      <c r="F97" s="6" t="inlineStr"/>
+      <c r="G97" s="6" t="inlineStr"/>
+      <c r="H97" s="6" t="inlineStr"/>
+    </row>
+    <row r="98" ht="24" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
         <is>
           <t>▸ Roots</t>
         </is>
       </c>
-      <c r="B100" s="3" t="n"/>
-      <c r="C100" s="3" t="n"/>
-      <c r="D100" s="3" t="n"/>
-      <c r="E100" s="3" t="n"/>
-      <c r="F100" s="3" t="n"/>
-      <c r="G100" s="3" t="n"/>
-      <c r="H100" s="4" t="inlineStr">
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="3" t="n"/>
+      <c r="D98" s="3" t="n"/>
+      <c r="E98" s="3" t="n"/>
+      <c r="F98" s="3" t="n"/>
+      <c r="G98" s="3" t="n"/>
+      <c r="H98" s="4" t="inlineStr">
         <is>
           <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Anna_Ebel</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Anna_Ebel</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Anna_Ebel@naba.it</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>Roots</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Ksenia_Puzankova</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Ksenia_Puzankova</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Ksenia_Puzankova@naba.it</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>Roots</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3795,17 +3795,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Anna_Ebel</t>
+          <t>Sevda_Sevim</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Anna_Ebel</t>
+          <t>Sevda Aleyna Sevim</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Anna_Ebel@naba.it</t>
+          <t>SevdaAleynaSevim@naba.it</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -3829,115 +3829,115 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="22" customHeight="1">
-      <c r="A102" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B102" s="5" t="inlineStr">
-        <is>
-          <t>Ksenia_Puzankova</t>
-        </is>
-      </c>
-      <c r="C102" s="5" t="inlineStr">
-        <is>
-          <t>Ksenia_Puzankova</t>
-        </is>
-      </c>
-      <c r="D102" s="5" t="inlineStr">
-        <is>
-          <t>Ksenia_Puzankova@naba.it</t>
-        </is>
-      </c>
-      <c r="E102" s="5" t="inlineStr">
-        <is>
-          <t>Roots</t>
-        </is>
-      </c>
-      <c r="F102" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G102" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H102" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="22" customHeight="1">
-      <c r="A103" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B103" s="5" t="inlineStr">
-        <is>
-          <t>Sevda_Sevim</t>
-        </is>
-      </c>
-      <c r="C103" s="5" t="inlineStr">
-        <is>
-          <t>Sevda Aleyna Sevim</t>
-        </is>
-      </c>
-      <c r="D103" s="5" t="inlineStr">
-        <is>
-          <t>SevdaAleynaSevim@naba.it</t>
-        </is>
-      </c>
-      <c r="E103" s="5" t="inlineStr">
-        <is>
-          <t>Roots</t>
-        </is>
-      </c>
-      <c r="F103" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G103" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H103" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="6" customHeight="1">
-      <c r="A104" s="6" t="inlineStr"/>
-      <c r="B104" s="6" t="inlineStr"/>
-      <c r="C104" s="6" t="inlineStr"/>
-      <c r="D104" s="6" t="inlineStr"/>
-      <c r="E104" s="6" t="inlineStr"/>
-      <c r="F104" s="6" t="inlineStr"/>
-      <c r="G104" s="6" t="inlineStr"/>
-      <c r="H104" s="6" t="inlineStr"/>
-    </row>
-    <row r="105" ht="24" customHeight="1">
-      <c r="A105" s="2" t="inlineStr">
+    <row r="102" ht="6" customHeight="1">
+      <c r="A102" s="6" t="inlineStr"/>
+      <c r="B102" s="6" t="inlineStr"/>
+      <c r="C102" s="6" t="inlineStr"/>
+      <c r="D102" s="6" t="inlineStr"/>
+      <c r="E102" s="6" t="inlineStr"/>
+      <c r="F102" s="6" t="inlineStr"/>
+      <c r="G102" s="6" t="inlineStr"/>
+      <c r="H102" s="6" t="inlineStr"/>
+    </row>
+    <row r="103" ht="24" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
         <is>
           <t>▸ SelfExe</t>
         </is>
       </c>
-      <c r="B105" s="3" t="n"/>
-      <c r="C105" s="3" t="n"/>
-      <c r="D105" s="3" t="n"/>
-      <c r="E105" s="3" t="n"/>
-      <c r="F105" s="3" t="n"/>
-      <c r="G105" s="3" t="n"/>
-      <c r="H105" s="4" t="inlineStr">
+      <c r="B103" s="3" t="n"/>
+      <c r="C103" s="3" t="n"/>
+      <c r="D103" s="3" t="n"/>
+      <c r="E103" s="3" t="n"/>
+      <c r="F103" s="3" t="n"/>
+      <c r="G103" s="3" t="n"/>
+      <c r="H103" s="4" t="inlineStr">
         <is>
           <t>5 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga@naba.it</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="inlineStr">
+        <is>
+          <t>SelfExe</t>
+        </is>
+      </c>
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G104" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H104" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni@naba.it</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="inlineStr">
+        <is>
+          <t>SelfExe</t>
+        </is>
+      </c>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H105" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3949,17 +3949,17 @@
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>Andrian_Cerga</t>
+          <t>Giulia_Scordino</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>Andrian_Cerga</t>
+          <t>Giulia_Scordino</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>Andrian_Cerga@naba.it</t>
+          <t>Giulia_Scordino@naba.it</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
@@ -3991,17 +3991,17 @@
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>Giacomo_Grioni</t>
+          <t>Jacopo_Ansaloni</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>Giacomo_Grioni</t>
+          <t>Jacopo_Ansaloni</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>Giacomo_Grioni@naba.it</t>
+          <t>Jacopo_Ansaloni@naba.it</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
@@ -4033,17 +4033,17 @@
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>Giulia_Scordino</t>
+          <t>Sonia_DiGennaro</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>Giulia_Scordino</t>
+          <t>Sonia_DiGennaro</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>Giulia_Scordino@naba.it</t>
+          <t>Sonia_DiGennaro@naba.it</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
@@ -4067,115 +4067,115 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="22" customHeight="1">
-      <c r="A109" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B109" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni</t>
-        </is>
-      </c>
-      <c r="C109" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni</t>
-        </is>
-      </c>
-      <c r="D109" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni@naba.it</t>
-        </is>
-      </c>
-      <c r="E109" s="7" t="inlineStr">
-        <is>
-          <t>SelfExe</t>
-        </is>
-      </c>
-      <c r="F109" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G109" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H109" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="22" customHeight="1">
-      <c r="A110" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B110" s="7" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro</t>
-        </is>
-      </c>
-      <c r="C110" s="7" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro</t>
-        </is>
-      </c>
-      <c r="D110" s="7" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro@naba.it</t>
-        </is>
-      </c>
-      <c r="E110" s="7" t="inlineStr">
-        <is>
-          <t>SelfExe</t>
-        </is>
-      </c>
-      <c r="F110" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G110" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H110" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="6" customHeight="1">
-      <c r="A111" s="6" t="inlineStr"/>
-      <c r="B111" s="6" t="inlineStr"/>
-      <c r="C111" s="6" t="inlineStr"/>
-      <c r="D111" s="6" t="inlineStr"/>
-      <c r="E111" s="6" t="inlineStr"/>
-      <c r="F111" s="6" t="inlineStr"/>
-      <c r="G111" s="6" t="inlineStr"/>
-      <c r="H111" s="6" t="inlineStr"/>
-    </row>
-    <row r="112" ht="24" customHeight="1">
-      <c r="A112" s="2" t="inlineStr">
+    <row r="109" ht="6" customHeight="1">
+      <c r="A109" s="6" t="inlineStr"/>
+      <c r="B109" s="6" t="inlineStr"/>
+      <c r="C109" s="6" t="inlineStr"/>
+      <c r="D109" s="6" t="inlineStr"/>
+      <c r="E109" s="6" t="inlineStr"/>
+      <c r="F109" s="6" t="inlineStr"/>
+      <c r="G109" s="6" t="inlineStr"/>
+      <c r="H109" s="6" t="inlineStr"/>
+    </row>
+    <row r="110" ht="24" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>▸ Taison</t>
         </is>
       </c>
-      <c r="B112" s="3" t="n"/>
-      <c r="C112" s="3" t="n"/>
-      <c r="D112" s="3" t="n"/>
-      <c r="E112" s="3" t="n"/>
-      <c r="F112" s="3" t="n"/>
-      <c r="G112" s="3" t="n"/>
-      <c r="H112" s="4" t="inlineStr">
+      <c r="B110" s="3" t="n"/>
+      <c r="C110" s="3" t="n"/>
+      <c r="D110" s="3" t="n"/>
+      <c r="E110" s="3" t="n"/>
+      <c r="F110" s="3" t="n"/>
+      <c r="G110" s="3" t="n"/>
+      <c r="H110" s="4" t="inlineStr">
         <is>
           <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>isabella_bari</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>isabella_bari</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>isabella_bari@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>Taison</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>maria_villarroel</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>maria_villarroel</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>maria_villarroel@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>Taison</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4187,17 +4187,17 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>victor_fernandes</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>victor_fernandes</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari@VS_MAIN</t>
+          <t>victor_fernandes@VS_MAIN</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
@@ -4221,115 +4221,115 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="22" customHeight="1">
-      <c r="A114" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B114" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel</t>
-        </is>
-      </c>
-      <c r="D114" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>Taison</t>
-        </is>
-      </c>
-      <c r="F114" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G114" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H114" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="22" customHeight="1">
-      <c r="A115" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B115" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="D115" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="inlineStr">
-        <is>
-          <t>Taison</t>
-        </is>
-      </c>
-      <c r="F115" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G115" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H115" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="6" customHeight="1">
-      <c r="A116" s="6" t="inlineStr"/>
-      <c r="B116" s="6" t="inlineStr"/>
-      <c r="C116" s="6" t="inlineStr"/>
-      <c r="D116" s="6" t="inlineStr"/>
-      <c r="E116" s="6" t="inlineStr"/>
-      <c r="F116" s="6" t="inlineStr"/>
-      <c r="G116" s="6" t="inlineStr"/>
-      <c r="H116" s="6" t="inlineStr"/>
-    </row>
-    <row r="117" ht="24" customHeight="1">
-      <c r="A117" s="2" t="inlineStr">
+    <row r="114" ht="6" customHeight="1">
+      <c r="A114" s="6" t="inlineStr"/>
+      <c r="B114" s="6" t="inlineStr"/>
+      <c r="C114" s="6" t="inlineStr"/>
+      <c r="D114" s="6" t="inlineStr"/>
+      <c r="E114" s="6" t="inlineStr"/>
+      <c r="F114" s="6" t="inlineStr"/>
+      <c r="G114" s="6" t="inlineStr"/>
+      <c r="H114" s="6" t="inlineStr"/>
+    </row>
+    <row r="115" ht="24" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
         <is>
           <t>▸ TrainOfThoughts</t>
         </is>
       </c>
-      <c r="B117" s="3" t="n"/>
-      <c r="C117" s="3" t="n"/>
-      <c r="D117" s="3" t="n"/>
-      <c r="E117" s="3" t="n"/>
-      <c r="F117" s="3" t="n"/>
-      <c r="G117" s="3" t="n"/>
-      <c r="H117" s="4" t="inlineStr">
+      <c r="B115" s="3" t="n"/>
+      <c r="C115" s="3" t="n"/>
+      <c r="D115" s="3" t="n"/>
+      <c r="E115" s="3" t="n"/>
+      <c r="F115" s="3" t="n"/>
+      <c r="G115" s="3" t="n"/>
+      <c r="H115" s="4" t="inlineStr">
         <is>
           <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale@naba.it</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="inlineStr">
+        <is>
+          <t>TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G116" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H116" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>Bianca_Montobbio</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>Bianca_Montobbio</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>Bianca_Montobbio@naba.it</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G117" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H117" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4341,17 +4341,17 @@
       </c>
       <c r="B118" s="7" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale</t>
+          <t>Francesca_Huang</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale</t>
+          <t>Francesca_Huang</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale@naba.it</t>
+          <t>Francesca_Huang@naba.it</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
@@ -4383,17 +4383,17 @@
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
-          <t>Bianca_Montobbio</t>
+          <t>Martina_Tedesco</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>Bianca_Montobbio</t>
+          <t>Martina_Tedesco</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>Bianca_Montobbio@naba.it</t>
+          <t>Martina_Tedesco@naba.it</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
@@ -4417,115 +4417,115 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="22" customHeight="1">
-      <c r="A120" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B120" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang</t>
-        </is>
-      </c>
-      <c r="C120" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang</t>
-        </is>
-      </c>
-      <c r="D120" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang@naba.it</t>
-        </is>
-      </c>
-      <c r="E120" s="7" t="inlineStr">
-        <is>
-          <t>TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="F120" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G120" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H120" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="22" customHeight="1">
-      <c r="A121" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B121" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco</t>
-        </is>
-      </c>
-      <c r="C121" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco</t>
-        </is>
-      </c>
-      <c r="D121" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco@naba.it</t>
-        </is>
-      </c>
-      <c r="E121" s="7" t="inlineStr">
-        <is>
-          <t>TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="F121" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G121" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H121" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="6" customHeight="1">
-      <c r="A122" s="6" t="inlineStr"/>
-      <c r="B122" s="6" t="inlineStr"/>
-      <c r="C122" s="6" t="inlineStr"/>
-      <c r="D122" s="6" t="inlineStr"/>
-      <c r="E122" s="6" t="inlineStr"/>
-      <c r="F122" s="6" t="inlineStr"/>
-      <c r="G122" s="6" t="inlineStr"/>
-      <c r="H122" s="6" t="inlineStr"/>
-    </row>
-    <row r="123" ht="24" customHeight="1">
-      <c r="A123" s="2" t="inlineStr">
+    <row r="120" ht="6" customHeight="1">
+      <c r="A120" s="6" t="inlineStr"/>
+      <c r="B120" s="6" t="inlineStr"/>
+      <c r="C120" s="6" t="inlineStr"/>
+      <c r="D120" s="6" t="inlineStr"/>
+      <c r="E120" s="6" t="inlineStr"/>
+      <c r="F120" s="6" t="inlineStr"/>
+      <c r="G120" s="6" t="inlineStr"/>
+      <c r="H120" s="6" t="inlineStr"/>
+    </row>
+    <row r="121" ht="24" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
         <is>
           <t>▸ Unassigned</t>
         </is>
       </c>
-      <c r="B123" s="3" t="n"/>
-      <c r="C123" s="3" t="n"/>
-      <c r="D123" s="3" t="n"/>
-      <c r="E123" s="3" t="n"/>
-      <c r="F123" s="3" t="n"/>
-      <c r="G123" s="3" t="n"/>
-      <c r="H123" s="4" t="inlineStr">
+      <c r="B121" s="3" t="n"/>
+      <c r="C121" s="3" t="n"/>
+      <c r="D121" s="3" t="n"/>
+      <c r="E121" s="3" t="n"/>
+      <c r="F121" s="3" t="n"/>
+      <c r="G121" s="3" t="n"/>
+      <c r="H121" s="4" t="inlineStr">
         <is>
           <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>administrator</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>administator</t>
+        </is>
+      </c>
+      <c r="D122" s="5" t="inlineStr">
+        <is>
+          <t>tech@naba.it</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H122" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>anna_brue</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Anna Brue</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>anna.brue@naba.it</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4537,17 +4537,17 @@
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>administrator</t>
+          <t>rendernodes</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>administator</t>
+          <t>rendernodes</t>
         </is>
       </c>
       <c r="D124" s="5" t="inlineStr">
         <is>
-          <t>tech@naba.it</t>
+          <t>rendernodes@naba.it</t>
         </is>
       </c>
       <c r="E124" s="5" t="inlineStr">
@@ -4566,90 +4566,6 @@
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="22" customHeight="1">
-      <c r="A125" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B125" s="5" t="inlineStr">
-        <is>
-          <t>anna_brue</t>
-        </is>
-      </c>
-      <c r="C125" s="5" t="inlineStr">
-        <is>
-          <t>Anna Brue</t>
-        </is>
-      </c>
-      <c r="D125" s="5" t="inlineStr">
-        <is>
-          <t>anna.brue@naba.it</t>
-        </is>
-      </c>
-      <c r="E125" s="5" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="F125" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G125" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H125" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="22" customHeight="1">
-      <c r="A126" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B126" s="5" t="inlineStr">
-        <is>
-          <t>rendernodes</t>
-        </is>
-      </c>
-      <c r="C126" s="5" t="inlineStr">
-        <is>
-          <t>rendernodes</t>
-        </is>
-      </c>
-      <c r="D126" s="5" t="inlineStr">
-        <is>
-          <t>rendernodes@naba.it</t>
-        </is>
-      </c>
-      <c r="E126" s="5" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="F126" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G126" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H126" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-16 12:26 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H124"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1532,7 +1532,7 @@
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>▸ Delta</t>
+          <t>▸ Epsilon</t>
         </is>
       </c>
       <c r="B32" s="3" t="n"/>
@@ -1550,27 +1550,27 @@
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 18:13:51</t>
+          <t>2026-04-16 12:26:25</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>camilla_ferioli</t>
+          <t>emanuele_lomello</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Camilla Ferioli</t>
+          <t>Emanuele Lomello</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>camillaf3rioli@gmail.com</t>
+          <t>lvilla.garbage@gmail.com</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Delta</t>
+          <t>Epsilon</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -2708,7 +2708,7 @@
     <row r="68" ht="24" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>▸ Omega</t>
+          <t>▸ Overload</t>
         </is>
       </c>
       <c r="B68" s="3" t="n"/>
@@ -2719,39 +2719,39 @@
       <c r="G68" s="3" t="n"/>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>1 membri</t>
+          <t>4 membri</t>
         </is>
       </c>
     </row>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>2026-04-15 10:36:52</t>
+          <t>2026-04-14 14:03:18</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>giovanni_visai</t>
+          <t>gabriele_dallari</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Giovanni Visai</t>
+          <t>gabriele_dallari</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>giovanni.visai@naba.it</t>
+          <t>gabriele_dallari@VS_MAIN</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Omega</t>
+          <t>Overload</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -2761,161 +2761,161 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="6" customHeight="1">
-      <c r="A70" s="6" t="inlineStr"/>
-      <c r="B70" s="6" t="inlineStr"/>
-      <c r="C70" s="6" t="inlineStr"/>
-      <c r="D70" s="6" t="inlineStr"/>
-      <c r="E70" s="6" t="inlineStr"/>
-      <c r="F70" s="6" t="inlineStr"/>
-      <c r="G70" s="6" t="inlineStr"/>
-      <c r="H70" s="6" t="inlineStr"/>
-    </row>
-    <row r="71" ht="24" customHeight="1">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>▸ Overload</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="n"/>
-      <c r="C71" s="3" t="n"/>
-      <c r="D71" s="3" t="n"/>
-      <c r="E71" s="3" t="n"/>
-      <c r="F71" s="3" t="n"/>
-      <c r="G71" s="3" t="n"/>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>4 membri</t>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>lorenzo_fiorentino</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>lorenzo_fiorentino</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>lorenzo_fiorentino@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>luigi_cirelli</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>luigi_cirelli</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>luigi_cirelli@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>gabriele_dallari</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>gabriele_dallari</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>gabriele_dallari@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>riccardo_landoni</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>riccardo_landoni</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>riccardo_landoni@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
         <is>
           <t>Overload</t>
         </is>
       </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H72" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="22" customHeight="1">
-      <c r="A73" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>lorenzo_fiorentino</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>lorenzo_fiorentino</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>lorenzo_fiorentino@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>Overload</t>
-        </is>
-      </c>
-      <c r="F73" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H73" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>luigi_cirelli</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>luigi_cirelli</t>
-        </is>
-      </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>luigi_cirelli@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="inlineStr">
-        <is>
-          <t>Overload</t>
-        </is>
-      </c>
-      <c r="F74" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G74" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H74" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="6" customHeight="1">
+      <c r="A73" s="6" t="inlineStr"/>
+      <c r="B73" s="6" t="inlineStr"/>
+      <c r="C73" s="6" t="inlineStr"/>
+      <c r="D73" s="6" t="inlineStr"/>
+      <c r="E73" s="6" t="inlineStr"/>
+      <c r="F73" s="6" t="inlineStr"/>
+      <c r="G73" s="6" t="inlineStr"/>
+      <c r="H73" s="6" t="inlineStr"/>
+    </row>
+    <row r="74" ht="24" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>▸ Psicostasia</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="n"/>
+      <c r="C74" s="3" t="n"/>
+      <c r="D74" s="3" t="n"/>
+      <c r="E74" s="3" t="n"/>
+      <c r="F74" s="3" t="n"/>
+      <c r="G74" s="3" t="n"/>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
         </is>
       </c>
     </row>
@@ -2927,22 +2927,22 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>riccardo_landoni</t>
+          <t>Beatrice_Bessone</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>riccardo_landoni</t>
+          <t>Beatrice_Bessone</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>riccardo_landoni@VS_MAIN</t>
+          <t>Beatrice_Bessone@naba.it</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>Overload</t>
+          <t>Psicostasia</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
@@ -2961,241 +2961,241 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="6" customHeight="1">
-      <c r="A76" s="6" t="inlineStr"/>
-      <c r="B76" s="6" t="inlineStr"/>
-      <c r="C76" s="6" t="inlineStr"/>
-      <c r="D76" s="6" t="inlineStr"/>
-      <c r="E76" s="6" t="inlineStr"/>
-      <c r="F76" s="6" t="inlineStr"/>
-      <c r="G76" s="6" t="inlineStr"/>
-      <c r="H76" s="6" t="inlineStr"/>
-    </row>
-    <row r="77" ht="24" customHeight="1">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>▸ Psicostasia</t>
-        </is>
-      </c>
-      <c r="B77" s="3" t="n"/>
-      <c r="C77" s="3" t="n"/>
-      <c r="D77" s="3" t="n"/>
-      <c r="E77" s="3" t="n"/>
-      <c r="F77" s="3" t="n"/>
-      <c r="G77" s="3" t="n"/>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>6 membri</t>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Carmen_Alfano@naba.it</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Psicostasia</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Emanuele_Boschi</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Emanuele_Boschi</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Emanuele_Boschi@naba.it</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Psicostasia</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="78" ht="22" customHeight="1">
-      <c r="A78" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B78" s="7" t="inlineStr">
-        <is>
-          <t>Beatrice_Bessone</t>
-        </is>
-      </c>
-      <c r="C78" s="7" t="inlineStr">
-        <is>
-          <t>Beatrice_Bessone</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="inlineStr">
-        <is>
-          <t>Beatrice_Bessone@naba.it</t>
-        </is>
-      </c>
-      <c r="E78" s="7" t="inlineStr">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Ge_Jiang</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Ge_Jiang</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Ge_Jiang@naba.it</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F78" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G78" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="7" t="inlineStr">
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="79" ht="22" customHeight="1">
-      <c r="A79" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B79" s="7" t="inlineStr">
-        <is>
-          <t>Carmen_Alfano</t>
-        </is>
-      </c>
-      <c r="C79" s="7" t="inlineStr">
-        <is>
-          <t>Carmen_Alfano</t>
-        </is>
-      </c>
-      <c r="D79" s="7" t="inlineStr">
-        <is>
-          <t>Carmen_Alfano@naba.it</t>
-        </is>
-      </c>
-      <c r="E79" s="7" t="inlineStr">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Haotian_Cheng</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Haotian_Cheng</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Haotian_Cheng@naba.it</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G79" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H79" s="7" t="inlineStr">
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="80" ht="22" customHeight="1">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B80" s="7" t="inlineStr">
-        <is>
-          <t>Emanuele_Boschi</t>
-        </is>
-      </c>
-      <c r="C80" s="7" t="inlineStr">
-        <is>
-          <t>Emanuele_Boschi</t>
-        </is>
-      </c>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t>Emanuele_Boschi@naba.it</t>
-        </is>
-      </c>
-      <c r="E80" s="7" t="inlineStr">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Martina_Rotella</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Martina_Rotella</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Martina_Rotella@naba.it</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F80" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H80" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="22" customHeight="1">
-      <c r="A81" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B81" s="7" t="inlineStr">
-        <is>
-          <t>Ge_Jiang</t>
-        </is>
-      </c>
-      <c r="C81" s="7" t="inlineStr">
-        <is>
-          <t>Ge_Jiang</t>
-        </is>
-      </c>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>Ge_Jiang@naba.it</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="inlineStr">
-        <is>
-          <t>Psicostasia</t>
-        </is>
-      </c>
-      <c r="F81" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G81" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H81" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="22" customHeight="1">
-      <c r="A82" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B82" s="7" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng</t>
-        </is>
-      </c>
-      <c r="C82" s="7" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="inlineStr">
-        <is>
-          <t>Haotian_Cheng@naba.it</t>
-        </is>
-      </c>
-      <c r="E82" s="7" t="inlineStr">
-        <is>
-          <t>Psicostasia</t>
-        </is>
-      </c>
-      <c r="F82" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G82" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H82" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="6" customHeight="1">
+      <c r="A81" s="6" t="inlineStr"/>
+      <c r="B81" s="6" t="inlineStr"/>
+      <c r="C81" s="6" t="inlineStr"/>
+      <c r="D81" s="6" t="inlineStr"/>
+      <c r="E81" s="6" t="inlineStr"/>
+      <c r="F81" s="6" t="inlineStr"/>
+      <c r="G81" s="6" t="inlineStr"/>
+      <c r="H81" s="6" t="inlineStr"/>
+    </row>
+    <row r="82" ht="24" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>▸ Reality</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="n"/>
+      <c r="C82" s="3" t="n"/>
+      <c r="D82" s="3" t="n"/>
+      <c r="E82" s="3" t="n"/>
+      <c r="F82" s="3" t="n"/>
+      <c r="G82" s="3" t="n"/>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
@@ -3207,22 +3207,22 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>Martina_Rotella</t>
+          <t>isabella_bari</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Martina_Rotella</t>
+          <t>isabella_bari</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Martina_Rotella@naba.it</t>
+          <t>isabella_bari@VS_MAIN</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>Psicostasia</t>
+          <t>Reality</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr">
@@ -3241,115 +3241,115 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="6" customHeight="1">
-      <c r="A84" s="6" t="inlineStr"/>
-      <c r="B84" s="6" t="inlineStr"/>
-      <c r="C84" s="6" t="inlineStr"/>
-      <c r="D84" s="6" t="inlineStr"/>
-      <c r="E84" s="6" t="inlineStr"/>
-      <c r="F84" s="6" t="inlineStr"/>
-      <c r="G84" s="6" t="inlineStr"/>
-      <c r="H84" s="6" t="inlineStr"/>
-    </row>
-    <row r="85" ht="24" customHeight="1">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>▸ Reality</t>
-        </is>
-      </c>
-      <c r="B85" s="3" t="n"/>
-      <c r="C85" s="3" t="n"/>
-      <c r="D85" s="3" t="n"/>
-      <c r="E85" s="3" t="n"/>
-      <c r="F85" s="3" t="n"/>
-      <c r="G85" s="3" t="n"/>
-      <c r="H85" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="22" customHeight="1">
-      <c r="A86" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="inlineStr">
-        <is>
-          <t>isabella_bari</t>
-        </is>
-      </c>
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>isabella_bari</t>
-        </is>
-      </c>
-      <c r="D86" s="5" t="inlineStr">
-        <is>
-          <t>isabella_bari@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E86" s="5" t="inlineStr">
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>maria_villarroel</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>maria_villarroel</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>maria_villarroel@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
         <is>
           <t>Reality</t>
         </is>
       </c>
-      <c r="F86" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G86" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H86" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="22" customHeight="1">
-      <c r="A87" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="inlineStr">
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H84" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>victor_fernandes@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
         <is>
           <t>Reality</t>
         </is>
       </c>
-      <c r="F87" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G87" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H87" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="6" customHeight="1">
+      <c r="A86" s="6" t="inlineStr"/>
+      <c r="B86" s="6" t="inlineStr"/>
+      <c r="C86" s="6" t="inlineStr"/>
+      <c r="D86" s="6" t="inlineStr"/>
+      <c r="E86" s="6" t="inlineStr"/>
+      <c r="F86" s="6" t="inlineStr"/>
+      <c r="G86" s="6" t="inlineStr"/>
+      <c r="H86" s="6" t="inlineStr"/>
+    </row>
+    <row r="87" ht="24" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>▸ RitmoNulla</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="n"/>
+      <c r="C87" s="3" t="n"/>
+      <c r="D87" s="3" t="n"/>
+      <c r="E87" s="3" t="n"/>
+      <c r="F87" s="3" t="n"/>
+      <c r="G87" s="3" t="n"/>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
         </is>
       </c>
     </row>
@@ -3361,22 +3361,22 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>victor_fernandes</t>
+          <t>Alessandro_Caime</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>victor_fernandes</t>
+          <t>Alessandro_Caime</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>victor_fernandes@VS_MAIN</t>
+          <t>Alessandro_Caime@naba.it</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>Reality</t>
+          <t>RitmoNulla</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
@@ -3395,241 +3395,241 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="6" customHeight="1">
-      <c r="A89" s="6" t="inlineStr"/>
-      <c r="B89" s="6" t="inlineStr"/>
-      <c r="C89" s="6" t="inlineStr"/>
-      <c r="D89" s="6" t="inlineStr"/>
-      <c r="E89" s="6" t="inlineStr"/>
-      <c r="F89" s="6" t="inlineStr"/>
-      <c r="G89" s="6" t="inlineStr"/>
-      <c r="H89" s="6" t="inlineStr"/>
-    </row>
-    <row r="90" ht="24" customHeight="1">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>▸ RitmoNulla</t>
-        </is>
-      </c>
-      <c r="B90" s="3" t="n"/>
-      <c r="C90" s="3" t="n"/>
-      <c r="D90" s="3" t="n"/>
-      <c r="E90" s="3" t="n"/>
-      <c r="F90" s="3" t="n"/>
-      <c r="G90" s="3" t="n"/>
-      <c r="H90" s="4" t="inlineStr">
-        <is>
-          <t>6 membri</t>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Feng_Yuchen@naba.it</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Filippo_Damiano</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Filippo_Damiano</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Filippo_Damiano@naba.it</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="91" ht="22" customHeight="1">
-      <c r="A91" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B91" s="7" t="inlineStr">
-        <is>
-          <t>Alessandro_Caime</t>
-        </is>
-      </c>
-      <c r="C91" s="7" t="inlineStr">
-        <is>
-          <t>Alessandro_Caime</t>
-        </is>
-      </c>
-      <c r="D91" s="7" t="inlineStr">
-        <is>
-          <t>Alessandro_Caime@naba.it</t>
-        </is>
-      </c>
-      <c r="E91" s="7" t="inlineStr">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Gaia_Cinti</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Gaia_Cinti</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Gaia_Cinti@naba.it</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F91" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G91" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H91" s="7" t="inlineStr">
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="92" ht="22" customHeight="1">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B92" s="7" t="inlineStr">
-        <is>
-          <t>Feng_Yuchen</t>
-        </is>
-      </c>
-      <c r="C92" s="7" t="inlineStr">
-        <is>
-          <t>Feng_Yuchen</t>
-        </is>
-      </c>
-      <c r="D92" s="7" t="inlineStr">
-        <is>
-          <t>Feng_Yuchen@naba.it</t>
-        </is>
-      </c>
-      <c r="E92" s="7" t="inlineStr">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Maria_Contesi</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Maria_Contesi</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Maria_Contesi@naba.it</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F92" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G92" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H92" s="7" t="inlineStr">
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="93" ht="22" customHeight="1">
-      <c r="A93" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B93" s="7" t="inlineStr">
-        <is>
-          <t>Filippo_Damiano</t>
-        </is>
-      </c>
-      <c r="C93" s="7" t="inlineStr">
-        <is>
-          <t>Filippo_Damiano</t>
-        </is>
-      </c>
-      <c r="D93" s="7" t="inlineStr">
-        <is>
-          <t>Filippo_Damiano@naba.it</t>
-        </is>
-      </c>
-      <c r="E93" s="7" t="inlineStr">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Raul_Chavez</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Raul_Chavez</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Raul_Chavez@naba.it</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F93" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H93" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="22" customHeight="1">
-      <c r="A94" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B94" s="7" t="inlineStr">
-        <is>
-          <t>Gaia_Cinti</t>
-        </is>
-      </c>
-      <c r="C94" s="7" t="inlineStr">
-        <is>
-          <t>Gaia_Cinti</t>
-        </is>
-      </c>
-      <c r="D94" s="7" t="inlineStr">
-        <is>
-          <t>Gaia_Cinti@naba.it</t>
-        </is>
-      </c>
-      <c r="E94" s="7" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F94" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G94" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H94" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="22" customHeight="1">
-      <c r="A95" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B95" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi</t>
-        </is>
-      </c>
-      <c r="C95" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi</t>
-        </is>
-      </c>
-      <c r="D95" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi@naba.it</t>
-        </is>
-      </c>
-      <c r="E95" s="7" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G95" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H95" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="6" customHeight="1">
+      <c r="A94" s="6" t="inlineStr"/>
+      <c r="B94" s="6" t="inlineStr"/>
+      <c r="C94" s="6" t="inlineStr"/>
+      <c r="D94" s="6" t="inlineStr"/>
+      <c r="E94" s="6" t="inlineStr"/>
+      <c r="F94" s="6" t="inlineStr"/>
+      <c r="G94" s="6" t="inlineStr"/>
+      <c r="H94" s="6" t="inlineStr"/>
+    </row>
+    <row r="95" ht="24" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>▸ Roots</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="3" t="n"/>
+      <c r="D95" s="3" t="n"/>
+      <c r="E95" s="3" t="n"/>
+      <c r="F95" s="3" t="n"/>
+      <c r="G95" s="3" t="n"/>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
@@ -3641,22 +3641,22 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Raul_Chavez</t>
+          <t>Anna_Ebel</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>Raul_Chavez</t>
+          <t>Anna_Ebel</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Raul_Chavez@naba.it</t>
+          <t>Anna_Ebel@naba.it</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>RitmoNulla</t>
+          <t>Roots</t>
         </is>
       </c>
       <c r="F96" s="7" t="inlineStr">
@@ -3675,115 +3675,115 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="6" customHeight="1">
-      <c r="A97" s="6" t="inlineStr"/>
-      <c r="B97" s="6" t="inlineStr"/>
-      <c r="C97" s="6" t="inlineStr"/>
-      <c r="D97" s="6" t="inlineStr"/>
-      <c r="E97" s="6" t="inlineStr"/>
-      <c r="F97" s="6" t="inlineStr"/>
-      <c r="G97" s="6" t="inlineStr"/>
-      <c r="H97" s="6" t="inlineStr"/>
-    </row>
-    <row r="98" ht="24" customHeight="1">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>▸ Roots</t>
-        </is>
-      </c>
-      <c r="B98" s="3" t="n"/>
-      <c r="C98" s="3" t="n"/>
-      <c r="D98" s="3" t="n"/>
-      <c r="E98" s="3" t="n"/>
-      <c r="F98" s="3" t="n"/>
-      <c r="G98" s="3" t="n"/>
-      <c r="H98" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="22" customHeight="1">
-      <c r="A99" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B99" s="5" t="inlineStr">
-        <is>
-          <t>Anna_Ebel</t>
-        </is>
-      </c>
-      <c r="C99" s="5" t="inlineStr">
-        <is>
-          <t>Anna_Ebel</t>
-        </is>
-      </c>
-      <c r="D99" s="5" t="inlineStr">
-        <is>
-          <t>Anna_Ebel@naba.it</t>
-        </is>
-      </c>
-      <c r="E99" s="5" t="inlineStr">
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>Ksenia_Puzankova</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Ksenia_Puzankova</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>Ksenia_Puzankova@naba.it</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
         <is>
           <t>Roots</t>
         </is>
       </c>
-      <c r="F99" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G99" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H99" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="22" customHeight="1">
-      <c r="A100" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B100" s="5" t="inlineStr">
-        <is>
-          <t>Ksenia_Puzankova</t>
-        </is>
-      </c>
-      <c r="C100" s="5" t="inlineStr">
-        <is>
-          <t>Ksenia_Puzankova</t>
-        </is>
-      </c>
-      <c r="D100" s="5" t="inlineStr">
-        <is>
-          <t>Ksenia_Puzankova@naba.it</t>
-        </is>
-      </c>
-      <c r="E100" s="5" t="inlineStr">
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H97" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>Sevda_Sevim</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>Sevda Aleyna Sevim</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>SevdaAleynaSevim@naba.it</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="inlineStr">
         <is>
           <t>Roots</t>
         </is>
       </c>
-      <c r="F100" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G100" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H100" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H98" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="6" customHeight="1">
+      <c r="A99" s="6" t="inlineStr"/>
+      <c r="B99" s="6" t="inlineStr"/>
+      <c r="C99" s="6" t="inlineStr"/>
+      <c r="D99" s="6" t="inlineStr"/>
+      <c r="E99" s="6" t="inlineStr"/>
+      <c r="F99" s="6" t="inlineStr"/>
+      <c r="G99" s="6" t="inlineStr"/>
+      <c r="H99" s="6" t="inlineStr"/>
+    </row>
+    <row r="100" ht="24" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>▸ SelfExe</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="n"/>
+      <c r="C100" s="3" t="n"/>
+      <c r="D100" s="3" t="n"/>
+      <c r="E100" s="3" t="n"/>
+      <c r="F100" s="3" t="n"/>
+      <c r="G100" s="3" t="n"/>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
         </is>
       </c>
     </row>
@@ -3795,22 +3795,22 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Sevda_Sevim</t>
+          <t>Andrian_Cerga</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Sevda Aleyna Sevim</t>
+          <t>Andrian_Cerga</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>SevdaAleynaSevim@naba.it</t>
+          <t>Andrian_Cerga@naba.it</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>Roots</t>
+          <t>SelfExe</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
@@ -3829,199 +3829,199 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="6" customHeight="1">
-      <c r="A102" s="6" t="inlineStr"/>
-      <c r="B102" s="6" t="inlineStr"/>
-      <c r="C102" s="6" t="inlineStr"/>
-      <c r="D102" s="6" t="inlineStr"/>
-      <c r="E102" s="6" t="inlineStr"/>
-      <c r="F102" s="6" t="inlineStr"/>
-      <c r="G102" s="6" t="inlineStr"/>
-      <c r="H102" s="6" t="inlineStr"/>
-    </row>
-    <row r="103" ht="24" customHeight="1">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>▸ SelfExe</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="n"/>
-      <c r="C103" s="3" t="n"/>
-      <c r="D103" s="3" t="n"/>
-      <c r="E103" s="3" t="n"/>
-      <c r="F103" s="3" t="n"/>
-      <c r="G103" s="3" t="n"/>
-      <c r="H103" s="4" t="inlineStr">
-        <is>
-          <t>5 membri</t>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Giacomo_Grioni@naba.it</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>SelfExe</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Giulia_Scordino</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Giulia_Scordino</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>Giulia_Scordino@naba.it</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>SelfExe</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="104" ht="22" customHeight="1">
-      <c r="A104" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B104" s="7" t="inlineStr">
-        <is>
-          <t>Andrian_Cerga</t>
-        </is>
-      </c>
-      <c r="C104" s="7" t="inlineStr">
-        <is>
-          <t>Andrian_Cerga</t>
-        </is>
-      </c>
-      <c r="D104" s="7" t="inlineStr">
-        <is>
-          <t>Andrian_Cerga@naba.it</t>
-        </is>
-      </c>
-      <c r="E104" s="7" t="inlineStr">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>Jacopo_Ansaloni</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Jacopo_Ansaloni</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>Jacopo_Ansaloni@naba.it</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F104" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G104" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H104" s="7" t="inlineStr">
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H104" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="105" ht="22" customHeight="1">
-      <c r="A105" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B105" s="7" t="inlineStr">
-        <is>
-          <t>Giacomo_Grioni</t>
-        </is>
-      </c>
-      <c r="C105" s="7" t="inlineStr">
-        <is>
-          <t>Giacomo_Grioni</t>
-        </is>
-      </c>
-      <c r="D105" s="7" t="inlineStr">
-        <is>
-          <t>Giacomo_Grioni@naba.it</t>
-        </is>
-      </c>
-      <c r="E105" s="7" t="inlineStr">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Sonia_DiGennaro</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Sonia_DiGennaro</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>Sonia_DiGennaro@naba.it</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F105" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G105" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H105" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="22" customHeight="1">
-      <c r="A106" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B106" s="7" t="inlineStr">
-        <is>
-          <t>Giulia_Scordino</t>
-        </is>
-      </c>
-      <c r="C106" s="7" t="inlineStr">
-        <is>
-          <t>Giulia_Scordino</t>
-        </is>
-      </c>
-      <c r="D106" s="7" t="inlineStr">
-        <is>
-          <t>Giulia_Scordino@naba.it</t>
-        </is>
-      </c>
-      <c r="E106" s="7" t="inlineStr">
-        <is>
-          <t>SelfExe</t>
-        </is>
-      </c>
-      <c r="F106" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G106" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H106" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="22" customHeight="1">
-      <c r="A107" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B107" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni</t>
-        </is>
-      </c>
-      <c r="C107" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni@naba.it</t>
-        </is>
-      </c>
-      <c r="E107" s="7" t="inlineStr">
-        <is>
-          <t>SelfExe</t>
-        </is>
-      </c>
-      <c r="F107" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G107" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H107" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="6" customHeight="1">
+      <c r="A106" s="6" t="inlineStr"/>
+      <c r="B106" s="6" t="inlineStr"/>
+      <c r="C106" s="6" t="inlineStr"/>
+      <c r="D106" s="6" t="inlineStr"/>
+      <c r="E106" s="6" t="inlineStr"/>
+      <c r="F106" s="6" t="inlineStr"/>
+      <c r="G106" s="6" t="inlineStr"/>
+      <c r="H106" s="6" t="inlineStr"/>
+    </row>
+    <row r="107" ht="24" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>▸ Taison</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="n"/>
+      <c r="C107" s="3" t="n"/>
+      <c r="D107" s="3" t="n"/>
+      <c r="E107" s="3" t="n"/>
+      <c r="F107" s="3" t="n"/>
+      <c r="G107" s="3" t="n"/>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>Sonia_DiGennaro</t>
+          <t>isabella_bari</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>Sonia_DiGennaro</t>
+          <t>isabella_bari</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>Sonia_DiGennaro@naba.it</t>
+          <t>isabella_bari@VS_MAIN</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>SelfExe</t>
+          <t>Taison</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr">
@@ -4067,115 +4067,115 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="6" customHeight="1">
-      <c r="A109" s="6" t="inlineStr"/>
-      <c r="B109" s="6" t="inlineStr"/>
-      <c r="C109" s="6" t="inlineStr"/>
-      <c r="D109" s="6" t="inlineStr"/>
-      <c r="E109" s="6" t="inlineStr"/>
-      <c r="F109" s="6" t="inlineStr"/>
-      <c r="G109" s="6" t="inlineStr"/>
-      <c r="H109" s="6" t="inlineStr"/>
-    </row>
-    <row r="110" ht="24" customHeight="1">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>▸ Taison</t>
-        </is>
-      </c>
-      <c r="B110" s="3" t="n"/>
-      <c r="C110" s="3" t="n"/>
-      <c r="D110" s="3" t="n"/>
-      <c r="E110" s="3" t="n"/>
-      <c r="F110" s="3" t="n"/>
-      <c r="G110" s="3" t="n"/>
-      <c r="H110" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="22" customHeight="1">
-      <c r="A111" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B111" s="5" t="inlineStr">
-        <is>
-          <t>isabella_bari</t>
-        </is>
-      </c>
-      <c r="C111" s="5" t="inlineStr">
-        <is>
-          <t>isabella_bari</t>
-        </is>
-      </c>
-      <c r="D111" s="5" t="inlineStr">
-        <is>
-          <t>isabella_bari@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E111" s="5" t="inlineStr">
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>maria_villarroel</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>maria_villarroel</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="inlineStr">
+        <is>
+          <t>maria_villarroel@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="inlineStr">
         <is>
           <t>Taison</t>
         </is>
       </c>
-      <c r="F111" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G111" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H111" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="22" customHeight="1">
-      <c r="A112" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B112" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel</t>
-        </is>
-      </c>
-      <c r="C112" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel</t>
-        </is>
-      </c>
-      <c r="D112" s="5" t="inlineStr">
-        <is>
-          <t>maria_villarroel@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E112" s="5" t="inlineStr">
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G109" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H109" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="inlineStr">
+        <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="inlineStr">
+        <is>
+          <t>victor_fernandes@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="inlineStr">
         <is>
           <t>Taison</t>
         </is>
       </c>
-      <c r="F112" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G112" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H112" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F110" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G110" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H110" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="6" customHeight="1">
+      <c r="A111" s="6" t="inlineStr"/>
+      <c r="B111" s="6" t="inlineStr"/>
+      <c r="C111" s="6" t="inlineStr"/>
+      <c r="D111" s="6" t="inlineStr"/>
+      <c r="E111" s="6" t="inlineStr"/>
+      <c r="F111" s="6" t="inlineStr"/>
+      <c r="G111" s="6" t="inlineStr"/>
+      <c r="H111" s="6" t="inlineStr"/>
+    </row>
+    <row r="112" ht="24" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>▸ TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="n"/>
+      <c r="C112" s="3" t="n"/>
+      <c r="D112" s="3" t="n"/>
+      <c r="E112" s="3" t="n"/>
+      <c r="F112" s="3" t="n"/>
+      <c r="G112" s="3" t="n"/>
+      <c r="H112" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
         </is>
       </c>
     </row>
@@ -4187,22 +4187,22 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>victor_fernandes</t>
+          <t>Alessia_DiGiannatale</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>victor_fernandes</t>
+          <t>Alessia_DiGiannatale</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>victor_fernandes@VS_MAIN</t>
+          <t>Alessia_DiGiannatale@naba.it</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>Taison</t>
+          <t>TrainOfThoughts</t>
         </is>
       </c>
       <c r="F113" s="5" t="inlineStr">
@@ -4221,157 +4221,157 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="6" customHeight="1">
-      <c r="A114" s="6" t="inlineStr"/>
-      <c r="B114" s="6" t="inlineStr"/>
-      <c r="C114" s="6" t="inlineStr"/>
-      <c r="D114" s="6" t="inlineStr"/>
-      <c r="E114" s="6" t="inlineStr"/>
-      <c r="F114" s="6" t="inlineStr"/>
-      <c r="G114" s="6" t="inlineStr"/>
-      <c r="H114" s="6" t="inlineStr"/>
-    </row>
-    <row r="115" ht="24" customHeight="1">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>▸ TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="n"/>
-      <c r="C115" s="3" t="n"/>
-      <c r="D115" s="3" t="n"/>
-      <c r="E115" s="3" t="n"/>
-      <c r="F115" s="3" t="n"/>
-      <c r="G115" s="3" t="n"/>
-      <c r="H115" s="4" t="inlineStr">
-        <is>
-          <t>4 membri</t>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Bianca_Montobbio</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Bianca_Montobbio</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>Bianca_Montobbio@naba.it</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Francesca_Huang</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Francesca_Huang</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>Francesca_Huang@naba.it</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="116" ht="22" customHeight="1">
-      <c r="A116" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B116" s="7" t="inlineStr">
-        <is>
-          <t>Alessia_DiGiannatale</t>
-        </is>
-      </c>
-      <c r="C116" s="7" t="inlineStr">
-        <is>
-          <t>Alessia_DiGiannatale</t>
-        </is>
-      </c>
-      <c r="D116" s="7" t="inlineStr">
-        <is>
-          <t>Alessia_DiGiannatale@naba.it</t>
-        </is>
-      </c>
-      <c r="E116" s="7" t="inlineStr">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco@naba.it</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
         <is>
           <t>TrainOfThoughts</t>
         </is>
       </c>
-      <c r="F116" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G116" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H116" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="22" customHeight="1">
-      <c r="A117" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B117" s="7" t="inlineStr">
-        <is>
-          <t>Bianca_Montobbio</t>
-        </is>
-      </c>
-      <c r="C117" s="7" t="inlineStr">
-        <is>
-          <t>Bianca_Montobbio</t>
-        </is>
-      </c>
-      <c r="D117" s="7" t="inlineStr">
-        <is>
-          <t>Bianca_Montobbio@naba.it</t>
-        </is>
-      </c>
-      <c r="E117" s="7" t="inlineStr">
-        <is>
-          <t>TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="F117" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G117" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H117" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="22" customHeight="1">
-      <c r="A118" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B118" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang</t>
-        </is>
-      </c>
-      <c r="C118" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang</t>
-        </is>
-      </c>
-      <c r="D118" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang@naba.it</t>
-        </is>
-      </c>
-      <c r="E118" s="7" t="inlineStr">
-        <is>
-          <t>TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="F118" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G118" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H118" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="6" customHeight="1">
+      <c r="A117" s="6" t="inlineStr"/>
+      <c r="B117" s="6" t="inlineStr"/>
+      <c r="C117" s="6" t="inlineStr"/>
+      <c r="D117" s="6" t="inlineStr"/>
+      <c r="E117" s="6" t="inlineStr"/>
+      <c r="F117" s="6" t="inlineStr"/>
+      <c r="G117" s="6" t="inlineStr"/>
+      <c r="H117" s="6" t="inlineStr"/>
+    </row>
+    <row r="118" ht="24" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>▸ Unassigned</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="n"/>
+      <c r="C118" s="3" t="n"/>
+      <c r="D118" s="3" t="n"/>
+      <c r="E118" s="3" t="n"/>
+      <c r="F118" s="3" t="n"/>
+      <c r="G118" s="3" t="n"/>
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
@@ -4383,22 +4383,22 @@
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
-          <t>Martina_Tedesco</t>
+          <t>administrator</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>Martina_Tedesco</t>
+          <t>administator</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>Martina_Tedesco@naba.it</t>
+          <t>tech@naba.it</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>TrainOfThoughts</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="F119" s="7" t="inlineStr">
@@ -4417,155 +4417,85 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="6" customHeight="1">
-      <c r="A120" s="6" t="inlineStr"/>
-      <c r="B120" s="6" t="inlineStr"/>
-      <c r="C120" s="6" t="inlineStr"/>
-      <c r="D120" s="6" t="inlineStr"/>
-      <c r="E120" s="6" t="inlineStr"/>
-      <c r="F120" s="6" t="inlineStr"/>
-      <c r="G120" s="6" t="inlineStr"/>
-      <c r="H120" s="6" t="inlineStr"/>
-    </row>
-    <row r="121" ht="24" customHeight="1">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>▸ Unassigned</t>
-        </is>
-      </c>
-      <c r="B121" s="3" t="n"/>
-      <c r="C121" s="3" t="n"/>
-      <c r="D121" s="3" t="n"/>
-      <c r="E121" s="3" t="n"/>
-      <c r="F121" s="3" t="n"/>
-      <c r="G121" s="3" t="n"/>
-      <c r="H121" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="22" customHeight="1">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B122" s="5" t="inlineStr">
-        <is>
-          <t>administrator</t>
-        </is>
-      </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>administator</t>
-        </is>
-      </c>
-      <c r="D122" s="5" t="inlineStr">
-        <is>
-          <t>tech@naba.it</t>
-        </is>
-      </c>
-      <c r="E122" s="5" t="inlineStr">
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>anna_brue</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>Anna Brue</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t>anna.brue@naba.it</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="F122" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G122" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H122" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="22" customHeight="1">
-      <c r="A123" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B123" s="5" t="inlineStr">
-        <is>
-          <t>anna_brue</t>
-        </is>
-      </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>Anna Brue</t>
-        </is>
-      </c>
-      <c r="D123" s="5" t="inlineStr">
-        <is>
-          <t>anna.brue@naba.it</t>
-        </is>
-      </c>
-      <c r="E123" s="5" t="inlineStr">
+      <c r="F120" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G120" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H120" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>rendernodes</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>rendernodes</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>rendernodes@naba.it</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="F123" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G123" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H123" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="22" customHeight="1">
-      <c r="A124" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="inlineStr">
-        <is>
-          <t>rendernodes</t>
-        </is>
-      </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>rendernodes</t>
-        </is>
-      </c>
-      <c r="D124" s="5" t="inlineStr">
-        <is>
-          <t>rendernodes@naba.it</t>
-        </is>
-      </c>
-      <c r="E124" s="5" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="F124" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G124" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H124" s="5" t="inlineStr">
+      <c r="F121" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H121" s="7" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-20 15:04 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -1532,7 +1532,7 @@
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>▸ Epsilon</t>
+          <t>▸ FloraExMachina</t>
         </is>
       </c>
       <c r="B32" s="3" t="n"/>
@@ -1543,39 +1543,39 @@
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>1 membri</t>
+          <t>3 membri</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>2026-04-16 12:26:25</t>
+          <t>2026-04-14 14:03:18</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>emanuele_lomello</t>
+          <t>alessandro_cova</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Emanuele Lomello</t>
+          <t>alessandro_cova</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>lvilla.garbage@gmail.com</t>
+          <t>alessandro_cova@VS_MAIN</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Epsilon</t>
+          <t>FloraExMachina</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -1585,119 +1585,119 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="6" customHeight="1">
-      <c r="A34" s="6" t="inlineStr"/>
-      <c r="B34" s="6" t="inlineStr"/>
-      <c r="C34" s="6" t="inlineStr"/>
-      <c r="D34" s="6" t="inlineStr"/>
-      <c r="E34" s="6" t="inlineStr"/>
-      <c r="F34" s="6" t="inlineStr"/>
-      <c r="G34" s="6" t="inlineStr"/>
-      <c r="H34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>▸ FloraExMachina</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>alessandro_cova</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>alessandro_cova</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>alessandro_cova@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>denise_bottecchia</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>denise_bottecchia</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>denise_bottecchia@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>FloraExMachina</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>denise_bottecchia@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>kiyomi_corinti@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>FloraExMachina</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="6" customHeight="1">
+      <c r="A36" s="6" t="inlineStr"/>
+      <c r="B36" s="6" t="inlineStr"/>
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr"/>
+      <c r="H36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>▸ HideAndSeek</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
         </is>
       </c>
     </row>
@@ -1709,22 +1709,22 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>kiyomi_corinti</t>
+          <t>Jiayi_Li</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>kiyomi_corinti</t>
+          <t>Jiayi_Li</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>kiyomi_corinti@VS_MAIN</t>
+          <t>Jiayi_Li@naba.it</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>FloraExMachina</t>
+          <t>HideAndSeek</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -1743,157 +1743,157 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="6" customHeight="1">
-      <c r="A39" s="6" t="inlineStr"/>
-      <c r="B39" s="6" t="inlineStr"/>
-      <c r="C39" s="6" t="inlineStr"/>
-      <c r="D39" s="6" t="inlineStr"/>
-      <c r="E39" s="6" t="inlineStr"/>
-      <c r="F39" s="6" t="inlineStr"/>
-      <c r="G39" s="6" t="inlineStr"/>
-      <c r="H39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>▸ HideAndSeek</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>4 membri</t>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Julia_Bergman</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Julia_Bergman</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Julia_Bergman@naba.it</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>HideAndSeek</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Wilma_Sved</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>wilma sved</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>wilma_sved@studenti.naba.it</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>HideAndSeek</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Jiayi_Li</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Jiayi_Li</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>Jiayi_Li@naba.it</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Zhengying_Xu@naba.it</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>HideAndSeek</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Julia_Bergman</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Julia_Bergman</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>Julia_Bergman@naba.it</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>HideAndSeek</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G42" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t>Wilma_Sved</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>wilma sved</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>wilma_sved@studenti.naba.it</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>HideAndSeek</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="6" customHeight="1">
+      <c r="A42" s="6" t="inlineStr"/>
+      <c r="B42" s="6" t="inlineStr"/>
+      <c r="C42" s="6" t="inlineStr"/>
+      <c r="D42" s="6" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr"/>
+      <c r="F42" s="6" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr"/>
+      <c r="H42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>▸ Imagery</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="3" t="n"/>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
         </is>
       </c>
     </row>
@@ -1905,22 +1905,22 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Zhengying_Xu</t>
+          <t>Anastasia_Miani</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Zhengying_Xu</t>
+          <t>Anastasia_Miani</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Zhengying_Xu@naba.it</t>
+          <t>Anastasia_Miani@naba.it</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>HideAndSeek</t>
+          <t>Imagery</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
@@ -1939,241 +1939,241 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="6" customHeight="1">
-      <c r="A45" s="6" t="inlineStr"/>
-      <c r="B45" s="6" t="inlineStr"/>
-      <c r="C45" s="6" t="inlineStr"/>
-      <c r="D45" s="6" t="inlineStr"/>
-      <c r="E45" s="6" t="inlineStr"/>
-      <c r="F45" s="6" t="inlineStr"/>
-      <c r="G45" s="6" t="inlineStr"/>
-      <c r="H45" s="6" t="inlineStr"/>
-    </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>▸ Imagery</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="n"/>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
-      <c r="F46" s="3" t="n"/>
-      <c r="G46" s="3" t="n"/>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>6 membri</t>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Lorenzo_Mari</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Lorenzo_Mari</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Lorenzo_Mari@naba.it</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Imagery</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Lucrezia_D'Amico</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Lucrezia_D'Amico</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Lucrezia_D'Amico@naba.it</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Imagery</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Anastasia_Miani</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Anastasia_Miani</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Anastasia_Miani@naba.it</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Mattia_Bombace</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Mattia_Bombace</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Mattia_Bombace@naba.it</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>Imagery</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Lorenzo_Mari</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Lorenzo_Mari</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Lorenzo_Mari@naba.it</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Serena_Lin</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Serena_Lin</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Serena_Lin@naba.it</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>Imagery</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Lucrezia_D'Amico</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>Lucrezia_D'Amico</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Lucrezia_D'Amico@naba.it</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Youfan_Lin</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Youfan_Lin</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Youfan_Lin@naba.it</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>Imagery</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Mattia_Bombace</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Mattia_Bombace</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Mattia_Bombace@naba.it</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Imagery</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Serena_Lin</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>Serena_Lin</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Serena_Lin@naba.it</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Imagery</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="6" customHeight="1">
+      <c r="A50" s="6" t="inlineStr"/>
+      <c r="B50" s="6" t="inlineStr"/>
+      <c r="C50" s="6" t="inlineStr"/>
+      <c r="D50" s="6" t="inlineStr"/>
+      <c r="E50" s="6" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr"/>
+      <c r="H50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51" ht="24" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>▸ Kronos</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n"/>
+      <c r="C51" s="3" t="n"/>
+      <c r="D51" s="3" t="n"/>
+      <c r="E51" s="3" t="n"/>
+      <c r="F51" s="3" t="n"/>
+      <c r="G51" s="3" t="n"/>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
         </is>
       </c>
     </row>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Youfan_Lin</t>
+          <t>Alberto_Cervillio</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Youfan_Lin</t>
+          <t>Alberto_Cervillio</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Youfan_Lin@naba.it</t>
+          <t>Alberto_Cervillio@naba.it</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Imagery</t>
+          <t>Kronos</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -2219,226 +2219,226 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="6" customHeight="1">
-      <c r="A53" s="6" t="inlineStr"/>
-      <c r="B53" s="6" t="inlineStr"/>
-      <c r="C53" s="6" t="inlineStr"/>
-      <c r="D53" s="6" t="inlineStr"/>
-      <c r="E53" s="6" t="inlineStr"/>
-      <c r="F53" s="6" t="inlineStr"/>
-      <c r="G53" s="6" t="inlineStr"/>
-      <c r="H53" s="6" t="inlineStr"/>
-    </row>
-    <row r="54" ht="24" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>▸ Kronos</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="n"/>
-      <c r="C54" s="3" t="n"/>
-      <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n"/>
-      <c r="G54" s="3" t="n"/>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>5 membri</t>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Bruno_Bisogno</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Bruno_Bisogno</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Bruno_Bisogno@naba.it</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Kronos</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Gaia_Aprile</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Gaia_Aprile</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Gaia_Aprile@naba.it</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Kronos</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>Alberto_Cervillio</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="inlineStr">
-        <is>
-          <t>Alberto_Cervillio</t>
-        </is>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>Alberto_Cervillio@naba.it</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Jacopo_Bruschi</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Jacopo_Bruschi</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Jacopo_Bruschi@naba-da.com</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>Kronos</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
     </row>
     <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>Bruno_Bisogno</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>Bruno_Bisogno</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
-        <is>
-          <t>Bruno_Bisogno@naba.it</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Riccardo_Bassani</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Riccardo_Bassani</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Riccardo_Bassani@naba.it</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>Kronos</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H56" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>Gaia_Aprile</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>Gaia_Aprile</t>
-        </is>
-      </c>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>Gaia_Aprile@naba.it</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>Kronos</t>
-        </is>
-      </c>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Bruschi</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Bruschi</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Bruschi@naba-da.com</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>Kronos</t>
-        </is>
-      </c>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="6" customHeight="1">
+      <c r="A57" s="6" t="inlineStr"/>
+      <c r="B57" s="6" t="inlineStr"/>
+      <c r="C57" s="6" t="inlineStr"/>
+      <c r="D57" s="6" t="inlineStr"/>
+      <c r="E57" s="6" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr"/>
+      <c r="G57" s="6" t="inlineStr"/>
+      <c r="H57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58" ht="24" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>▸ Megametal</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n"/>
+      <c r="C58" s="3" t="n"/>
+      <c r="D58" s="3" t="n"/>
+      <c r="E58" s="3" t="n"/>
+      <c r="F58" s="3" t="n"/>
+      <c r="G58" s="3" t="n"/>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>1 membri</t>
         </is>
       </c>
     </row>
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-20 15:03:59</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Riccardo_Bassani</t>
+          <t>giovanni_visai</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Riccardo_Bassani</t>
+          <t>Giovanni Visai</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Riccardo_Bassani@naba.it</t>
+          <t>giovanni.visai@gmail.com</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Kronos</t>
+          <t>Megametal</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
@@ -2448,12 +2448,12 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-22 13:47 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2453,7 +2453,7 @@
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
     <row r="68" ht="24" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>▸ Overload</t>
+          <t>▸ Omega</t>
         </is>
       </c>
       <c r="B68" s="3" t="n"/>
@@ -2719,203 +2719,203 @@
       <c r="G68" s="3" t="n"/>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>4 membri</t>
+          <t>1 membri</t>
         </is>
       </c>
     </row>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-22 13:47:12</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
+          <t>umberto_punzi</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Umberto Punzi</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>umberto.punzi@gmail.com</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Omega</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="6" customHeight="1">
+      <c r="A70" s="6" t="inlineStr"/>
+      <c r="B70" s="6" t="inlineStr"/>
+      <c r="C70" s="6" t="inlineStr"/>
+      <c r="D70" s="6" t="inlineStr"/>
+      <c r="E70" s="6" t="inlineStr"/>
+      <c r="F70" s="6" t="inlineStr"/>
+      <c r="G70" s="6" t="inlineStr"/>
+      <c r="H70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71" ht="24" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>▸ Overload</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="n"/>
+      <c r="C71" s="3" t="n"/>
+      <c r="D71" s="3" t="n"/>
+      <c r="E71" s="3" t="n"/>
+      <c r="F71" s="3" t="n"/>
+      <c r="G71" s="3" t="n"/>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
           <t>gabriele_dallari</t>
         </is>
       </c>
-      <c r="C69" s="7" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>gabriele_dallari</t>
         </is>
       </c>
-      <c r="D69" s="7" t="inlineStr">
+      <c r="D72" s="5" t="inlineStr">
         <is>
           <t>gabriele_dallari@VS_MAIN</t>
         </is>
       </c>
-      <c r="E69" s="7" t="inlineStr">
+      <c r="E72" s="5" t="inlineStr">
         <is>
           <t>Overload</t>
         </is>
       </c>
-      <c r="F69" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G69" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H69" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B70" s="7" t="inlineStr">
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>lorenzo_fiorentino</t>
         </is>
       </c>
-      <c r="C70" s="7" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>lorenzo_fiorentino</t>
         </is>
       </c>
-      <c r="D70" s="7" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>lorenzo_fiorentino@VS_MAIN</t>
         </is>
       </c>
-      <c r="E70" s="7" t="inlineStr">
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>Overload</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>luigi_cirelli</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>luigi_cirelli</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>luigi_cirelli@VS_MAIN</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr">
         <is>
           <t>Overload</t>
         </is>
       </c>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B72" s="7" t="inlineStr">
-        <is>
-          <t>riccardo_landoni</t>
-        </is>
-      </c>
-      <c r="C72" s="7" t="inlineStr">
-        <is>
-          <t>riccardo_landoni</t>
-        </is>
-      </c>
-      <c r="D72" s="7" t="inlineStr">
-        <is>
-          <t>riccardo_landoni@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E72" s="7" t="inlineStr">
-        <is>
-          <t>Overload</t>
-        </is>
-      </c>
-      <c r="F72" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G72" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H72" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="6" customHeight="1">
-      <c r="A73" s="6" t="inlineStr"/>
-      <c r="B73" s="6" t="inlineStr"/>
-      <c r="C73" s="6" t="inlineStr"/>
-      <c r="D73" s="6" t="inlineStr"/>
-      <c r="E73" s="6" t="inlineStr"/>
-      <c r="F73" s="6" t="inlineStr"/>
-      <c r="G73" s="6" t="inlineStr"/>
-      <c r="H73" s="6" t="inlineStr"/>
-    </row>
-    <row r="74" ht="24" customHeight="1">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>▸ Psicostasia</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="n"/>
-      <c r="C74" s="3" t="n"/>
-      <c r="D74" s="3" t="n"/>
-      <c r="E74" s="3" t="n"/>
-      <c r="F74" s="3" t="n"/>
-      <c r="G74" s="3" t="n"/>
-      <c r="H74" s="4" t="inlineStr">
-        <is>
-          <t>6 membri</t>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -2927,275 +2927,275 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
+          <t>riccardo_landoni</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>riccardo_landoni</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>riccardo_landoni@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="6" customHeight="1">
+      <c r="A76" s="6" t="inlineStr"/>
+      <c r="B76" s="6" t="inlineStr"/>
+      <c r="C76" s="6" t="inlineStr"/>
+      <c r="D76" s="6" t="inlineStr"/>
+      <c r="E76" s="6" t="inlineStr"/>
+      <c r="F76" s="6" t="inlineStr"/>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77" ht="24" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>▸ Psicostasia</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="n"/>
+      <c r="C77" s="3" t="n"/>
+      <c r="D77" s="3" t="n"/>
+      <c r="E77" s="3" t="n"/>
+      <c r="F77" s="3" t="n"/>
+      <c r="G77" s="3" t="n"/>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
           <t>Beatrice_Bessone</t>
         </is>
       </c>
-      <c r="C75" s="5" t="inlineStr">
+      <c r="C78" s="7" t="inlineStr">
         <is>
           <t>Beatrice_Bessone</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr">
+      <c r="D78" s="7" t="inlineStr">
         <is>
           <t>Beatrice_Bessone@naba.it</t>
         </is>
       </c>
-      <c r="E75" s="5" t="inlineStr">
+      <c r="E78" s="7" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F75" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G75" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H75" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="22" customHeight="1">
-      <c r="A76" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
         <is>
           <t>Carmen_Alfano</t>
         </is>
       </c>
-      <c r="C76" s="5" t="inlineStr">
+      <c r="C79" s="7" t="inlineStr">
         <is>
           <t>Carmen_Alfano</t>
         </is>
       </c>
-      <c r="D76" s="5" t="inlineStr">
+      <c r="D79" s="7" t="inlineStr">
         <is>
           <t>Carmen_Alfano@naba.it</t>
         </is>
       </c>
-      <c r="E76" s="5" t="inlineStr">
+      <c r="E79" s="7" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F76" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G76" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H76" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="22" customHeight="1">
-      <c r="A77" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
         <is>
           <t>Emanuele_Boschi</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
+      <c r="C80" s="7" t="inlineStr">
         <is>
           <t>Emanuele_Boschi</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
+      <c r="D80" s="7" t="inlineStr">
         <is>
           <t>Emanuele_Boschi@naba.it</t>
         </is>
       </c>
-      <c r="E77" s="5" t="inlineStr">
+      <c r="E80" s="7" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F77" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="22" customHeight="1">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
         <is>
           <t>Ge_Jiang</t>
         </is>
       </c>
-      <c r="C78" s="5" t="inlineStr">
+      <c r="C81" s="7" t="inlineStr">
         <is>
           <t>Ge_Jiang</t>
         </is>
       </c>
-      <c r="D78" s="5" t="inlineStr">
+      <c r="D81" s="7" t="inlineStr">
         <is>
           <t>Ge_Jiang@naba.it</t>
         </is>
       </c>
-      <c r="E78" s="5" t="inlineStr">
+      <c r="E81" s="7" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F78" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G78" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="22" customHeight="1">
-      <c r="A79" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="inlineStr">
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
         <is>
           <t>Haotian_Cheng</t>
         </is>
       </c>
-      <c r="C79" s="5" t="inlineStr">
+      <c r="C82" s="7" t="inlineStr">
         <is>
           <t>Haotian_Cheng</t>
         </is>
       </c>
-      <c r="D79" s="5" t="inlineStr">
+      <c r="D82" s="7" t="inlineStr">
         <is>
           <t>Haotian_Cheng@naba.it</t>
         </is>
       </c>
-      <c r="E79" s="5" t="inlineStr">
+      <c r="E82" s="7" t="inlineStr">
         <is>
           <t>Psicostasia</t>
         </is>
       </c>
-      <c r="F79" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G79" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H79" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="22" customHeight="1">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Rotella</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Rotella</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Rotella@naba.it</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>Psicostasia</t>
-        </is>
-      </c>
-      <c r="F80" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G80" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H80" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="6" customHeight="1">
-      <c r="A81" s="6" t="inlineStr"/>
-      <c r="B81" s="6" t="inlineStr"/>
-      <c r="C81" s="6" t="inlineStr"/>
-      <c r="D81" s="6" t="inlineStr"/>
-      <c r="E81" s="6" t="inlineStr"/>
-      <c r="F81" s="6" t="inlineStr"/>
-      <c r="G81" s="6" t="inlineStr"/>
-      <c r="H81" s="6" t="inlineStr"/>
-    </row>
-    <row r="82" ht="24" customHeight="1">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>▸ Reality</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="n"/>
-      <c r="C82" s="3" t="n"/>
-      <c r="D82" s="3" t="n"/>
-      <c r="E82" s="3" t="n"/>
-      <c r="F82" s="3" t="n"/>
-      <c r="G82" s="3" t="n"/>
-      <c r="H82" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3207,149 +3207,149 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
+          <t>Martina_Rotella</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Martina_Rotella</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Martina_Rotella@naba.it</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>Psicostasia</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="6" customHeight="1">
+      <c r="A84" s="6" t="inlineStr"/>
+      <c r="B84" s="6" t="inlineStr"/>
+      <c r="C84" s="6" t="inlineStr"/>
+      <c r="D84" s="6" t="inlineStr"/>
+      <c r="E84" s="6" t="inlineStr"/>
+      <c r="F84" s="6" t="inlineStr"/>
+      <c r="G84" s="6" t="inlineStr"/>
+      <c r="H84" s="6" t="inlineStr"/>
+    </row>
+    <row r="85" ht="24" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>▸ Reality</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n"/>
+      <c r="C85" s="3" t="n"/>
+      <c r="D85" s="3" t="n"/>
+      <c r="E85" s="3" t="n"/>
+      <c r="F85" s="3" t="n"/>
+      <c r="G85" s="3" t="n"/>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
           <t>isabella_bari</t>
         </is>
       </c>
-      <c r="C83" s="7" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>isabella_bari</t>
         </is>
       </c>
-      <c r="D83" s="7" t="inlineStr">
+      <c r="D86" s="5" t="inlineStr">
         <is>
           <t>isabella_bari@VS_MAIN</t>
         </is>
       </c>
-      <c r="E83" s="7" t="inlineStr">
+      <c r="E86" s="5" t="inlineStr">
         <is>
           <t>Reality</t>
         </is>
       </c>
-      <c r="F83" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G83" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H83" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="22" customHeight="1">
-      <c r="A84" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B84" s="7" t="inlineStr">
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
         <is>
           <t>maria_villarroel</t>
         </is>
       </c>
-      <c r="C84" s="7" t="inlineStr">
+      <c r="C87" s="5" t="inlineStr">
         <is>
           <t>maria_villarroel</t>
         </is>
       </c>
-      <c r="D84" s="7" t="inlineStr">
+      <c r="D87" s="5" t="inlineStr">
         <is>
           <t>maria_villarroel@VS_MAIN</t>
         </is>
       </c>
-      <c r="E84" s="7" t="inlineStr">
+      <c r="E87" s="5" t="inlineStr">
         <is>
           <t>Reality</t>
         </is>
       </c>
-      <c r="F84" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G84" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H84" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="22" customHeight="1">
-      <c r="A85" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B85" s="7" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="C85" s="7" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="D85" s="7" t="inlineStr">
-        <is>
-          <t>victor_fernandes@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E85" s="7" t="inlineStr">
-        <is>
-          <t>Reality</t>
-        </is>
-      </c>
-      <c r="F85" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G85" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H85" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="6" customHeight="1">
-      <c r="A86" s="6" t="inlineStr"/>
-      <c r="B86" s="6" t="inlineStr"/>
-      <c r="C86" s="6" t="inlineStr"/>
-      <c r="D86" s="6" t="inlineStr"/>
-      <c r="E86" s="6" t="inlineStr"/>
-      <c r="F86" s="6" t="inlineStr"/>
-      <c r="G86" s="6" t="inlineStr"/>
-      <c r="H86" s="6" t="inlineStr"/>
-    </row>
-    <row r="87" ht="24" customHeight="1">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>▸ RitmoNulla</t>
-        </is>
-      </c>
-      <c r="B87" s="3" t="n"/>
-      <c r="C87" s="3" t="n"/>
-      <c r="D87" s="3" t="n"/>
-      <c r="E87" s="3" t="n"/>
-      <c r="F87" s="3" t="n"/>
-      <c r="G87" s="3" t="n"/>
-      <c r="H87" s="4" t="inlineStr">
-        <is>
-          <t>6 membri</t>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3361,275 +3361,275 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>victor_fernandes@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Reality</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="6" customHeight="1">
+      <c r="A89" s="6" t="inlineStr"/>
+      <c r="B89" s="6" t="inlineStr"/>
+      <c r="C89" s="6" t="inlineStr"/>
+      <c r="D89" s="6" t="inlineStr"/>
+      <c r="E89" s="6" t="inlineStr"/>
+      <c r="F89" s="6" t="inlineStr"/>
+      <c r="G89" s="6" t="inlineStr"/>
+      <c r="H89" s="6" t="inlineStr"/>
+    </row>
+    <row r="90" ht="24" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>▸ RitmoNulla</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="3" t="n"/>
+      <c r="D90" s="3" t="n"/>
+      <c r="E90" s="3" t="n"/>
+      <c r="F90" s="3" t="n"/>
+      <c r="G90" s="3" t="n"/>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
           <t>Alessandro_Caime</t>
         </is>
       </c>
-      <c r="C88" s="5" t="inlineStr">
+      <c r="C91" s="7" t="inlineStr">
         <is>
           <t>Alessandro_Caime</t>
         </is>
       </c>
-      <c r="D88" s="5" t="inlineStr">
+      <c r="D91" s="7" t="inlineStr">
         <is>
           <t>Alessandro_Caime@naba.it</t>
         </is>
       </c>
-      <c r="E88" s="5" t="inlineStr">
+      <c r="E91" s="7" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F88" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H88" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="22" customHeight="1">
-      <c r="A89" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>Feng_Yuchen</t>
         </is>
       </c>
-      <c r="C89" s="5" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr">
         <is>
           <t>Feng_Yuchen</t>
         </is>
       </c>
-      <c r="D89" s="5" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>Feng_Yuchen@naba.it</t>
         </is>
       </c>
-      <c r="E89" s="5" t="inlineStr">
+      <c r="E92" s="7" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F89" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G89" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H89" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="22" customHeight="1">
-      <c r="A90" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B90" s="5" t="inlineStr">
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
         <is>
           <t>Filippo_Damiano</t>
         </is>
       </c>
-      <c r="C90" s="5" t="inlineStr">
+      <c r="C93" s="7" t="inlineStr">
         <is>
           <t>Filippo_Damiano</t>
         </is>
       </c>
-      <c r="D90" s="5" t="inlineStr">
+      <c r="D93" s="7" t="inlineStr">
         <is>
           <t>Filippo_Damiano@naba.it</t>
         </is>
       </c>
-      <c r="E90" s="5" t="inlineStr">
+      <c r="E93" s="7" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F90" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H90" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="22" customHeight="1">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B91" s="5" t="inlineStr">
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H93" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
         <is>
           <t>Gaia_Cinti</t>
         </is>
       </c>
-      <c r="C91" s="5" t="inlineStr">
+      <c r="C94" s="7" t="inlineStr">
         <is>
           <t>Gaia_Cinti</t>
         </is>
       </c>
-      <c r="D91" s="5" t="inlineStr">
+      <c r="D94" s="7" t="inlineStr">
         <is>
           <t>Gaia_Cinti@naba.it</t>
         </is>
       </c>
-      <c r="E91" s="5" t="inlineStr">
+      <c r="E94" s="7" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F91" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H91" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="22" customHeight="1">
-      <c r="A92" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B92" s="5" t="inlineStr">
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
         <is>
           <t>Maria_Contesi</t>
         </is>
       </c>
-      <c r="C92" s="5" t="inlineStr">
+      <c r="C95" s="7" t="inlineStr">
         <is>
           <t>Maria_Contesi</t>
         </is>
       </c>
-      <c r="D92" s="5" t="inlineStr">
+      <c r="D95" s="7" t="inlineStr">
         <is>
           <t>Maria_Contesi@naba.it</t>
         </is>
       </c>
-      <c r="E92" s="5" t="inlineStr">
+      <c r="E95" s="7" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F92" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G92" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H92" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="22" customHeight="1">
-      <c r="A93" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B93" s="5" t="inlineStr">
-        <is>
-          <t>Raul_Chavez</t>
-        </is>
-      </c>
-      <c r="C93" s="5" t="inlineStr">
-        <is>
-          <t>Raul_Chavez</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
-        <is>
-          <t>Raul_Chavez@naba.it</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F93" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G93" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H93" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="6" customHeight="1">
-      <c r="A94" s="6" t="inlineStr"/>
-      <c r="B94" s="6" t="inlineStr"/>
-      <c r="C94" s="6" t="inlineStr"/>
-      <c r="D94" s="6" t="inlineStr"/>
-      <c r="E94" s="6" t="inlineStr"/>
-      <c r="F94" s="6" t="inlineStr"/>
-      <c r="G94" s="6" t="inlineStr"/>
-      <c r="H94" s="6" t="inlineStr"/>
-    </row>
-    <row r="95" ht="24" customHeight="1">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>▸ Roots</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="n"/>
-      <c r="C95" s="3" t="n"/>
-      <c r="D95" s="3" t="n"/>
-      <c r="E95" s="3" t="n"/>
-      <c r="F95" s="3" t="n"/>
-      <c r="G95" s="3" t="n"/>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H95" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3641,149 +3641,149 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
+          <t>Raul_Chavez</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Raul_Chavez</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>Raul_Chavez@naba.it</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G96" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H96" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="6" customHeight="1">
+      <c r="A97" s="6" t="inlineStr"/>
+      <c r="B97" s="6" t="inlineStr"/>
+      <c r="C97" s="6" t="inlineStr"/>
+      <c r="D97" s="6" t="inlineStr"/>
+      <c r="E97" s="6" t="inlineStr"/>
+      <c r="F97" s="6" t="inlineStr"/>
+      <c r="G97" s="6" t="inlineStr"/>
+      <c r="H97" s="6" t="inlineStr"/>
+    </row>
+    <row r="98" ht="24" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>▸ Roots</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="3" t="n"/>
+      <c r="D98" s="3" t="n"/>
+      <c r="E98" s="3" t="n"/>
+      <c r="F98" s="3" t="n"/>
+      <c r="G98" s="3" t="n"/>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
           <t>Anna_Ebel</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C99" s="5" t="inlineStr">
         <is>
           <t>Anna_Ebel</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D99" s="5" t="inlineStr">
         <is>
           <t>Anna_Ebel@naba.it</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr">
+      <c r="E99" s="5" t="inlineStr">
         <is>
           <t>Roots</t>
         </is>
       </c>
-      <c r="F96" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G96" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H96" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="22" customHeight="1">
-      <c r="A97" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B97" s="7" t="inlineStr">
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
         <is>
           <t>Ksenia_Puzankova</t>
         </is>
       </c>
-      <c r="C97" s="7" t="inlineStr">
+      <c r="C100" s="5" t="inlineStr">
         <is>
           <t>Ksenia_Puzankova</t>
         </is>
       </c>
-      <c r="D97" s="7" t="inlineStr">
+      <c r="D100" s="5" t="inlineStr">
         <is>
           <t>Ksenia_Puzankova@naba.it</t>
         </is>
       </c>
-      <c r="E97" s="7" t="inlineStr">
+      <c r="E100" s="5" t="inlineStr">
         <is>
           <t>Roots</t>
         </is>
       </c>
-      <c r="F97" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G97" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H97" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="22" customHeight="1">
-      <c r="A98" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B98" s="7" t="inlineStr">
-        <is>
-          <t>Sevda_Sevim</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr">
-        <is>
-          <t>Sevda Aleyna Sevim</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>SevdaAleynaSevim@naba.it</t>
-        </is>
-      </c>
-      <c r="E98" s="7" t="inlineStr">
-        <is>
-          <t>Roots</t>
-        </is>
-      </c>
-      <c r="F98" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G98" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H98" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="6" customHeight="1">
-      <c r="A99" s="6" t="inlineStr"/>
-      <c r="B99" s="6" t="inlineStr"/>
-      <c r="C99" s="6" t="inlineStr"/>
-      <c r="D99" s="6" t="inlineStr"/>
-      <c r="E99" s="6" t="inlineStr"/>
-      <c r="F99" s="6" t="inlineStr"/>
-      <c r="G99" s="6" t="inlineStr"/>
-      <c r="H99" s="6" t="inlineStr"/>
-    </row>
-    <row r="100" ht="24" customHeight="1">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>▸ SelfExe</t>
-        </is>
-      </c>
-      <c r="B100" s="3" t="n"/>
-      <c r="C100" s="3" t="n"/>
-      <c r="D100" s="3" t="n"/>
-      <c r="E100" s="3" t="n"/>
-      <c r="F100" s="3" t="n"/>
-      <c r="G100" s="3" t="n"/>
-      <c r="H100" s="4" t="inlineStr">
-        <is>
-          <t>5 membri</t>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3795,233 +3795,233 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
+          <t>Sevda_Sevim</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Sevda Aleyna Sevim</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>SevdaAleynaSevim@naba.it</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>Roots</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="6" customHeight="1">
+      <c r="A102" s="6" t="inlineStr"/>
+      <c r="B102" s="6" t="inlineStr"/>
+      <c r="C102" s="6" t="inlineStr"/>
+      <c r="D102" s="6" t="inlineStr"/>
+      <c r="E102" s="6" t="inlineStr"/>
+      <c r="F102" s="6" t="inlineStr"/>
+      <c r="G102" s="6" t="inlineStr"/>
+      <c r="H102" s="6" t="inlineStr"/>
+    </row>
+    <row r="103" ht="24" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>▸ SelfExe</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="n"/>
+      <c r="C103" s="3" t="n"/>
+      <c r="D103" s="3" t="n"/>
+      <c r="E103" s="3" t="n"/>
+      <c r="F103" s="3" t="n"/>
+      <c r="G103" s="3" t="n"/>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
           <t>Andrian_Cerga</t>
         </is>
       </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="C104" s="7" t="inlineStr">
         <is>
           <t>Andrian_Cerga</t>
         </is>
       </c>
-      <c r="D101" s="5" t="inlineStr">
+      <c r="D104" s="7" t="inlineStr">
         <is>
           <t>Andrian_Cerga@naba.it</t>
         </is>
       </c>
-      <c r="E101" s="5" t="inlineStr">
+      <c r="E104" s="7" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F101" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G101" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H101" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="22" customHeight="1">
-      <c r="A102" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B102" s="5" t="inlineStr">
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G104" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H104" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
         <is>
           <t>Giacomo_Grioni</t>
         </is>
       </c>
-      <c r="C102" s="5" t="inlineStr">
+      <c r="C105" s="7" t="inlineStr">
         <is>
           <t>Giacomo_Grioni</t>
         </is>
       </c>
-      <c r="D102" s="5" t="inlineStr">
+      <c r="D105" s="7" t="inlineStr">
         <is>
           <t>Giacomo_Grioni@naba.it</t>
         </is>
       </c>
-      <c r="E102" s="5" t="inlineStr">
+      <c r="E105" s="7" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F102" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G102" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H102" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="22" customHeight="1">
-      <c r="A103" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B103" s="5" t="inlineStr">
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H105" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
         <is>
           <t>Giulia_Scordino</t>
         </is>
       </c>
-      <c r="C103" s="5" t="inlineStr">
+      <c r="C106" s="7" t="inlineStr">
         <is>
           <t>Giulia_Scordino</t>
         </is>
       </c>
-      <c r="D103" s="5" t="inlineStr">
+      <c r="D106" s="7" t="inlineStr">
         <is>
           <t>Giulia_Scordino@naba.it</t>
         </is>
       </c>
-      <c r="E103" s="5" t="inlineStr">
+      <c r="E106" s="7" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F103" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G103" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H103" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="22" customHeight="1">
-      <c r="A104" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B104" s="5" t="inlineStr">
+      <c r="F106" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G106" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H106" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
         <is>
           <t>Jacopo_Ansaloni</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C107" s="7" t="inlineStr">
         <is>
           <t>Jacopo_Ansaloni</t>
         </is>
       </c>
-      <c r="D104" s="5" t="inlineStr">
+      <c r="D107" s="7" t="inlineStr">
         <is>
           <t>Jacopo_Ansaloni@naba.it</t>
         </is>
       </c>
-      <c r="E104" s="5" t="inlineStr">
+      <c r="E107" s="7" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F104" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G104" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H104" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="22" customHeight="1">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro</t>
-        </is>
-      </c>
-      <c r="C105" s="5" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro</t>
-        </is>
-      </c>
-      <c r="D105" s="5" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro@naba.it</t>
-        </is>
-      </c>
-      <c r="E105" s="5" t="inlineStr">
-        <is>
-          <t>SelfExe</t>
-        </is>
-      </c>
-      <c r="F105" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G105" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H105" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="6" customHeight="1">
-      <c r="A106" s="6" t="inlineStr"/>
-      <c r="B106" s="6" t="inlineStr"/>
-      <c r="C106" s="6" t="inlineStr"/>
-      <c r="D106" s="6" t="inlineStr"/>
-      <c r="E106" s="6" t="inlineStr"/>
-      <c r="F106" s="6" t="inlineStr"/>
-      <c r="G106" s="6" t="inlineStr"/>
-      <c r="H106" s="6" t="inlineStr"/>
-    </row>
-    <row r="107" ht="24" customHeight="1">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>▸ Taison</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="n"/>
-      <c r="C107" s="3" t="n"/>
-      <c r="D107" s="3" t="n"/>
-      <c r="E107" s="3" t="n"/>
-      <c r="F107" s="3" t="n"/>
-      <c r="G107" s="3" t="n"/>
-      <c r="H107" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4033,149 +4033,149 @@
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
+          <t>Sonia_DiGennaro</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>Sonia_DiGennaro</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="inlineStr">
+        <is>
+          <t>Sonia_DiGennaro@naba.it</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="inlineStr">
+        <is>
+          <t>SelfExe</t>
+        </is>
+      </c>
+      <c r="F108" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G108" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H108" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="6" customHeight="1">
+      <c r="A109" s="6" t="inlineStr"/>
+      <c r="B109" s="6" t="inlineStr"/>
+      <c r="C109" s="6" t="inlineStr"/>
+      <c r="D109" s="6" t="inlineStr"/>
+      <c r="E109" s="6" t="inlineStr"/>
+      <c r="F109" s="6" t="inlineStr"/>
+      <c r="G109" s="6" t="inlineStr"/>
+      <c r="H109" s="6" t="inlineStr"/>
+    </row>
+    <row r="110" ht="24" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>▸ Taison</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="n"/>
+      <c r="C110" s="3" t="n"/>
+      <c r="D110" s="3" t="n"/>
+      <c r="E110" s="3" t="n"/>
+      <c r="F110" s="3" t="n"/>
+      <c r="G110" s="3" t="n"/>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
           <t>isabella_bari</t>
         </is>
       </c>
-      <c r="C108" s="7" t="inlineStr">
+      <c r="C111" s="5" t="inlineStr">
         <is>
           <t>isabella_bari</t>
         </is>
       </c>
-      <c r="D108" s="7" t="inlineStr">
+      <c r="D111" s="5" t="inlineStr">
         <is>
           <t>isabella_bari@VS_MAIN</t>
         </is>
       </c>
-      <c r="E108" s="7" t="inlineStr">
+      <c r="E111" s="5" t="inlineStr">
         <is>
           <t>Taison</t>
         </is>
       </c>
-      <c r="F108" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G108" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H108" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="22" customHeight="1">
-      <c r="A109" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B109" s="7" t="inlineStr">
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
         <is>
           <t>maria_villarroel</t>
         </is>
       </c>
-      <c r="C109" s="7" t="inlineStr">
+      <c r="C112" s="5" t="inlineStr">
         <is>
           <t>maria_villarroel</t>
         </is>
       </c>
-      <c r="D109" s="7" t="inlineStr">
+      <c r="D112" s="5" t="inlineStr">
         <is>
           <t>maria_villarroel@VS_MAIN</t>
         </is>
       </c>
-      <c r="E109" s="7" t="inlineStr">
+      <c r="E112" s="5" t="inlineStr">
         <is>
           <t>Taison</t>
         </is>
       </c>
-      <c r="F109" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G109" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H109" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="22" customHeight="1">
-      <c r="A110" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B110" s="7" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="C110" s="7" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="D110" s="7" t="inlineStr">
-        <is>
-          <t>victor_fernandes@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E110" s="7" t="inlineStr">
-        <is>
-          <t>Taison</t>
-        </is>
-      </c>
-      <c r="F110" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G110" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H110" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="6" customHeight="1">
-      <c r="A111" s="6" t="inlineStr"/>
-      <c r="B111" s="6" t="inlineStr"/>
-      <c r="C111" s="6" t="inlineStr"/>
-      <c r="D111" s="6" t="inlineStr"/>
-      <c r="E111" s="6" t="inlineStr"/>
-      <c r="F111" s="6" t="inlineStr"/>
-      <c r="G111" s="6" t="inlineStr"/>
-      <c r="H111" s="6" t="inlineStr"/>
-    </row>
-    <row r="112" ht="24" customHeight="1">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>▸ TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="n"/>
-      <c r="C112" s="3" t="n"/>
-      <c r="D112" s="3" t="n"/>
-      <c r="E112" s="3" t="n"/>
-      <c r="F112" s="3" t="n"/>
-      <c r="G112" s="3" t="n"/>
-      <c r="H112" s="4" t="inlineStr">
-        <is>
-          <t>4 membri</t>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4187,191 +4187,191 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>victor_fernandes@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Taison</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="6" customHeight="1">
+      <c r="A114" s="6" t="inlineStr"/>
+      <c r="B114" s="6" t="inlineStr"/>
+      <c r="C114" s="6" t="inlineStr"/>
+      <c r="D114" s="6" t="inlineStr"/>
+      <c r="E114" s="6" t="inlineStr"/>
+      <c r="F114" s="6" t="inlineStr"/>
+      <c r="G114" s="6" t="inlineStr"/>
+      <c r="H114" s="6" t="inlineStr"/>
+    </row>
+    <row r="115" ht="24" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>▸ TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="n"/>
+      <c r="C115" s="3" t="n"/>
+      <c r="D115" s="3" t="n"/>
+      <c r="E115" s="3" t="n"/>
+      <c r="F115" s="3" t="n"/>
+      <c r="G115" s="3" t="n"/>
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
           <t>Alessia_DiGiannatale</t>
         </is>
       </c>
-      <c r="C113" s="5" t="inlineStr">
+      <c r="C116" s="7" t="inlineStr">
         <is>
           <t>Alessia_DiGiannatale</t>
         </is>
       </c>
-      <c r="D113" s="5" t="inlineStr">
+      <c r="D116" s="7" t="inlineStr">
         <is>
           <t>Alessia_DiGiannatale@naba.it</t>
         </is>
       </c>
-      <c r="E113" s="5" t="inlineStr">
+      <c r="E116" s="7" t="inlineStr">
         <is>
           <t>TrainOfThoughts</t>
         </is>
       </c>
-      <c r="F113" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G113" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H113" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="22" customHeight="1">
-      <c r="A114" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B114" s="5" t="inlineStr">
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G116" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H116" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
         <is>
           <t>Bianca_Montobbio</t>
         </is>
       </c>
-      <c r="C114" s="5" t="inlineStr">
+      <c r="C117" s="7" t="inlineStr">
         <is>
           <t>Bianca_Montobbio</t>
         </is>
       </c>
-      <c r="D114" s="5" t="inlineStr">
+      <c r="D117" s="7" t="inlineStr">
         <is>
           <t>Bianca_Montobbio@naba.it</t>
         </is>
       </c>
-      <c r="E114" s="5" t="inlineStr">
+      <c r="E117" s="7" t="inlineStr">
         <is>
           <t>TrainOfThoughts</t>
         </is>
       </c>
-      <c r="F114" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G114" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H114" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="22" customHeight="1">
-      <c r="A115" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B115" s="5" t="inlineStr">
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G117" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H117" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
         <is>
           <t>Francesca_Huang</t>
         </is>
       </c>
-      <c r="C115" s="5" t="inlineStr">
+      <c r="C118" s="7" t="inlineStr">
         <is>
           <t>Francesca_Huang</t>
         </is>
       </c>
-      <c r="D115" s="5" t="inlineStr">
+      <c r="D118" s="7" t="inlineStr">
         <is>
           <t>Francesca_Huang@naba.it</t>
         </is>
       </c>
-      <c r="E115" s="5" t="inlineStr">
+      <c r="E118" s="7" t="inlineStr">
         <is>
           <t>TrainOfThoughts</t>
         </is>
       </c>
-      <c r="F115" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G115" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H115" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="22" customHeight="1">
-      <c r="A116" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B116" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco</t>
-        </is>
-      </c>
-      <c r="C116" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco</t>
-        </is>
-      </c>
-      <c r="D116" s="5" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco@naba.it</t>
-        </is>
-      </c>
-      <c r="E116" s="5" t="inlineStr">
-        <is>
-          <t>TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="F116" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G116" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H116" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="6" customHeight="1">
-      <c r="A117" s="6" t="inlineStr"/>
-      <c r="B117" s="6" t="inlineStr"/>
-      <c r="C117" s="6" t="inlineStr"/>
-      <c r="D117" s="6" t="inlineStr"/>
-      <c r="E117" s="6" t="inlineStr"/>
-      <c r="F117" s="6" t="inlineStr"/>
-      <c r="G117" s="6" t="inlineStr"/>
-      <c r="H117" s="6" t="inlineStr"/>
-    </row>
-    <row r="118" ht="24" customHeight="1">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>▸ Unassigned</t>
-        </is>
-      </c>
-      <c r="B118" s="3" t="n"/>
-      <c r="C118" s="3" t="n"/>
-      <c r="D118" s="3" t="n"/>
-      <c r="E118" s="3" t="n"/>
-      <c r="F118" s="3" t="n"/>
-      <c r="G118" s="3" t="n"/>
-      <c r="H118" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F118" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G118" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H118" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4383,119 +4383,189 @@
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
+          <t>Martina_Tedesco</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco@naba.it</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="F119" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G119" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H119" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="6" customHeight="1">
+      <c r="A120" s="6" t="inlineStr"/>
+      <c r="B120" s="6" t="inlineStr"/>
+      <c r="C120" s="6" t="inlineStr"/>
+      <c r="D120" s="6" t="inlineStr"/>
+      <c r="E120" s="6" t="inlineStr"/>
+      <c r="F120" s="6" t="inlineStr"/>
+      <c r="G120" s="6" t="inlineStr"/>
+      <c r="H120" s="6" t="inlineStr"/>
+    </row>
+    <row r="121" ht="24" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>▸ Unassigned</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="n"/>
+      <c r="C121" s="3" t="n"/>
+      <c r="D121" s="3" t="n"/>
+      <c r="E121" s="3" t="n"/>
+      <c r="F121" s="3" t="n"/>
+      <c r="G121" s="3" t="n"/>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
           <t>administrator</t>
         </is>
       </c>
-      <c r="C119" s="7" t="inlineStr">
+      <c r="C122" s="5" t="inlineStr">
         <is>
           <t>administator</t>
         </is>
       </c>
-      <c r="D119" s="7" t="inlineStr">
+      <c r="D122" s="5" t="inlineStr">
         <is>
           <t>tech@naba.it</t>
         </is>
       </c>
-      <c r="E119" s="7" t="inlineStr">
+      <c r="E122" s="5" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="F119" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G119" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H119" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="22" customHeight="1">
-      <c r="A120" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B120" s="7" t="inlineStr">
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H122" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
         <is>
           <t>anna_brue</t>
         </is>
       </c>
-      <c r="C120" s="7" t="inlineStr">
+      <c r="C123" s="5" t="inlineStr">
         <is>
           <t>Anna Brue</t>
         </is>
       </c>
-      <c r="D120" s="7" t="inlineStr">
+      <c r="D123" s="5" t="inlineStr">
         <is>
           <t>anna.brue@naba.it</t>
         </is>
       </c>
-      <c r="E120" s="7" t="inlineStr">
+      <c r="E123" s="5" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="F120" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G120" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H120" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="22" customHeight="1">
-      <c r="A121" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B121" s="7" t="inlineStr">
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
         <is>
           <t>rendernodes</t>
         </is>
       </c>
-      <c r="C121" s="7" t="inlineStr">
+      <c r="C124" s="5" t="inlineStr">
         <is>
           <t>rendernodes</t>
         </is>
       </c>
-      <c r="D121" s="7" t="inlineStr">
+      <c r="D124" s="5" t="inlineStr">
         <is>
           <t>rendernodes@naba.it</t>
         </is>
       </c>
-      <c r="E121" s="7" t="inlineStr">
+      <c r="E124" s="5" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="F121" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G121" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H121" s="7" t="inlineStr">
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H124" s="5" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>

</xml_diff>

<commit_message>
feat: new user registration - 2026-04-23 15:31 UTC
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -494,17 +494,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H124"/>
+  <dimension ref="A1:H128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -3408,7 +3408,7 @@
     <row r="90" ht="24" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>▸ RitmoNulla</t>
+          <t>▸ Residual</t>
         </is>
       </c>
       <c r="B90" s="3" t="n"/>
@@ -3419,39 +3419,39 @@
       <c r="G90" s="3" t="n"/>
       <c r="H90" s="4" t="inlineStr">
         <is>
-          <t>6 membri</t>
+          <t>2 membri</t>
         </is>
       </c>
     </row>
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-23 15:31:10</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Alessandro_Caime</t>
+          <t>gaia_colciago</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>Alessandro_Caime</t>
+          <t>Gaia Colciago</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>Alessandro_Caime@naba.it</t>
+          <t>gaia_colciago@studenti.naba.it</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>RitmoNulla</t>
+          <t>Residual</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
@@ -3461,245 +3461,245 @@
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Duplicate</t>
         </is>
       </c>
     </row>
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="7" t="inlineStr">
         <is>
-          <t>2026-04-14 14:03:18</t>
+          <t>2026-04-23 15:31:10</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
+          <t>lorenzo_mari</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>Lorenzo Mari</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>lorenzo_mari@studenti.naba.it</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>Residual</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>Sì</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="6" customHeight="1">
+      <c r="A93" s="6" t="inlineStr"/>
+      <c r="B93" s="6" t="inlineStr"/>
+      <c r="C93" s="6" t="inlineStr"/>
+      <c r="D93" s="6" t="inlineStr"/>
+      <c r="E93" s="6" t="inlineStr"/>
+      <c r="F93" s="6" t="inlineStr"/>
+      <c r="G93" s="6" t="inlineStr"/>
+      <c r="H93" s="6" t="inlineStr"/>
+    </row>
+    <row r="94" ht="24" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>▸ RitmoNulla</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="3" t="n"/>
+      <c r="D94" s="3" t="n"/>
+      <c r="E94" s="3" t="n"/>
+      <c r="F94" s="3" t="n"/>
+      <c r="G94" s="3" t="n"/>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>6 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Alessandro_Caime@naba.it</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
           <t>Feng_Yuchen</t>
         </is>
       </c>
-      <c r="C92" s="7" t="inlineStr">
+      <c r="C96" s="5" t="inlineStr">
         <is>
           <t>Feng_Yuchen</t>
         </is>
       </c>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="D96" s="5" t="inlineStr">
         <is>
           <t>Feng_Yuchen@naba.it</t>
         </is>
       </c>
-      <c r="E92" s="7" t="inlineStr">
+      <c r="E96" s="5" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F92" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G92" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H92" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="22" customHeight="1">
-      <c r="A93" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B93" s="7" t="inlineStr">
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
         <is>
           <t>Filippo_Damiano</t>
         </is>
       </c>
-      <c r="C93" s="7" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>Filippo_Damiano</t>
         </is>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>Filippo_Damiano@naba.it</t>
         </is>
       </c>
-      <c r="E93" s="7" t="inlineStr">
+      <c r="E97" s="5" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F93" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H93" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="22" customHeight="1">
-      <c r="A94" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B94" s="7" t="inlineStr">
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
         <is>
           <t>Gaia_Cinti</t>
         </is>
       </c>
-      <c r="C94" s="7" t="inlineStr">
+      <c r="C98" s="5" t="inlineStr">
         <is>
           <t>Gaia_Cinti</t>
         </is>
       </c>
-      <c r="D94" s="7" t="inlineStr">
+      <c r="D98" s="5" t="inlineStr">
         <is>
           <t>Gaia_Cinti@naba.it</t>
         </is>
       </c>
-      <c r="E94" s="7" t="inlineStr">
+      <c r="E98" s="5" t="inlineStr">
         <is>
           <t>RitmoNulla</t>
         </is>
       </c>
-      <c r="F94" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G94" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H94" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="22" customHeight="1">
-      <c r="A95" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B95" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi</t>
-        </is>
-      </c>
-      <c r="C95" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi</t>
-        </is>
-      </c>
-      <c r="D95" s="7" t="inlineStr">
-        <is>
-          <t>Maria_Contesi@naba.it</t>
-        </is>
-      </c>
-      <c r="E95" s="7" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G95" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H95" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="22" customHeight="1">
-      <c r="A96" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B96" s="7" t="inlineStr">
-        <is>
-          <t>Raul_Chavez</t>
-        </is>
-      </c>
-      <c r="C96" s="7" t="inlineStr">
-        <is>
-          <t>Raul_Chavez</t>
-        </is>
-      </c>
-      <c r="D96" s="7" t="inlineStr">
-        <is>
-          <t>Raul_Chavez@naba.it</t>
-        </is>
-      </c>
-      <c r="E96" s="7" t="inlineStr">
-        <is>
-          <t>RitmoNulla</t>
-        </is>
-      </c>
-      <c r="F96" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G96" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H96" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="6" customHeight="1">
-      <c r="A97" s="6" t="inlineStr"/>
-      <c r="B97" s="6" t="inlineStr"/>
-      <c r="C97" s="6" t="inlineStr"/>
-      <c r="D97" s="6" t="inlineStr"/>
-      <c r="E97" s="6" t="inlineStr"/>
-      <c r="F97" s="6" t="inlineStr"/>
-      <c r="G97" s="6" t="inlineStr"/>
-      <c r="H97" s="6" t="inlineStr"/>
-    </row>
-    <row r="98" ht="24" customHeight="1">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>▸ Roots</t>
-        </is>
-      </c>
-      <c r="B98" s="3" t="n"/>
-      <c r="C98" s="3" t="n"/>
-      <c r="D98" s="3" t="n"/>
-      <c r="E98" s="3" t="n"/>
-      <c r="F98" s="3" t="n"/>
-      <c r="G98" s="3" t="n"/>
-      <c r="H98" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3711,22 +3711,22 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Anna_Ebel</t>
+          <t>Maria_Contesi</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Anna_Ebel</t>
+          <t>Maria_Contesi</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>Anna_Ebel@naba.it</t>
+          <t>Maria_Contesi@naba.it</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>Roots</t>
+          <t>RitmoNulla</t>
         </is>
       </c>
       <c r="F99" s="5" t="inlineStr">
@@ -3753,107 +3753,107 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>Ksenia_Puzankova</t>
+          <t>Raul_Chavez</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Ksenia_Puzankova</t>
+          <t>Raul_Chavez</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>Ksenia_Puzankova@naba.it</t>
+          <t>Raul_Chavez@naba.it</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
+          <t>RitmoNulla</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="6" customHeight="1">
+      <c r="A101" s="6" t="inlineStr"/>
+      <c r="B101" s="6" t="inlineStr"/>
+      <c r="C101" s="6" t="inlineStr"/>
+      <c r="D101" s="6" t="inlineStr"/>
+      <c r="E101" s="6" t="inlineStr"/>
+      <c r="F101" s="6" t="inlineStr"/>
+      <c r="G101" s="6" t="inlineStr"/>
+      <c r="H101" s="6" t="inlineStr"/>
+    </row>
+    <row r="102" ht="24" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>▸ Roots</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="n"/>
+      <c r="C102" s="3" t="n"/>
+      <c r="D102" s="3" t="n"/>
+      <c r="E102" s="3" t="n"/>
+      <c r="F102" s="3" t="n"/>
+      <c r="G102" s="3" t="n"/>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>Anna_Ebel</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>Anna_Ebel</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
+          <t>Anna_Ebel@naba.it</t>
+        </is>
+      </c>
+      <c r="E103" s="7" t="inlineStr">
+        <is>
           <t>Roots</t>
         </is>
       </c>
-      <c r="F100" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G100" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H100" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="22" customHeight="1">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B101" s="5" t="inlineStr">
-        <is>
-          <t>Sevda_Sevim</t>
-        </is>
-      </c>
-      <c r="C101" s="5" t="inlineStr">
-        <is>
-          <t>Sevda Aleyna Sevim</t>
-        </is>
-      </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>SevdaAleynaSevim@naba.it</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="inlineStr">
-        <is>
-          <t>Roots</t>
-        </is>
-      </c>
-      <c r="F101" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G101" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H101" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="6" customHeight="1">
-      <c r="A102" s="6" t="inlineStr"/>
-      <c r="B102" s="6" t="inlineStr"/>
-      <c r="C102" s="6" t="inlineStr"/>
-      <c r="D102" s="6" t="inlineStr"/>
-      <c r="E102" s="6" t="inlineStr"/>
-      <c r="F102" s="6" t="inlineStr"/>
-      <c r="G102" s="6" t="inlineStr"/>
-      <c r="H102" s="6" t="inlineStr"/>
-    </row>
-    <row r="103" ht="24" customHeight="1">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>▸ SelfExe</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="n"/>
-      <c r="C103" s="3" t="n"/>
-      <c r="D103" s="3" t="n"/>
-      <c r="E103" s="3" t="n"/>
-      <c r="F103" s="3" t="n"/>
-      <c r="G103" s="3" t="n"/>
-      <c r="H103" s="4" t="inlineStr">
-        <is>
-          <t>5 membri</t>
+      <c r="F103" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G103" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H103" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>Andrian_Cerga</t>
+          <t>Ksenia_Puzankova</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>Andrian_Cerga</t>
+          <t>Ksenia_Puzankova</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>Andrian_Cerga@naba.it</t>
+          <t>Ksenia_Puzankova@naba.it</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>SelfExe</t>
+          <t>Roots</t>
         </is>
       </c>
       <c r="F104" s="7" t="inlineStr">
@@ -3907,191 +3907,191 @@
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
+          <t>Sevda_Sevim</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>Sevda Aleyna Sevim</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="inlineStr">
+        <is>
+          <t>SevdaAleynaSevim@naba.it</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="inlineStr">
+        <is>
+          <t>Roots</t>
+        </is>
+      </c>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H105" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="6" customHeight="1">
+      <c r="A106" s="6" t="inlineStr"/>
+      <c r="B106" s="6" t="inlineStr"/>
+      <c r="C106" s="6" t="inlineStr"/>
+      <c r="D106" s="6" t="inlineStr"/>
+      <c r="E106" s="6" t="inlineStr"/>
+      <c r="F106" s="6" t="inlineStr"/>
+      <c r="G106" s="6" t="inlineStr"/>
+      <c r="H106" s="6" t="inlineStr"/>
+    </row>
+    <row r="107" ht="24" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>▸ SelfExe</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="n"/>
+      <c r="C107" s="3" t="n"/>
+      <c r="D107" s="3" t="n"/>
+      <c r="E107" s="3" t="n"/>
+      <c r="F107" s="3" t="n"/>
+      <c r="G107" s="3" t="n"/>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>5 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>Andrian_Cerga@naba.it</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>SelfExe</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
           <t>Giacomo_Grioni</t>
         </is>
       </c>
-      <c r="C105" s="7" t="inlineStr">
+      <c r="C109" s="5" t="inlineStr">
         <is>
           <t>Giacomo_Grioni</t>
         </is>
       </c>
-      <c r="D105" s="7" t="inlineStr">
+      <c r="D109" s="5" t="inlineStr">
         <is>
           <t>Giacomo_Grioni@naba.it</t>
         </is>
       </c>
-      <c r="E105" s="7" t="inlineStr">
+      <c r="E109" s="5" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F105" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G105" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H105" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="22" customHeight="1">
-      <c r="A106" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B106" s="7" t="inlineStr">
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H109" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
         <is>
           <t>Giulia_Scordino</t>
         </is>
       </c>
-      <c r="C106" s="7" t="inlineStr">
+      <c r="C110" s="5" t="inlineStr">
         <is>
           <t>Giulia_Scordino</t>
         </is>
       </c>
-      <c r="D106" s="7" t="inlineStr">
+      <c r="D110" s="5" t="inlineStr">
         <is>
           <t>Giulia_Scordino@naba.it</t>
         </is>
       </c>
-      <c r="E106" s="7" t="inlineStr">
+      <c r="E110" s="5" t="inlineStr">
         <is>
           <t>SelfExe</t>
         </is>
       </c>
-      <c r="F106" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G106" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H106" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="22" customHeight="1">
-      <c r="A107" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B107" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni</t>
-        </is>
-      </c>
-      <c r="C107" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>Jacopo_Ansaloni@naba.it</t>
-        </is>
-      </c>
-      <c r="E107" s="7" t="inlineStr">
-        <is>
-          <t>SelfExe</t>
-        </is>
-      </c>
-      <c r="F107" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G107" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H107" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="22" customHeight="1">
-      <c r="A108" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B108" s="7" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro</t>
-        </is>
-      </c>
-      <c r="C108" s="7" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro</t>
-        </is>
-      </c>
-      <c r="D108" s="7" t="inlineStr">
-        <is>
-          <t>Sonia_DiGennaro@naba.it</t>
-        </is>
-      </c>
-      <c r="E108" s="7" t="inlineStr">
-        <is>
-          <t>SelfExe</t>
-        </is>
-      </c>
-      <c r="F108" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G108" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H108" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="6" customHeight="1">
-      <c r="A109" s="6" t="inlineStr"/>
-      <c r="B109" s="6" t="inlineStr"/>
-      <c r="C109" s="6" t="inlineStr"/>
-      <c r="D109" s="6" t="inlineStr"/>
-      <c r="E109" s="6" t="inlineStr"/>
-      <c r="F109" s="6" t="inlineStr"/>
-      <c r="G109" s="6" t="inlineStr"/>
-      <c r="H109" s="6" t="inlineStr"/>
-    </row>
-    <row r="110" ht="24" customHeight="1">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>▸ Taison</t>
-        </is>
-      </c>
-      <c r="B110" s="3" t="n"/>
-      <c r="C110" s="3" t="n"/>
-      <c r="D110" s="3" t="n"/>
-      <c r="E110" s="3" t="n"/>
-      <c r="F110" s="3" t="n"/>
-      <c r="G110" s="3" t="n"/>
-      <c r="H110" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4103,22 +4103,22 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>Jacopo_Ansaloni</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari</t>
+          <t>Jacopo_Ansaloni</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>isabella_bari@VS_MAIN</t>
+          <t>Jacopo_Ansaloni@naba.it</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>Taison</t>
+          <t>SelfExe</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
@@ -4145,107 +4145,107 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>maria_villarroel</t>
+          <t>Sonia_DiGennaro</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>maria_villarroel</t>
+          <t>Sonia_DiGennaro</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t>maria_villarroel@VS_MAIN</t>
+          <t>Sonia_DiGennaro@naba.it</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
+          <t>SelfExe</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="6" customHeight="1">
+      <c r="A113" s="6" t="inlineStr"/>
+      <c r="B113" s="6" t="inlineStr"/>
+      <c r="C113" s="6" t="inlineStr"/>
+      <c r="D113" s="6" t="inlineStr"/>
+      <c r="E113" s="6" t="inlineStr"/>
+      <c r="F113" s="6" t="inlineStr"/>
+      <c r="G113" s="6" t="inlineStr"/>
+      <c r="H113" s="6" t="inlineStr"/>
+    </row>
+    <row r="114" ht="24" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>▸ Taison</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="n"/>
+      <c r="C114" s="3" t="n"/>
+      <c r="D114" s="3" t="n"/>
+      <c r="E114" s="3" t="n"/>
+      <c r="F114" s="3" t="n"/>
+      <c r="G114" s="3" t="n"/>
+      <c r="H114" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>isabella_bari</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>isabella_bari</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>isabella_bari@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
           <t>Taison</t>
         </is>
       </c>
-      <c r="F112" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G112" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H112" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="22" customHeight="1">
-      <c r="A113" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B113" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes</t>
-        </is>
-      </c>
-      <c r="D113" s="5" t="inlineStr">
-        <is>
-          <t>victor_fernandes@VS_MAIN</t>
-        </is>
-      </c>
-      <c r="E113" s="5" t="inlineStr">
-        <is>
-          <t>Taison</t>
-        </is>
-      </c>
-      <c r="F113" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G113" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H113" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="6" customHeight="1">
-      <c r="A114" s="6" t="inlineStr"/>
-      <c r="B114" s="6" t="inlineStr"/>
-      <c r="C114" s="6" t="inlineStr"/>
-      <c r="D114" s="6" t="inlineStr"/>
-      <c r="E114" s="6" t="inlineStr"/>
-      <c r="F114" s="6" t="inlineStr"/>
-      <c r="G114" s="6" t="inlineStr"/>
-      <c r="H114" s="6" t="inlineStr"/>
-    </row>
-    <row r="115" ht="24" customHeight="1">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>▸ TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="n"/>
-      <c r="C115" s="3" t="n"/>
-      <c r="D115" s="3" t="n"/>
-      <c r="E115" s="3" t="n"/>
-      <c r="F115" s="3" t="n"/>
-      <c r="G115" s="3" t="n"/>
-      <c r="H115" s="4" t="inlineStr">
-        <is>
-          <t>4 membri</t>
+      <c r="F115" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G115" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H115" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4257,22 +4257,22 @@
       </c>
       <c r="B116" s="7" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale</t>
+          <t>maria_villarroel</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale</t>
+          <t>maria_villarroel</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>Alessia_DiGiannatale@naba.it</t>
+          <t>maria_villarroel@VS_MAIN</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>TrainOfThoughts</t>
+          <t>Taison</t>
         </is>
       </c>
       <c r="F116" s="7" t="inlineStr">
@@ -4299,149 +4299,149 @@
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>victor_fernandes</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>victor_fernandes@VS_MAIN</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>Taison</t>
+        </is>
+      </c>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G117" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H117" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="6" customHeight="1">
+      <c r="A118" s="6" t="inlineStr"/>
+      <c r="B118" s="6" t="inlineStr"/>
+      <c r="C118" s="6" t="inlineStr"/>
+      <c r="D118" s="6" t="inlineStr"/>
+      <c r="E118" s="6" t="inlineStr"/>
+      <c r="F118" s="6" t="inlineStr"/>
+      <c r="G118" s="6" t="inlineStr"/>
+      <c r="H118" s="6" t="inlineStr"/>
+    </row>
+    <row r="119" ht="24" customHeight="1">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>▸ TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="n"/>
+      <c r="C119" s="3" t="n"/>
+      <c r="D119" s="3" t="n"/>
+      <c r="E119" s="3" t="n"/>
+      <c r="F119" s="3" t="n"/>
+      <c r="G119" s="3" t="n"/>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>4 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>Alessia_DiGiannatale@naba.it</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G120" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H120" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
           <t>Bianca_Montobbio</t>
         </is>
       </c>
-      <c r="C117" s="7" t="inlineStr">
+      <c r="C121" s="5" t="inlineStr">
         <is>
           <t>Bianca_Montobbio</t>
         </is>
       </c>
-      <c r="D117" s="7" t="inlineStr">
+      <c r="D121" s="5" t="inlineStr">
         <is>
           <t>Bianca_Montobbio@naba.it</t>
         </is>
       </c>
-      <c r="E117" s="7" t="inlineStr">
+      <c r="E121" s="5" t="inlineStr">
         <is>
           <t>TrainOfThoughts</t>
         </is>
       </c>
-      <c r="F117" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G117" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H117" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="22" customHeight="1">
-      <c r="A118" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B118" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang</t>
-        </is>
-      </c>
-      <c r="C118" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang</t>
-        </is>
-      </c>
-      <c r="D118" s="7" t="inlineStr">
-        <is>
-          <t>Francesca_Huang@naba.it</t>
-        </is>
-      </c>
-      <c r="E118" s="7" t="inlineStr">
-        <is>
-          <t>TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="F118" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G118" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H118" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="22" customHeight="1">
-      <c r="A119" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B119" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco</t>
-        </is>
-      </c>
-      <c r="C119" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco</t>
-        </is>
-      </c>
-      <c r="D119" s="7" t="inlineStr">
-        <is>
-          <t>Martina_Tedesco@naba.it</t>
-        </is>
-      </c>
-      <c r="E119" s="7" t="inlineStr">
-        <is>
-          <t>TrainOfThoughts</t>
-        </is>
-      </c>
-      <c r="F119" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G119" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H119" s="7" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="6" customHeight="1">
-      <c r="A120" s="6" t="inlineStr"/>
-      <c r="B120" s="6" t="inlineStr"/>
-      <c r="C120" s="6" t="inlineStr"/>
-      <c r="D120" s="6" t="inlineStr"/>
-      <c r="E120" s="6" t="inlineStr"/>
-      <c r="F120" s="6" t="inlineStr"/>
-      <c r="G120" s="6" t="inlineStr"/>
-      <c r="H120" s="6" t="inlineStr"/>
-    </row>
-    <row r="121" ht="24" customHeight="1">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>▸ Unassigned</t>
-        </is>
-      </c>
-      <c r="B121" s="3" t="n"/>
-      <c r="C121" s="3" t="n"/>
-      <c r="D121" s="3" t="n"/>
-      <c r="E121" s="3" t="n"/>
-      <c r="F121" s="3" t="n"/>
-      <c r="G121" s="3" t="n"/>
-      <c r="H121" s="4" t="inlineStr">
-        <is>
-          <t>3 membri</t>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H121" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
         </is>
       </c>
     </row>
@@ -4453,22 +4453,22 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>administrator</t>
+          <t>Francesca_Huang</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>administator</t>
+          <t>Francesca_Huang</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr">
         <is>
-          <t>tech@naba.it</t>
+          <t>Francesca_Huang@naba.it</t>
         </is>
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>TrainOfThoughts</t>
         </is>
       </c>
       <c r="F122" s="5" t="inlineStr">
@@ -4495,77 +4495,189 @@
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
+          <t>Martina_Tedesco</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>Martina_Tedesco@naba.it</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>TrainOfThoughts</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="6" customHeight="1">
+      <c r="A124" s="6" t="inlineStr"/>
+      <c r="B124" s="6" t="inlineStr"/>
+      <c r="C124" s="6" t="inlineStr"/>
+      <c r="D124" s="6" t="inlineStr"/>
+      <c r="E124" s="6" t="inlineStr"/>
+      <c r="F124" s="6" t="inlineStr"/>
+      <c r="G124" s="6" t="inlineStr"/>
+      <c r="H124" s="6" t="inlineStr"/>
+    </row>
+    <row r="125" ht="24" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>▸ Unassigned</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="n"/>
+      <c r="C125" s="3" t="n"/>
+      <c r="D125" s="3" t="n"/>
+      <c r="E125" s="3" t="n"/>
+      <c r="F125" s="3" t="n"/>
+      <c r="G125" s="3" t="n"/>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>3 membri</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B126" s="7" t="inlineStr">
+        <is>
+          <t>administrator</t>
+        </is>
+      </c>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
+          <t>administator</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="inlineStr">
+        <is>
+          <t>tech@naba.it</t>
+        </is>
+      </c>
+      <c r="E126" s="7" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="F126" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G126" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H126" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="22" customHeight="1">
+      <c r="A127" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
           <t>anna_brue</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
+      <c r="C127" s="7" t="inlineStr">
         <is>
           <t>Anna Brue</t>
         </is>
       </c>
-      <c r="D123" s="5" t="inlineStr">
+      <c r="D127" s="7" t="inlineStr">
         <is>
           <t>anna.brue@naba.it</t>
         </is>
       </c>
-      <c r="E123" s="5" t="inlineStr">
+      <c r="E127" s="7" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="F123" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G123" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H123" s="5" t="inlineStr">
-        <is>
-          <t>Existing</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="22" customHeight="1">
-      <c r="A124" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-14 14:03:18</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="inlineStr">
+      <c r="F127" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G127" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H127" s="7" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="22" customHeight="1">
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:03:18</t>
+        </is>
+      </c>
+      <c r="B128" s="7" t="inlineStr">
         <is>
           <t>rendernodes</t>
         </is>
       </c>
-      <c r="C124" s="5" t="inlineStr">
+      <c r="C128" s="7" t="inlineStr">
         <is>
           <t>rendernodes</t>
         </is>
       </c>
-      <c r="D124" s="5" t="inlineStr">
+      <c r="D128" s="7" t="inlineStr">
         <is>
           <t>rendernodes@naba.it</t>
         </is>
       </c>
-      <c r="E124" s="5" t="inlineStr">
+      <c r="E128" s="7" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="F124" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G124" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H124" s="5" t="inlineStr">
+      <c r="F128" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G128" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H128" s="7" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>

</xml_diff>